<commit_message>
📊 Update NAIC content history - 2026-04-02
</commit_message>
<xml_diff>
--- a/docs/content_history/pbr-2026-vm20-table-f-g-current-spreads.xlsx
+++ b/docs/content_history/pbr-2026-vm20-table-f-g-current-spreads.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\PBR\VM20_VM22_ProductSupport\PBR Production Web Data\Current Year\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF3A357C-C7C4-4122-9D0F-596A52D110EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{799202CB-DE5D-43F8-B5E5-7B883A1D2518}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" tabRatio="795" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="39375" yWindow="3060" windowWidth="25140" windowHeight="15225" tabRatio="795" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="February_2026" sheetId="25" r:id="rId1"/>
-    <sheet name="January_2026" sheetId="24" r:id="rId2"/>
-    <sheet name="LEGAL DISCLAIMER" sheetId="11" r:id="rId3"/>
+    <sheet name="March_2026" sheetId="26" r:id="rId1"/>
+    <sheet name="February_2026" sheetId="25" r:id="rId2"/>
+    <sheet name="January_2026" sheetId="24" r:id="rId3"/>
+    <sheet name="LEGAL DISCLAIMER" sheetId="11" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -32,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="32">
   <si>
     <t>WAL</t>
   </si>
@@ -122,6 +123,12 @@
   </si>
   <si>
     <t>Table G. (02/27/2026) Below Investment Grade Current Benchmark Spreads (in bps)</t>
+  </si>
+  <si>
+    <t>Table F (03/31/2026)  Investment Grade Current Benchmark Spreads (in bps)</t>
+  </si>
+  <si>
+    <t>Table G. (03/31/2026) Below Investment Grade Current Benchmark Spreads (in bps)</t>
   </si>
 </sst>
 </file>
@@ -398,7 +405,7 @@
                   <a14:compatExt spid="_x0000_s4104"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000008100000}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000008100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -719,6 +726,2329 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{612EBB24-0E24-4D37-B6A7-8B4DA2BD1A51}">
+  <dimension ref="A1:W35"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="11.08984375" customWidth="1"/>
+    <col min="13" max="23" width="11.08984375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="M1" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="N1" s="14"/>
+      <c r="O1" s="14"/>
+      <c r="P1" s="14"/>
+      <c r="Q1" s="14"/>
+      <c r="R1" s="14"/>
+      <c r="S1" s="14"/>
+      <c r="T1" s="14"/>
+      <c r="U1" s="14"/>
+      <c r="V1" s="14"/>
+      <c r="W1" s="15"/>
+    </row>
+    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A2" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12"/>
+      <c r="K2" s="12"/>
+      <c r="M2" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="N2" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="O2" s="12"/>
+      <c r="P2" s="12"/>
+      <c r="Q2" s="12"/>
+      <c r="R2" s="12"/>
+      <c r="S2" s="12"/>
+      <c r="T2" s="12"/>
+      <c r="U2" s="12"/>
+      <c r="V2" s="12"/>
+      <c r="W2" s="12"/>
+    </row>
+    <row r="3" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A3" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="5">
+        <v>1</v>
+      </c>
+      <c r="C3" s="5">
+        <v>2</v>
+      </c>
+      <c r="D3" s="5">
+        <v>3</v>
+      </c>
+      <c r="E3" s="5">
+        <v>4</v>
+      </c>
+      <c r="F3" s="5">
+        <v>5</v>
+      </c>
+      <c r="G3" s="5">
+        <v>6</v>
+      </c>
+      <c r="H3" s="5">
+        <v>7</v>
+      </c>
+      <c r="I3" s="5">
+        <v>8</v>
+      </c>
+      <c r="J3" s="5">
+        <v>9</v>
+      </c>
+      <c r="K3" s="5">
+        <v>10</v>
+      </c>
+      <c r="M3" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="N3" s="5">
+        <v>11</v>
+      </c>
+      <c r="O3" s="5">
+        <v>12</v>
+      </c>
+      <c r="P3" s="5">
+        <v>13</v>
+      </c>
+      <c r="Q3" s="5">
+        <v>14</v>
+      </c>
+      <c r="R3" s="5">
+        <v>15</v>
+      </c>
+      <c r="S3" s="5">
+        <v>16</v>
+      </c>
+      <c r="T3" s="5">
+        <v>17</v>
+      </c>
+      <c r="U3" s="5">
+        <v>18</v>
+      </c>
+      <c r="V3" s="5">
+        <v>19</v>
+      </c>
+      <c r="W3" s="5">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A4" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="M4" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="P4" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q4" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="R4" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="S4" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="T4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="U4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="V4" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="W4" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A5" s="5">
+        <v>1</v>
+      </c>
+      <c r="B5" s="8">
+        <v>11.74</v>
+      </c>
+      <c r="C5" s="8">
+        <v>21.81</v>
+      </c>
+      <c r="D5" s="8">
+        <v>31.88</v>
+      </c>
+      <c r="E5" s="8">
+        <v>38.51</v>
+      </c>
+      <c r="F5" s="8">
+        <v>45.15</v>
+      </c>
+      <c r="G5" s="8">
+        <v>51.78</v>
+      </c>
+      <c r="H5" s="8">
+        <v>60.73</v>
+      </c>
+      <c r="I5" s="8">
+        <v>69.680000000000007</v>
+      </c>
+      <c r="J5" s="8">
+        <v>78.63</v>
+      </c>
+      <c r="K5" s="8">
+        <v>119.81</v>
+      </c>
+      <c r="M5" s="9">
+        <v>1</v>
+      </c>
+      <c r="N5" s="8">
+        <v>160.99</v>
+      </c>
+      <c r="O5" s="8">
+        <v>216.75</v>
+      </c>
+      <c r="P5" s="8">
+        <v>272.51</v>
+      </c>
+      <c r="Q5" s="8">
+        <v>328.27</v>
+      </c>
+      <c r="R5" s="8">
+        <v>384.03</v>
+      </c>
+      <c r="S5" s="8">
+        <v>587.35</v>
+      </c>
+      <c r="T5" s="8">
+        <v>790.68</v>
+      </c>
+      <c r="U5" s="8">
+        <v>994</v>
+      </c>
+      <c r="V5" s="8">
+        <v>1197.32</v>
+      </c>
+      <c r="W5" s="8">
+        <v>1400.65</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A6" s="5">
+        <v>2</v>
+      </c>
+      <c r="B6" s="8">
+        <v>14.61</v>
+      </c>
+      <c r="C6" s="8">
+        <v>25.45</v>
+      </c>
+      <c r="D6" s="8">
+        <v>36.29</v>
+      </c>
+      <c r="E6" s="8">
+        <v>43.37</v>
+      </c>
+      <c r="F6" s="8">
+        <v>50.45</v>
+      </c>
+      <c r="G6" s="8">
+        <v>57.53</v>
+      </c>
+      <c r="H6" s="8">
+        <v>67.489999999999995</v>
+      </c>
+      <c r="I6" s="8">
+        <v>77.45</v>
+      </c>
+      <c r="J6" s="8">
+        <v>87.41</v>
+      </c>
+      <c r="K6" s="8">
+        <v>124.2</v>
+      </c>
+      <c r="M6" s="9">
+        <v>2</v>
+      </c>
+      <c r="N6" s="8">
+        <v>160.99</v>
+      </c>
+      <c r="O6" s="8">
+        <v>216.75</v>
+      </c>
+      <c r="P6" s="8">
+        <v>272.51</v>
+      </c>
+      <c r="Q6" s="8">
+        <v>328.27</v>
+      </c>
+      <c r="R6" s="8">
+        <v>384.03</v>
+      </c>
+      <c r="S6" s="8">
+        <v>587.35</v>
+      </c>
+      <c r="T6" s="8">
+        <v>790.68</v>
+      </c>
+      <c r="U6" s="8">
+        <v>994</v>
+      </c>
+      <c r="V6" s="8">
+        <v>1197.32</v>
+      </c>
+      <c r="W6" s="8">
+        <v>1400.65</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A7" s="5">
+        <v>3</v>
+      </c>
+      <c r="B7" s="8">
+        <v>17.47</v>
+      </c>
+      <c r="C7" s="8">
+        <v>29.09</v>
+      </c>
+      <c r="D7" s="8">
+        <v>40.71</v>
+      </c>
+      <c r="E7" s="8">
+        <v>48.24</v>
+      </c>
+      <c r="F7" s="8">
+        <v>55.76</v>
+      </c>
+      <c r="G7" s="8">
+        <v>63.28</v>
+      </c>
+      <c r="H7" s="8">
+        <v>74.25</v>
+      </c>
+      <c r="I7" s="8">
+        <v>85.22</v>
+      </c>
+      <c r="J7" s="8">
+        <v>96.19</v>
+      </c>
+      <c r="K7" s="8">
+        <v>128.59</v>
+      </c>
+      <c r="M7" s="9">
+        <v>3</v>
+      </c>
+      <c r="N7" s="8">
+        <v>160.99</v>
+      </c>
+      <c r="O7" s="8">
+        <v>216.75</v>
+      </c>
+      <c r="P7" s="8">
+        <v>272.51</v>
+      </c>
+      <c r="Q7" s="8">
+        <v>328.27</v>
+      </c>
+      <c r="R7" s="8">
+        <v>384.03</v>
+      </c>
+      <c r="S7" s="8">
+        <v>587.35</v>
+      </c>
+      <c r="T7" s="8">
+        <v>790.68</v>
+      </c>
+      <c r="U7" s="8">
+        <v>994</v>
+      </c>
+      <c r="V7" s="8">
+        <v>1197.32</v>
+      </c>
+      <c r="W7" s="8">
+        <v>1400.65</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A8" s="5">
+        <v>4</v>
+      </c>
+      <c r="B8" s="8">
+        <v>20.329999999999998</v>
+      </c>
+      <c r="C8" s="8">
+        <v>32.729999999999997</v>
+      </c>
+      <c r="D8" s="8">
+        <v>45.13</v>
+      </c>
+      <c r="E8" s="8">
+        <v>53.1</v>
+      </c>
+      <c r="F8" s="8">
+        <v>61.07</v>
+      </c>
+      <c r="G8" s="8">
+        <v>69.03</v>
+      </c>
+      <c r="H8" s="8">
+        <v>81.010000000000005</v>
+      </c>
+      <c r="I8" s="8">
+        <v>92.99</v>
+      </c>
+      <c r="J8" s="8">
+        <v>104.96</v>
+      </c>
+      <c r="K8" s="8">
+        <v>132.97</v>
+      </c>
+      <c r="M8" s="9">
+        <v>4</v>
+      </c>
+      <c r="N8" s="8">
+        <v>160.99</v>
+      </c>
+      <c r="O8" s="8">
+        <v>216.75</v>
+      </c>
+      <c r="P8" s="8">
+        <v>272.51</v>
+      </c>
+      <c r="Q8" s="8">
+        <v>328.27</v>
+      </c>
+      <c r="R8" s="8">
+        <v>384.03</v>
+      </c>
+      <c r="S8" s="8">
+        <v>587.35</v>
+      </c>
+      <c r="T8" s="8">
+        <v>790.68</v>
+      </c>
+      <c r="U8" s="8">
+        <v>994</v>
+      </c>
+      <c r="V8" s="8">
+        <v>1197.32</v>
+      </c>
+      <c r="W8" s="8">
+        <v>1400.65</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A9" s="5">
+        <v>5</v>
+      </c>
+      <c r="B9" s="8">
+        <v>22.43</v>
+      </c>
+      <c r="C9" s="8">
+        <v>35.46</v>
+      </c>
+      <c r="D9" s="8">
+        <v>48.49</v>
+      </c>
+      <c r="E9" s="8">
+        <v>56.93</v>
+      </c>
+      <c r="F9" s="8">
+        <v>65.38</v>
+      </c>
+      <c r="G9" s="8">
+        <v>73.83</v>
+      </c>
+      <c r="H9" s="8">
+        <v>85.49</v>
+      </c>
+      <c r="I9" s="8">
+        <v>97.16</v>
+      </c>
+      <c r="J9" s="8">
+        <v>108.82</v>
+      </c>
+      <c r="K9" s="8">
+        <v>134.9</v>
+      </c>
+      <c r="M9" s="9">
+        <v>5</v>
+      </c>
+      <c r="N9" s="8">
+        <v>160.99</v>
+      </c>
+      <c r="O9" s="8">
+        <v>216.75</v>
+      </c>
+      <c r="P9" s="8">
+        <v>272.51</v>
+      </c>
+      <c r="Q9" s="8">
+        <v>328.27</v>
+      </c>
+      <c r="R9" s="8">
+        <v>384.03</v>
+      </c>
+      <c r="S9" s="8">
+        <v>587.35</v>
+      </c>
+      <c r="T9" s="8">
+        <v>790.68</v>
+      </c>
+      <c r="U9" s="8">
+        <v>994</v>
+      </c>
+      <c r="V9" s="8">
+        <v>1197.32</v>
+      </c>
+      <c r="W9" s="8">
+        <v>1400.65</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A10" s="5">
+        <v>6</v>
+      </c>
+      <c r="B10" s="8">
+        <v>24.52</v>
+      </c>
+      <c r="C10" s="8">
+        <v>38.18</v>
+      </c>
+      <c r="D10" s="8">
+        <v>51.84</v>
+      </c>
+      <c r="E10" s="8">
+        <v>60.77</v>
+      </c>
+      <c r="F10" s="8">
+        <v>69.69</v>
+      </c>
+      <c r="G10" s="8">
+        <v>78.62</v>
+      </c>
+      <c r="H10" s="8">
+        <v>89.97</v>
+      </c>
+      <c r="I10" s="8">
+        <v>101.33</v>
+      </c>
+      <c r="J10" s="8">
+        <v>112.69</v>
+      </c>
+      <c r="K10" s="8">
+        <v>136.84</v>
+      </c>
+      <c r="M10" s="9">
+        <v>6</v>
+      </c>
+      <c r="N10" s="8">
+        <v>160.99</v>
+      </c>
+      <c r="O10" s="8">
+        <v>216.75</v>
+      </c>
+      <c r="P10" s="8">
+        <v>272.51</v>
+      </c>
+      <c r="Q10" s="8">
+        <v>328.27</v>
+      </c>
+      <c r="R10" s="8">
+        <v>384.03</v>
+      </c>
+      <c r="S10" s="8">
+        <v>587.35</v>
+      </c>
+      <c r="T10" s="8">
+        <v>790.68</v>
+      </c>
+      <c r="U10" s="8">
+        <v>994</v>
+      </c>
+      <c r="V10" s="8">
+        <v>1197.32</v>
+      </c>
+      <c r="W10" s="8">
+        <v>1400.65</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A11" s="5">
+        <v>7</v>
+      </c>
+      <c r="B11" s="8">
+        <v>25.42</v>
+      </c>
+      <c r="C11" s="8">
+        <v>40.19</v>
+      </c>
+      <c r="D11" s="8">
+        <v>54.95</v>
+      </c>
+      <c r="E11" s="8">
+        <v>64.09</v>
+      </c>
+      <c r="F11" s="8">
+        <v>73.22</v>
+      </c>
+      <c r="G11" s="8">
+        <v>82.35</v>
+      </c>
+      <c r="H11" s="8">
+        <v>93.69</v>
+      </c>
+      <c r="I11" s="8">
+        <v>105.03</v>
+      </c>
+      <c r="J11" s="8">
+        <v>116.37</v>
+      </c>
+      <c r="K11" s="8">
+        <v>138.68</v>
+      </c>
+      <c r="M11" s="9">
+        <v>7</v>
+      </c>
+      <c r="N11" s="8">
+        <v>160.99</v>
+      </c>
+      <c r="O11" s="8">
+        <v>216.75</v>
+      </c>
+      <c r="P11" s="8">
+        <v>272.51</v>
+      </c>
+      <c r="Q11" s="8">
+        <v>328.27</v>
+      </c>
+      <c r="R11" s="8">
+        <v>384.03</v>
+      </c>
+      <c r="S11" s="8">
+        <v>587.35</v>
+      </c>
+      <c r="T11" s="8">
+        <v>790.68</v>
+      </c>
+      <c r="U11" s="8">
+        <v>994</v>
+      </c>
+      <c r="V11" s="8">
+        <v>1197.32</v>
+      </c>
+      <c r="W11" s="8">
+        <v>1400.65</v>
+      </c>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A12" s="5">
+        <v>8</v>
+      </c>
+      <c r="B12" s="8">
+        <v>26.32</v>
+      </c>
+      <c r="C12" s="8">
+        <v>42.19</v>
+      </c>
+      <c r="D12" s="8">
+        <v>58.07</v>
+      </c>
+      <c r="E12" s="8">
+        <v>67.41</v>
+      </c>
+      <c r="F12" s="8">
+        <v>76.75</v>
+      </c>
+      <c r="G12" s="8">
+        <v>86.09</v>
+      </c>
+      <c r="H12" s="8">
+        <v>97.42</v>
+      </c>
+      <c r="I12" s="8">
+        <v>108.74</v>
+      </c>
+      <c r="J12" s="8">
+        <v>120.06</v>
+      </c>
+      <c r="K12" s="8">
+        <v>140.52000000000001</v>
+      </c>
+      <c r="M12" s="9">
+        <v>8</v>
+      </c>
+      <c r="N12" s="8">
+        <v>160.99</v>
+      </c>
+      <c r="O12" s="8">
+        <v>216.75</v>
+      </c>
+      <c r="P12" s="8">
+        <v>272.51</v>
+      </c>
+      <c r="Q12" s="8">
+        <v>328.27</v>
+      </c>
+      <c r="R12" s="8">
+        <v>384.03</v>
+      </c>
+      <c r="S12" s="8">
+        <v>587.35</v>
+      </c>
+      <c r="T12" s="8">
+        <v>790.68</v>
+      </c>
+      <c r="U12" s="8">
+        <v>994</v>
+      </c>
+      <c r="V12" s="8">
+        <v>1197.32</v>
+      </c>
+      <c r="W12" s="8">
+        <v>1400.65</v>
+      </c>
+    </row>
+    <row r="13" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A13" s="5">
+        <v>9</v>
+      </c>
+      <c r="B13" s="8">
+        <v>27.22</v>
+      </c>
+      <c r="C13" s="8">
+        <v>44.2</v>
+      </c>
+      <c r="D13" s="8">
+        <v>61.18</v>
+      </c>
+      <c r="E13" s="8">
+        <v>70.73</v>
+      </c>
+      <c r="F13" s="8">
+        <v>80.28</v>
+      </c>
+      <c r="G13" s="8">
+        <v>89.83</v>
+      </c>
+      <c r="H13" s="8">
+        <v>101.14</v>
+      </c>
+      <c r="I13" s="8">
+        <v>112.44</v>
+      </c>
+      <c r="J13" s="8">
+        <v>123.75</v>
+      </c>
+      <c r="K13" s="8">
+        <v>142.37</v>
+      </c>
+      <c r="M13" s="9">
+        <v>9</v>
+      </c>
+      <c r="N13" s="8">
+        <v>160.99</v>
+      </c>
+      <c r="O13" s="8">
+        <v>216.75</v>
+      </c>
+      <c r="P13" s="8">
+        <v>272.51</v>
+      </c>
+      <c r="Q13" s="8">
+        <v>328.27</v>
+      </c>
+      <c r="R13" s="8">
+        <v>384.03</v>
+      </c>
+      <c r="S13" s="8">
+        <v>587.35</v>
+      </c>
+      <c r="T13" s="8">
+        <v>790.68</v>
+      </c>
+      <c r="U13" s="8">
+        <v>994</v>
+      </c>
+      <c r="V13" s="8">
+        <v>1197.32</v>
+      </c>
+      <c r="W13" s="8">
+        <v>1400.65</v>
+      </c>
+    </row>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A14" s="5">
+        <v>10</v>
+      </c>
+      <c r="B14" s="8">
+        <v>28.84</v>
+      </c>
+      <c r="C14" s="8">
+        <v>45.58</v>
+      </c>
+      <c r="D14" s="8">
+        <v>62.32</v>
+      </c>
+      <c r="E14" s="8">
+        <v>71.489999999999995</v>
+      </c>
+      <c r="F14" s="8">
+        <v>80.66</v>
+      </c>
+      <c r="G14" s="8">
+        <v>89.83</v>
+      </c>
+      <c r="H14" s="8">
+        <v>101.36</v>
+      </c>
+      <c r="I14" s="8">
+        <v>112.88</v>
+      </c>
+      <c r="J14" s="8">
+        <v>124.4</v>
+      </c>
+      <c r="K14" s="8">
+        <v>142.69</v>
+      </c>
+      <c r="M14" s="9">
+        <v>10</v>
+      </c>
+      <c r="N14" s="8">
+        <v>160.99</v>
+      </c>
+      <c r="O14" s="8">
+        <v>216.75</v>
+      </c>
+      <c r="P14" s="8">
+        <v>272.51</v>
+      </c>
+      <c r="Q14" s="8">
+        <v>328.27</v>
+      </c>
+      <c r="R14" s="8">
+        <v>384.03</v>
+      </c>
+      <c r="S14" s="8">
+        <v>587.35</v>
+      </c>
+      <c r="T14" s="8">
+        <v>790.68</v>
+      </c>
+      <c r="U14" s="8">
+        <v>994</v>
+      </c>
+      <c r="V14" s="8">
+        <v>1197.32</v>
+      </c>
+      <c r="W14" s="8">
+        <v>1400.65</v>
+      </c>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A15" s="5">
+        <v>11</v>
+      </c>
+      <c r="B15" s="8">
+        <v>30.46</v>
+      </c>
+      <c r="C15" s="8">
+        <v>46.96</v>
+      </c>
+      <c r="D15" s="8">
+        <v>63.46</v>
+      </c>
+      <c r="E15" s="8">
+        <v>72.25</v>
+      </c>
+      <c r="F15" s="8">
+        <v>81.05</v>
+      </c>
+      <c r="G15" s="8">
+        <v>89.84</v>
+      </c>
+      <c r="H15" s="8">
+        <v>101.58</v>
+      </c>
+      <c r="I15" s="8">
+        <v>113.31</v>
+      </c>
+      <c r="J15" s="8">
+        <v>125.04</v>
+      </c>
+      <c r="K15" s="8">
+        <v>143.01</v>
+      </c>
+      <c r="M15" s="9">
+        <v>11</v>
+      </c>
+      <c r="N15" s="8">
+        <v>160.99</v>
+      </c>
+      <c r="O15" s="8">
+        <v>216.75</v>
+      </c>
+      <c r="P15" s="8">
+        <v>272.51</v>
+      </c>
+      <c r="Q15" s="8">
+        <v>328.27</v>
+      </c>
+      <c r="R15" s="8">
+        <v>384.03</v>
+      </c>
+      <c r="S15" s="8">
+        <v>587.35</v>
+      </c>
+      <c r="T15" s="8">
+        <v>790.68</v>
+      </c>
+      <c r="U15" s="8">
+        <v>994</v>
+      </c>
+      <c r="V15" s="8">
+        <v>1197.32</v>
+      </c>
+      <c r="W15" s="8">
+        <v>1400.65</v>
+      </c>
+    </row>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A16" s="5">
+        <v>12</v>
+      </c>
+      <c r="B16" s="8">
+        <v>32.08</v>
+      </c>
+      <c r="C16" s="8">
+        <v>48.34</v>
+      </c>
+      <c r="D16" s="8">
+        <v>64.599999999999994</v>
+      </c>
+      <c r="E16" s="8">
+        <v>73.02</v>
+      </c>
+      <c r="F16" s="8">
+        <v>81.430000000000007</v>
+      </c>
+      <c r="G16" s="8">
+        <v>89.85</v>
+      </c>
+      <c r="H16" s="8">
+        <v>101.8</v>
+      </c>
+      <c r="I16" s="8">
+        <v>113.74</v>
+      </c>
+      <c r="J16" s="8">
+        <v>125.68</v>
+      </c>
+      <c r="K16" s="8">
+        <v>143.33000000000001</v>
+      </c>
+      <c r="M16" s="9">
+        <v>12</v>
+      </c>
+      <c r="N16" s="8">
+        <v>160.99</v>
+      </c>
+      <c r="O16" s="8">
+        <v>216.75</v>
+      </c>
+      <c r="P16" s="8">
+        <v>272.51</v>
+      </c>
+      <c r="Q16" s="8">
+        <v>328.27</v>
+      </c>
+      <c r="R16" s="8">
+        <v>384.03</v>
+      </c>
+      <c r="S16" s="8">
+        <v>587.35</v>
+      </c>
+      <c r="T16" s="8">
+        <v>790.68</v>
+      </c>
+      <c r="U16" s="8">
+        <v>994</v>
+      </c>
+      <c r="V16" s="8">
+        <v>1197.32</v>
+      </c>
+      <c r="W16" s="8">
+        <v>1400.65</v>
+      </c>
+    </row>
+    <row r="17" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A17" s="5">
+        <v>13</v>
+      </c>
+      <c r="B17" s="8">
+        <v>33.69</v>
+      </c>
+      <c r="C17" s="8">
+        <v>49.72</v>
+      </c>
+      <c r="D17" s="8">
+        <v>65.739999999999995</v>
+      </c>
+      <c r="E17" s="8">
+        <v>73.78</v>
+      </c>
+      <c r="F17" s="8">
+        <v>81.819999999999993</v>
+      </c>
+      <c r="G17" s="8">
+        <v>89.86</v>
+      </c>
+      <c r="H17" s="8">
+        <v>102.02</v>
+      </c>
+      <c r="I17" s="8">
+        <v>114.17</v>
+      </c>
+      <c r="J17" s="8">
+        <v>126.33</v>
+      </c>
+      <c r="K17" s="8">
+        <v>143.66</v>
+      </c>
+      <c r="M17" s="9">
+        <v>13</v>
+      </c>
+      <c r="N17" s="8">
+        <v>160.99</v>
+      </c>
+      <c r="O17" s="8">
+        <v>216.75</v>
+      </c>
+      <c r="P17" s="8">
+        <v>272.51</v>
+      </c>
+      <c r="Q17" s="8">
+        <v>328.27</v>
+      </c>
+      <c r="R17" s="8">
+        <v>384.03</v>
+      </c>
+      <c r="S17" s="8">
+        <v>587.35</v>
+      </c>
+      <c r="T17" s="8">
+        <v>790.68</v>
+      </c>
+      <c r="U17" s="8">
+        <v>994</v>
+      </c>
+      <c r="V17" s="8">
+        <v>1197.32</v>
+      </c>
+      <c r="W17" s="8">
+        <v>1400.65</v>
+      </c>
+    </row>
+    <row r="18" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A18" s="5">
+        <v>14</v>
+      </c>
+      <c r="B18" s="8">
+        <v>35.31</v>
+      </c>
+      <c r="C18" s="8">
+        <v>51.09</v>
+      </c>
+      <c r="D18" s="8">
+        <v>66.87</v>
+      </c>
+      <c r="E18" s="8">
+        <v>74.540000000000006</v>
+      </c>
+      <c r="F18" s="8">
+        <v>82.2</v>
+      </c>
+      <c r="G18" s="8">
+        <v>89.87</v>
+      </c>
+      <c r="H18" s="8">
+        <v>102.24</v>
+      </c>
+      <c r="I18" s="8">
+        <v>114.6</v>
+      </c>
+      <c r="J18" s="8">
+        <v>126.97</v>
+      </c>
+      <c r="K18" s="8">
+        <v>143.97999999999999</v>
+      </c>
+      <c r="M18" s="9">
+        <v>14</v>
+      </c>
+      <c r="N18" s="8">
+        <v>160.99</v>
+      </c>
+      <c r="O18" s="8">
+        <v>216.75</v>
+      </c>
+      <c r="P18" s="8">
+        <v>272.51</v>
+      </c>
+      <c r="Q18" s="8">
+        <v>328.27</v>
+      </c>
+      <c r="R18" s="8">
+        <v>384.03</v>
+      </c>
+      <c r="S18" s="8">
+        <v>587.35</v>
+      </c>
+      <c r="T18" s="8">
+        <v>790.68</v>
+      </c>
+      <c r="U18" s="8">
+        <v>994</v>
+      </c>
+      <c r="V18" s="8">
+        <v>1197.32</v>
+      </c>
+      <c r="W18" s="8">
+        <v>1400.65</v>
+      </c>
+    </row>
+    <row r="19" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A19" s="5">
+        <v>15</v>
+      </c>
+      <c r="B19" s="8">
+        <v>36.93</v>
+      </c>
+      <c r="C19" s="8">
+        <v>52.47</v>
+      </c>
+      <c r="D19" s="8">
+        <v>68.010000000000005</v>
+      </c>
+      <c r="E19" s="8">
+        <v>75.3</v>
+      </c>
+      <c r="F19" s="8">
+        <v>82.59</v>
+      </c>
+      <c r="G19" s="8">
+        <v>89.88</v>
+      </c>
+      <c r="H19" s="8">
+        <v>102.46</v>
+      </c>
+      <c r="I19" s="8">
+        <v>115.04</v>
+      </c>
+      <c r="J19" s="8">
+        <v>127.62</v>
+      </c>
+      <c r="K19" s="8">
+        <v>144.30000000000001</v>
+      </c>
+      <c r="M19" s="9">
+        <v>15</v>
+      </c>
+      <c r="N19" s="8">
+        <v>160.99</v>
+      </c>
+      <c r="O19" s="8">
+        <v>216.75</v>
+      </c>
+      <c r="P19" s="8">
+        <v>272.51</v>
+      </c>
+      <c r="Q19" s="8">
+        <v>328.27</v>
+      </c>
+      <c r="R19" s="8">
+        <v>384.03</v>
+      </c>
+      <c r="S19" s="8">
+        <v>587.35</v>
+      </c>
+      <c r="T19" s="8">
+        <v>790.68</v>
+      </c>
+      <c r="U19" s="8">
+        <v>994</v>
+      </c>
+      <c r="V19" s="8">
+        <v>1197.32</v>
+      </c>
+      <c r="W19" s="8">
+        <v>1400.65</v>
+      </c>
+    </row>
+    <row r="20" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A20" s="5">
+        <v>16</v>
+      </c>
+      <c r="B20" s="8">
+        <v>38.549999999999997</v>
+      </c>
+      <c r="C20" s="8">
+        <v>53.85</v>
+      </c>
+      <c r="D20" s="8">
+        <v>69.150000000000006</v>
+      </c>
+      <c r="E20" s="8">
+        <v>76.06</v>
+      </c>
+      <c r="F20" s="8">
+        <v>82.97</v>
+      </c>
+      <c r="G20" s="8">
+        <v>89.89</v>
+      </c>
+      <c r="H20" s="8">
+        <v>102.68</v>
+      </c>
+      <c r="I20" s="8">
+        <v>115.47</v>
+      </c>
+      <c r="J20" s="8">
+        <v>128.26</v>
+      </c>
+      <c r="K20" s="8">
+        <v>144.62</v>
+      </c>
+      <c r="M20" s="9">
+        <v>16</v>
+      </c>
+      <c r="N20" s="8">
+        <v>160.99</v>
+      </c>
+      <c r="O20" s="8">
+        <v>216.75</v>
+      </c>
+      <c r="P20" s="8">
+        <v>272.51</v>
+      </c>
+      <c r="Q20" s="8">
+        <v>328.27</v>
+      </c>
+      <c r="R20" s="8">
+        <v>384.03</v>
+      </c>
+      <c r="S20" s="8">
+        <v>587.35</v>
+      </c>
+      <c r="T20" s="8">
+        <v>790.68</v>
+      </c>
+      <c r="U20" s="8">
+        <v>994</v>
+      </c>
+      <c r="V20" s="8">
+        <v>1197.32</v>
+      </c>
+      <c r="W20" s="8">
+        <v>1400.65</v>
+      </c>
+    </row>
+    <row r="21" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A21" s="5">
+        <v>17</v>
+      </c>
+      <c r="B21" s="8">
+        <v>40.17</v>
+      </c>
+      <c r="C21" s="8">
+        <v>55.23</v>
+      </c>
+      <c r="D21" s="8">
+        <v>70.290000000000006</v>
+      </c>
+      <c r="E21" s="8">
+        <v>76.819999999999993</v>
+      </c>
+      <c r="F21" s="8">
+        <v>83.36</v>
+      </c>
+      <c r="G21" s="8">
+        <v>89.89</v>
+      </c>
+      <c r="H21" s="8">
+        <v>102.9</v>
+      </c>
+      <c r="I21" s="8">
+        <v>115.9</v>
+      </c>
+      <c r="J21" s="8">
+        <v>128.9</v>
+      </c>
+      <c r="K21" s="8">
+        <v>144.94</v>
+      </c>
+      <c r="M21" s="9">
+        <v>17</v>
+      </c>
+      <c r="N21" s="8">
+        <v>160.99</v>
+      </c>
+      <c r="O21" s="8">
+        <v>216.75</v>
+      </c>
+      <c r="P21" s="8">
+        <v>272.51</v>
+      </c>
+      <c r="Q21" s="8">
+        <v>328.27</v>
+      </c>
+      <c r="R21" s="8">
+        <v>384.03</v>
+      </c>
+      <c r="S21" s="8">
+        <v>587.35</v>
+      </c>
+      <c r="T21" s="8">
+        <v>790.68</v>
+      </c>
+      <c r="U21" s="8">
+        <v>994</v>
+      </c>
+      <c r="V21" s="8">
+        <v>1197.32</v>
+      </c>
+      <c r="W21" s="8">
+        <v>1400.65</v>
+      </c>
+    </row>
+    <row r="22" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A22" s="5">
+        <v>18</v>
+      </c>
+      <c r="B22" s="8">
+        <v>41.79</v>
+      </c>
+      <c r="C22" s="8">
+        <v>56.61</v>
+      </c>
+      <c r="D22" s="8">
+        <v>71.430000000000007</v>
+      </c>
+      <c r="E22" s="8">
+        <v>77.58</v>
+      </c>
+      <c r="F22" s="8">
+        <v>83.74</v>
+      </c>
+      <c r="G22" s="8">
+        <v>89.9</v>
+      </c>
+      <c r="H22" s="8">
+        <v>103.12</v>
+      </c>
+      <c r="I22" s="8">
+        <v>116.33</v>
+      </c>
+      <c r="J22" s="8">
+        <v>129.55000000000001</v>
+      </c>
+      <c r="K22" s="8">
+        <v>145.27000000000001</v>
+      </c>
+      <c r="M22" s="9">
+        <v>18</v>
+      </c>
+      <c r="N22" s="8">
+        <v>160.99</v>
+      </c>
+      <c r="O22" s="8">
+        <v>216.75</v>
+      </c>
+      <c r="P22" s="8">
+        <v>272.51</v>
+      </c>
+      <c r="Q22" s="8">
+        <v>328.27</v>
+      </c>
+      <c r="R22" s="8">
+        <v>384.03</v>
+      </c>
+      <c r="S22" s="8">
+        <v>587.35</v>
+      </c>
+      <c r="T22" s="8">
+        <v>790.68</v>
+      </c>
+      <c r="U22" s="8">
+        <v>994</v>
+      </c>
+      <c r="V22" s="8">
+        <v>1197.32</v>
+      </c>
+      <c r="W22" s="8">
+        <v>1400.65</v>
+      </c>
+    </row>
+    <row r="23" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A23" s="5">
+        <v>19</v>
+      </c>
+      <c r="B23" s="8">
+        <v>43.41</v>
+      </c>
+      <c r="C23" s="8">
+        <v>57.99</v>
+      </c>
+      <c r="D23" s="8">
+        <v>72.56</v>
+      </c>
+      <c r="E23" s="8">
+        <v>78.349999999999994</v>
+      </c>
+      <c r="F23" s="8">
+        <v>84.13</v>
+      </c>
+      <c r="G23" s="8">
+        <v>89.91</v>
+      </c>
+      <c r="H23" s="8">
+        <v>103.34</v>
+      </c>
+      <c r="I23" s="8">
+        <v>116.76</v>
+      </c>
+      <c r="J23" s="8">
+        <v>130.19</v>
+      </c>
+      <c r="K23" s="8">
+        <v>145.59</v>
+      </c>
+      <c r="M23" s="9">
+        <v>19</v>
+      </c>
+      <c r="N23" s="8">
+        <v>160.99</v>
+      </c>
+      <c r="O23" s="8">
+        <v>216.75</v>
+      </c>
+      <c r="P23" s="8">
+        <v>272.51</v>
+      </c>
+      <c r="Q23" s="8">
+        <v>328.27</v>
+      </c>
+      <c r="R23" s="8">
+        <v>384.03</v>
+      </c>
+      <c r="S23" s="8">
+        <v>587.35</v>
+      </c>
+      <c r="T23" s="8">
+        <v>790.68</v>
+      </c>
+      <c r="U23" s="8">
+        <v>994</v>
+      </c>
+      <c r="V23" s="8">
+        <v>1197.32</v>
+      </c>
+      <c r="W23" s="8">
+        <v>1400.65</v>
+      </c>
+    </row>
+    <row r="24" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A24" s="5">
+        <v>20</v>
+      </c>
+      <c r="B24" s="8">
+        <v>45.03</v>
+      </c>
+      <c r="C24" s="8">
+        <v>59.37</v>
+      </c>
+      <c r="D24" s="8">
+        <v>73.7</v>
+      </c>
+      <c r="E24" s="8">
+        <v>79.11</v>
+      </c>
+      <c r="F24" s="8">
+        <v>84.51</v>
+      </c>
+      <c r="G24" s="8">
+        <v>89.92</v>
+      </c>
+      <c r="H24" s="8">
+        <v>103.56</v>
+      </c>
+      <c r="I24" s="8">
+        <v>117.19</v>
+      </c>
+      <c r="J24" s="8">
+        <v>130.83000000000001</v>
+      </c>
+      <c r="K24" s="8">
+        <v>145.91</v>
+      </c>
+      <c r="M24" s="9">
+        <v>20</v>
+      </c>
+      <c r="N24" s="8">
+        <v>160.99</v>
+      </c>
+      <c r="O24" s="8">
+        <v>216.75</v>
+      </c>
+      <c r="P24" s="8">
+        <v>272.51</v>
+      </c>
+      <c r="Q24" s="8">
+        <v>328.27</v>
+      </c>
+      <c r="R24" s="8">
+        <v>384.03</v>
+      </c>
+      <c r="S24" s="8">
+        <v>587.35</v>
+      </c>
+      <c r="T24" s="8">
+        <v>790.68</v>
+      </c>
+      <c r="U24" s="8">
+        <v>994</v>
+      </c>
+      <c r="V24" s="8">
+        <v>1197.32</v>
+      </c>
+      <c r="W24" s="8">
+        <v>1400.65</v>
+      </c>
+    </row>
+    <row r="25" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A25" s="5">
+        <v>21</v>
+      </c>
+      <c r="B25" s="8">
+        <v>46.65</v>
+      </c>
+      <c r="C25" s="8">
+        <v>60.74</v>
+      </c>
+      <c r="D25" s="8">
+        <v>74.84</v>
+      </c>
+      <c r="E25" s="8">
+        <v>79.87</v>
+      </c>
+      <c r="F25" s="8">
+        <v>84.9</v>
+      </c>
+      <c r="G25" s="8">
+        <v>89.93</v>
+      </c>
+      <c r="H25" s="8">
+        <v>103.78</v>
+      </c>
+      <c r="I25" s="8">
+        <v>117.63</v>
+      </c>
+      <c r="J25" s="8">
+        <v>131.47999999999999</v>
+      </c>
+      <c r="K25" s="8">
+        <v>146.22999999999999</v>
+      </c>
+      <c r="M25" s="9">
+        <v>21</v>
+      </c>
+      <c r="N25" s="8">
+        <v>160.99</v>
+      </c>
+      <c r="O25" s="8">
+        <v>216.75</v>
+      </c>
+      <c r="P25" s="8">
+        <v>272.51</v>
+      </c>
+      <c r="Q25" s="8">
+        <v>328.27</v>
+      </c>
+      <c r="R25" s="8">
+        <v>384.03</v>
+      </c>
+      <c r="S25" s="8">
+        <v>587.35</v>
+      </c>
+      <c r="T25" s="8">
+        <v>790.68</v>
+      </c>
+      <c r="U25" s="8">
+        <v>994</v>
+      </c>
+      <c r="V25" s="8">
+        <v>1197.32</v>
+      </c>
+      <c r="W25" s="8">
+        <v>1400.65</v>
+      </c>
+    </row>
+    <row r="26" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A26" s="5">
+        <v>22</v>
+      </c>
+      <c r="B26" s="8">
+        <v>48.27</v>
+      </c>
+      <c r="C26" s="8">
+        <v>62.12</v>
+      </c>
+      <c r="D26" s="8">
+        <v>75.98</v>
+      </c>
+      <c r="E26" s="8">
+        <v>80.63</v>
+      </c>
+      <c r="F26" s="8">
+        <v>85.28</v>
+      </c>
+      <c r="G26" s="8">
+        <v>89.94</v>
+      </c>
+      <c r="H26" s="8">
+        <v>104</v>
+      </c>
+      <c r="I26" s="8">
+        <v>118.06</v>
+      </c>
+      <c r="J26" s="8">
+        <v>132.12</v>
+      </c>
+      <c r="K26" s="8">
+        <v>146.55000000000001</v>
+      </c>
+      <c r="M26" s="9">
+        <v>22</v>
+      </c>
+      <c r="N26" s="8">
+        <v>160.99</v>
+      </c>
+      <c r="O26" s="8">
+        <v>216.75</v>
+      </c>
+      <c r="P26" s="8">
+        <v>272.51</v>
+      </c>
+      <c r="Q26" s="8">
+        <v>328.27</v>
+      </c>
+      <c r="R26" s="8">
+        <v>384.03</v>
+      </c>
+      <c r="S26" s="8">
+        <v>587.35</v>
+      </c>
+      <c r="T26" s="8">
+        <v>790.68</v>
+      </c>
+      <c r="U26" s="8">
+        <v>994</v>
+      </c>
+      <c r="V26" s="8">
+        <v>1197.32</v>
+      </c>
+      <c r="W26" s="8">
+        <v>1400.65</v>
+      </c>
+    </row>
+    <row r="27" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A27" s="5">
+        <v>23</v>
+      </c>
+      <c r="B27" s="8">
+        <v>49.89</v>
+      </c>
+      <c r="C27" s="8">
+        <v>63.5</v>
+      </c>
+      <c r="D27" s="8">
+        <v>77.11</v>
+      </c>
+      <c r="E27" s="8">
+        <v>81.39</v>
+      </c>
+      <c r="F27" s="8">
+        <v>85.67</v>
+      </c>
+      <c r="G27" s="8">
+        <v>89.95</v>
+      </c>
+      <c r="H27" s="8">
+        <v>104.22</v>
+      </c>
+      <c r="I27" s="8">
+        <v>118.49</v>
+      </c>
+      <c r="J27" s="8">
+        <v>132.76</v>
+      </c>
+      <c r="K27" s="8">
+        <v>146.87</v>
+      </c>
+      <c r="M27" s="9">
+        <v>23</v>
+      </c>
+      <c r="N27" s="8">
+        <v>160.99</v>
+      </c>
+      <c r="O27" s="8">
+        <v>216.75</v>
+      </c>
+      <c r="P27" s="8">
+        <v>272.51</v>
+      </c>
+      <c r="Q27" s="8">
+        <v>328.27</v>
+      </c>
+      <c r="R27" s="8">
+        <v>384.03</v>
+      </c>
+      <c r="S27" s="8">
+        <v>587.35</v>
+      </c>
+      <c r="T27" s="8">
+        <v>790.68</v>
+      </c>
+      <c r="U27" s="8">
+        <v>994</v>
+      </c>
+      <c r="V27" s="8">
+        <v>1197.32</v>
+      </c>
+      <c r="W27" s="8">
+        <v>1400.65</v>
+      </c>
+    </row>
+    <row r="28" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A28" s="5">
+        <v>24</v>
+      </c>
+      <c r="B28" s="8">
+        <v>51.51</v>
+      </c>
+      <c r="C28" s="8">
+        <v>64.88</v>
+      </c>
+      <c r="D28" s="8">
+        <v>78.25</v>
+      </c>
+      <c r="E28" s="8">
+        <v>82.15</v>
+      </c>
+      <c r="F28" s="8">
+        <v>86.05</v>
+      </c>
+      <c r="G28" s="8">
+        <v>89.95</v>
+      </c>
+      <c r="H28" s="8">
+        <v>104.44</v>
+      </c>
+      <c r="I28" s="8">
+        <v>118.92</v>
+      </c>
+      <c r="J28" s="8">
+        <v>133.41</v>
+      </c>
+      <c r="K28" s="8">
+        <v>147.19999999999999</v>
+      </c>
+      <c r="M28" s="9">
+        <v>24</v>
+      </c>
+      <c r="N28" s="8">
+        <v>160.99</v>
+      </c>
+      <c r="O28" s="8">
+        <v>216.75</v>
+      </c>
+      <c r="P28" s="8">
+        <v>272.51</v>
+      </c>
+      <c r="Q28" s="8">
+        <v>328.27</v>
+      </c>
+      <c r="R28" s="8">
+        <v>384.03</v>
+      </c>
+      <c r="S28" s="8">
+        <v>587.35</v>
+      </c>
+      <c r="T28" s="8">
+        <v>790.68</v>
+      </c>
+      <c r="U28" s="8">
+        <v>994</v>
+      </c>
+      <c r="V28" s="8">
+        <v>1197.32</v>
+      </c>
+      <c r="W28" s="8">
+        <v>1400.65</v>
+      </c>
+    </row>
+    <row r="29" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A29" s="5">
+        <v>25</v>
+      </c>
+      <c r="B29" s="8">
+        <v>53.13</v>
+      </c>
+      <c r="C29" s="8">
+        <v>66.260000000000005</v>
+      </c>
+      <c r="D29" s="8">
+        <v>79.39</v>
+      </c>
+      <c r="E29" s="8">
+        <v>82.91</v>
+      </c>
+      <c r="F29" s="8">
+        <v>86.44</v>
+      </c>
+      <c r="G29" s="8">
+        <v>89.96</v>
+      </c>
+      <c r="H29" s="8">
+        <v>104.66</v>
+      </c>
+      <c r="I29" s="8">
+        <v>119.35</v>
+      </c>
+      <c r="J29" s="8">
+        <v>134.05000000000001</v>
+      </c>
+      <c r="K29" s="8">
+        <v>147.52000000000001</v>
+      </c>
+      <c r="M29" s="9">
+        <v>25</v>
+      </c>
+      <c r="N29" s="8">
+        <v>160.99</v>
+      </c>
+      <c r="O29" s="8">
+        <v>216.75</v>
+      </c>
+      <c r="P29" s="8">
+        <v>272.51</v>
+      </c>
+      <c r="Q29" s="8">
+        <v>328.27</v>
+      </c>
+      <c r="R29" s="8">
+        <v>384.03</v>
+      </c>
+      <c r="S29" s="8">
+        <v>587.35</v>
+      </c>
+      <c r="T29" s="8">
+        <v>790.68</v>
+      </c>
+      <c r="U29" s="8">
+        <v>994</v>
+      </c>
+      <c r="V29" s="8">
+        <v>1197.32</v>
+      </c>
+      <c r="W29" s="8">
+        <v>1400.65</v>
+      </c>
+    </row>
+    <row r="30" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A30" s="5">
+        <v>26</v>
+      </c>
+      <c r="B30" s="8">
+        <v>54.75</v>
+      </c>
+      <c r="C30" s="8">
+        <v>67.64</v>
+      </c>
+      <c r="D30" s="8">
+        <v>80.53</v>
+      </c>
+      <c r="E30" s="8">
+        <v>83.68</v>
+      </c>
+      <c r="F30" s="8">
+        <v>86.82</v>
+      </c>
+      <c r="G30" s="8">
+        <v>89.97</v>
+      </c>
+      <c r="H30" s="8">
+        <v>104.88</v>
+      </c>
+      <c r="I30" s="8">
+        <v>119.79</v>
+      </c>
+      <c r="J30" s="8">
+        <v>134.69</v>
+      </c>
+      <c r="K30" s="8">
+        <v>147.84</v>
+      </c>
+      <c r="M30" s="9">
+        <v>26</v>
+      </c>
+      <c r="N30" s="8">
+        <v>160.99</v>
+      </c>
+      <c r="O30" s="8">
+        <v>216.75</v>
+      </c>
+      <c r="P30" s="8">
+        <v>272.51</v>
+      </c>
+      <c r="Q30" s="8">
+        <v>328.27</v>
+      </c>
+      <c r="R30" s="8">
+        <v>384.03</v>
+      </c>
+      <c r="S30" s="8">
+        <v>587.35</v>
+      </c>
+      <c r="T30" s="8">
+        <v>790.68</v>
+      </c>
+      <c r="U30" s="8">
+        <v>994</v>
+      </c>
+      <c r="V30" s="8">
+        <v>1197.32</v>
+      </c>
+      <c r="W30" s="8">
+        <v>1400.65</v>
+      </c>
+    </row>
+    <row r="31" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A31" s="5">
+        <v>27</v>
+      </c>
+      <c r="B31" s="8">
+        <v>56.37</v>
+      </c>
+      <c r="C31" s="8">
+        <v>69.02</v>
+      </c>
+      <c r="D31" s="8">
+        <v>81.67</v>
+      </c>
+      <c r="E31" s="8">
+        <v>84.44</v>
+      </c>
+      <c r="F31" s="8">
+        <v>87.21</v>
+      </c>
+      <c r="G31" s="8">
+        <v>89.98</v>
+      </c>
+      <c r="H31" s="8">
+        <v>105.1</v>
+      </c>
+      <c r="I31" s="8">
+        <v>120.22</v>
+      </c>
+      <c r="J31" s="8">
+        <v>135.34</v>
+      </c>
+      <c r="K31" s="8">
+        <v>148.16</v>
+      </c>
+      <c r="M31" s="9">
+        <v>27</v>
+      </c>
+      <c r="N31" s="8">
+        <v>160.99</v>
+      </c>
+      <c r="O31" s="8">
+        <v>216.75</v>
+      </c>
+      <c r="P31" s="8">
+        <v>272.51</v>
+      </c>
+      <c r="Q31" s="8">
+        <v>328.27</v>
+      </c>
+      <c r="R31" s="8">
+        <v>384.03</v>
+      </c>
+      <c r="S31" s="8">
+        <v>587.35</v>
+      </c>
+      <c r="T31" s="8">
+        <v>790.68</v>
+      </c>
+      <c r="U31" s="8">
+        <v>994</v>
+      </c>
+      <c r="V31" s="8">
+        <v>1197.32</v>
+      </c>
+      <c r="W31" s="8">
+        <v>1400.65</v>
+      </c>
+    </row>
+    <row r="32" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A32" s="5">
+        <v>28</v>
+      </c>
+      <c r="B32" s="8">
+        <v>57.99</v>
+      </c>
+      <c r="C32" s="8">
+        <v>70.400000000000006</v>
+      </c>
+      <c r="D32" s="8">
+        <v>82.8</v>
+      </c>
+      <c r="E32" s="8">
+        <v>85.2</v>
+      </c>
+      <c r="F32" s="8">
+        <v>87.59</v>
+      </c>
+      <c r="G32" s="8">
+        <v>89.99</v>
+      </c>
+      <c r="H32" s="8">
+        <v>105.32</v>
+      </c>
+      <c r="I32" s="8">
+        <v>120.65</v>
+      </c>
+      <c r="J32" s="8">
+        <v>135.97999999999999</v>
+      </c>
+      <c r="K32" s="8">
+        <v>148.47999999999999</v>
+      </c>
+      <c r="M32" s="9">
+        <v>28</v>
+      </c>
+      <c r="N32" s="8">
+        <v>160.99</v>
+      </c>
+      <c r="O32" s="8">
+        <v>216.75</v>
+      </c>
+      <c r="P32" s="8">
+        <v>272.51</v>
+      </c>
+      <c r="Q32" s="8">
+        <v>328.27</v>
+      </c>
+      <c r="R32" s="8">
+        <v>384.03</v>
+      </c>
+      <c r="S32" s="8">
+        <v>587.35</v>
+      </c>
+      <c r="T32" s="8">
+        <v>790.68</v>
+      </c>
+      <c r="U32" s="8">
+        <v>994</v>
+      </c>
+      <c r="V32" s="8">
+        <v>1197.32</v>
+      </c>
+      <c r="W32" s="8">
+        <v>1400.65</v>
+      </c>
+    </row>
+    <row r="33" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A33" s="5">
+        <v>29</v>
+      </c>
+      <c r="B33" s="8">
+        <v>59.61</v>
+      </c>
+      <c r="C33" s="8">
+        <v>71.77</v>
+      </c>
+      <c r="D33" s="8">
+        <v>83.94</v>
+      </c>
+      <c r="E33" s="8">
+        <v>85.96</v>
+      </c>
+      <c r="F33" s="8">
+        <v>87.98</v>
+      </c>
+      <c r="G33" s="8">
+        <v>90</v>
+      </c>
+      <c r="H33" s="8">
+        <v>105.54</v>
+      </c>
+      <c r="I33" s="8">
+        <v>121.08</v>
+      </c>
+      <c r="J33" s="8">
+        <v>136.62</v>
+      </c>
+      <c r="K33" s="8">
+        <v>148.80000000000001</v>
+      </c>
+      <c r="M33" s="9">
+        <v>29</v>
+      </c>
+      <c r="N33" s="8">
+        <v>160.99</v>
+      </c>
+      <c r="O33" s="8">
+        <v>216.75</v>
+      </c>
+      <c r="P33" s="8">
+        <v>272.51</v>
+      </c>
+      <c r="Q33" s="8">
+        <v>328.27</v>
+      </c>
+      <c r="R33" s="8">
+        <v>384.03</v>
+      </c>
+      <c r="S33" s="8">
+        <v>587.35</v>
+      </c>
+      <c r="T33" s="8">
+        <v>790.68</v>
+      </c>
+      <c r="U33" s="8">
+        <v>994</v>
+      </c>
+      <c r="V33" s="8">
+        <v>1197.32</v>
+      </c>
+      <c r="W33" s="8">
+        <v>1400.65</v>
+      </c>
+    </row>
+    <row r="34" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A34" s="5">
+        <v>30</v>
+      </c>
+      <c r="B34" s="8">
+        <v>61.23</v>
+      </c>
+      <c r="C34" s="8">
+        <v>73.150000000000006</v>
+      </c>
+      <c r="D34" s="8">
+        <v>85.08</v>
+      </c>
+      <c r="E34" s="8">
+        <v>86.72</v>
+      </c>
+      <c r="F34" s="8">
+        <v>88.36</v>
+      </c>
+      <c r="G34" s="8">
+        <v>90.01</v>
+      </c>
+      <c r="H34" s="8">
+        <v>105.76</v>
+      </c>
+      <c r="I34" s="8">
+        <v>121.51</v>
+      </c>
+      <c r="J34" s="8">
+        <v>137.27000000000001</v>
+      </c>
+      <c r="K34" s="8">
+        <v>149.13</v>
+      </c>
+      <c r="M34" s="9">
+        <v>30</v>
+      </c>
+      <c r="N34" s="8">
+        <v>160.99</v>
+      </c>
+      <c r="O34" s="8">
+        <v>216.75</v>
+      </c>
+      <c r="P34" s="8">
+        <v>272.51</v>
+      </c>
+      <c r="Q34" s="8">
+        <v>328.27</v>
+      </c>
+      <c r="R34" s="8">
+        <v>384.03</v>
+      </c>
+      <c r="S34" s="8">
+        <v>587.35</v>
+      </c>
+      <c r="T34" s="8">
+        <v>790.68</v>
+      </c>
+      <c r="U34" s="8">
+        <v>994</v>
+      </c>
+      <c r="V34" s="8">
+        <v>1197.32</v>
+      </c>
+      <c r="W34" s="8">
+        <v>1400.65</v>
+      </c>
+    </row>
+    <row r="35" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A35" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B35" s="8">
+        <v>37.857333333333337</v>
+      </c>
+      <c r="C35" s="8">
+        <v>51.866333333333344</v>
+      </c>
+      <c r="D35" s="8">
+        <v>65.87533333333333</v>
+      </c>
+      <c r="E35" s="8">
+        <v>72.146666666666675</v>
+      </c>
+      <c r="F35" s="8">
+        <v>78.417000000000002</v>
+      </c>
+      <c r="G35" s="8">
+        <v>84.688666666666691</v>
+      </c>
+      <c r="H35" s="8">
+        <v>97.53166666666668</v>
+      </c>
+      <c r="I35" s="8">
+        <v>110.371</v>
+      </c>
+      <c r="J35" s="8">
+        <v>123.21233333333335</v>
+      </c>
+      <c r="K35" s="8">
+        <v>142.09866666666667</v>
+      </c>
+      <c r="M35" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="N35" s="10">
+        <v>160.98999999999987</v>
+      </c>
+      <c r="O35" s="10">
+        <v>216.75</v>
+      </c>
+      <c r="P35" s="10">
+        <v>272.51000000000016</v>
+      </c>
+      <c r="Q35" s="10">
+        <v>328.27000000000027</v>
+      </c>
+      <c r="R35" s="10">
+        <v>384.03000000000003</v>
+      </c>
+      <c r="S35" s="10">
+        <v>587.35000000000014</v>
+      </c>
+      <c r="T35" s="10">
+        <v>790.68000000000018</v>
+      </c>
+      <c r="U35" s="10">
+        <v>994</v>
+      </c>
+      <c r="V35" s="10">
+        <v>1197.32</v>
+      </c>
+      <c r="W35" s="10">
+        <v>1400.6500000000008</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B2:K2"/>
+    <mergeCell ref="M1:W1"/>
+    <mergeCell ref="N2:W2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A2E7E46-B70B-4DB0-97AE-2138287FA00A}">
   <dimension ref="A1:W35"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -3041,7 +5371,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D32525DC-1FAE-40FA-B3A1-6E6C0B62B72E}">
   <dimension ref="A1:W35"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -5364,7 +7694,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <sheetPr codeName="Sheet9">
     <tabColor rgb="FFFFFF00"/>

</xml_diff>

<commit_message>
📊 Update NAIC content history - 2026-05-02
</commit_message>
<xml_diff>
--- a/docs/content_history/pbr-2026-vm20-table-f-g-current-spreads.xlsx
+++ b/docs/content_history/pbr-2026-vm20-table-f-g-current-spreads.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\PBR\VM20_VM22_ProductSupport\PBR Production Web Data\Current Year\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{799202CB-DE5D-43F8-B5E5-7B883A1D2518}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF0A3062-E358-4E67-AC54-79F2A4C44FD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="39375" yWindow="3060" windowWidth="25140" windowHeight="15225" tabRatio="795" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="795" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="March_2026" sheetId="26" r:id="rId1"/>
-    <sheet name="February_2026" sheetId="25" r:id="rId2"/>
-    <sheet name="January_2026" sheetId="24" r:id="rId3"/>
-    <sheet name="LEGAL DISCLAIMER" sheetId="11" r:id="rId4"/>
+    <sheet name="April_2026" sheetId="27" r:id="rId1"/>
+    <sheet name="March_2026" sheetId="26" r:id="rId2"/>
+    <sheet name="February_2026" sheetId="25" r:id="rId3"/>
+    <sheet name="January_2026" sheetId="24" r:id="rId4"/>
+    <sheet name="LEGAL DISCLAIMER" sheetId="11" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="34">
   <si>
     <t>WAL</t>
   </si>
@@ -129,6 +130,12 @@
   </si>
   <si>
     <t>Table G. (03/31/2026) Below Investment Grade Current Benchmark Spreads (in bps)</t>
+  </si>
+  <si>
+    <t>Table F (04/30/2026)  Investment Grade Current Benchmark Spreads (in bps)</t>
+  </si>
+  <si>
+    <t>Table G. (04/30/2026) Below Investment Grade Current Benchmark Spreads (in bps)</t>
   </si>
 </sst>
 </file>
@@ -405,7 +412,7 @@
                   <a14:compatExt spid="_x0000_s4104"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000008100000}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000008100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -726,15 +733,2338 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3EEC94F4-4E93-438D-92F8-5C9CBA48C22A}">
+  <dimension ref="A1:W35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.140625" customWidth="1"/>
+    <col min="13" max="23" width="11.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="M1" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="N1" s="14"/>
+      <c r="O1" s="14"/>
+      <c r="P1" s="14"/>
+      <c r="Q1" s="14"/>
+      <c r="R1" s="14"/>
+      <c r="S1" s="14"/>
+      <c r="T1" s="14"/>
+      <c r="U1" s="14"/>
+      <c r="V1" s="14"/>
+      <c r="W1" s="15"/>
+    </row>
+    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12"/>
+      <c r="K2" s="12"/>
+      <c r="M2" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="N2" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="O2" s="12"/>
+      <c r="P2" s="12"/>
+      <c r="Q2" s="12"/>
+      <c r="R2" s="12"/>
+      <c r="S2" s="12"/>
+      <c r="T2" s="12"/>
+      <c r="U2" s="12"/>
+      <c r="V2" s="12"/>
+      <c r="W2" s="12"/>
+    </row>
+    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="5">
+        <v>1</v>
+      </c>
+      <c r="C3" s="5">
+        <v>2</v>
+      </c>
+      <c r="D3" s="5">
+        <v>3</v>
+      </c>
+      <c r="E3" s="5">
+        <v>4</v>
+      </c>
+      <c r="F3" s="5">
+        <v>5</v>
+      </c>
+      <c r="G3" s="5">
+        <v>6</v>
+      </c>
+      <c r="H3" s="5">
+        <v>7</v>
+      </c>
+      <c r="I3" s="5">
+        <v>8</v>
+      </c>
+      <c r="J3" s="5">
+        <v>9</v>
+      </c>
+      <c r="K3" s="5">
+        <v>10</v>
+      </c>
+      <c r="M3" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="N3" s="5">
+        <v>11</v>
+      </c>
+      <c r="O3" s="5">
+        <v>12</v>
+      </c>
+      <c r="P3" s="5">
+        <v>13</v>
+      </c>
+      <c r="Q3" s="5">
+        <v>14</v>
+      </c>
+      <c r="R3" s="5">
+        <v>15</v>
+      </c>
+      <c r="S3" s="5">
+        <v>16</v>
+      </c>
+      <c r="T3" s="5">
+        <v>17</v>
+      </c>
+      <c r="U3" s="5">
+        <v>18</v>
+      </c>
+      <c r="V3" s="5">
+        <v>19</v>
+      </c>
+      <c r="W3" s="5">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="M4" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="P4" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q4" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="R4" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="S4" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="T4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="U4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="V4" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="W4" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A5" s="5">
+        <v>1</v>
+      </c>
+      <c r="B5" s="8">
+        <v>18.170000000000002</v>
+      </c>
+      <c r="C5" s="8">
+        <v>23.59</v>
+      </c>
+      <c r="D5" s="8">
+        <v>29</v>
+      </c>
+      <c r="E5" s="8">
+        <v>35.08</v>
+      </c>
+      <c r="F5" s="8">
+        <v>41.16</v>
+      </c>
+      <c r="G5" s="8">
+        <v>47.23</v>
+      </c>
+      <c r="H5" s="8">
+        <v>55.49</v>
+      </c>
+      <c r="I5" s="8">
+        <v>63.75</v>
+      </c>
+      <c r="J5" s="8">
+        <v>72</v>
+      </c>
+      <c r="K5" s="8">
+        <v>105.08</v>
+      </c>
+      <c r="M5" s="9">
+        <v>1</v>
+      </c>
+      <c r="N5" s="8">
+        <v>138.15</v>
+      </c>
+      <c r="O5" s="8">
+        <v>187.66</v>
+      </c>
+      <c r="P5" s="8">
+        <v>237.17</v>
+      </c>
+      <c r="Q5" s="8">
+        <v>286.68</v>
+      </c>
+      <c r="R5" s="8">
+        <v>336.18</v>
+      </c>
+      <c r="S5" s="8">
+        <v>527.12</v>
+      </c>
+      <c r="T5" s="8">
+        <v>718.06</v>
+      </c>
+      <c r="U5" s="8">
+        <v>909</v>
+      </c>
+      <c r="V5" s="8">
+        <v>1099.94</v>
+      </c>
+      <c r="W5" s="8">
+        <v>1290.8800000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A6" s="5">
+        <v>2</v>
+      </c>
+      <c r="B6" s="8">
+        <v>17.149999999999999</v>
+      </c>
+      <c r="C6" s="8">
+        <v>24.9</v>
+      </c>
+      <c r="D6" s="8">
+        <v>32.659999999999997</v>
+      </c>
+      <c r="E6" s="8">
+        <v>39.18</v>
+      </c>
+      <c r="F6" s="8">
+        <v>45.7</v>
+      </c>
+      <c r="G6" s="8">
+        <v>52.23</v>
+      </c>
+      <c r="H6" s="8">
+        <v>61.09</v>
+      </c>
+      <c r="I6" s="8">
+        <v>69.959999999999994</v>
+      </c>
+      <c r="J6" s="8">
+        <v>78.83</v>
+      </c>
+      <c r="K6" s="8">
+        <v>108.49</v>
+      </c>
+      <c r="M6" s="9">
+        <v>2</v>
+      </c>
+      <c r="N6" s="8">
+        <v>138.15</v>
+      </c>
+      <c r="O6" s="8">
+        <v>187.66</v>
+      </c>
+      <c r="P6" s="8">
+        <v>237.17</v>
+      </c>
+      <c r="Q6" s="8">
+        <v>286.68</v>
+      </c>
+      <c r="R6" s="8">
+        <v>336.18</v>
+      </c>
+      <c r="S6" s="8">
+        <v>527.12</v>
+      </c>
+      <c r="T6" s="8">
+        <v>718.06</v>
+      </c>
+      <c r="U6" s="8">
+        <v>909</v>
+      </c>
+      <c r="V6" s="8">
+        <v>1099.94</v>
+      </c>
+      <c r="W6" s="8">
+        <v>1290.8800000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A7" s="5">
+        <v>3</v>
+      </c>
+      <c r="B7" s="8">
+        <v>16.13</v>
+      </c>
+      <c r="C7" s="8">
+        <v>26.22</v>
+      </c>
+      <c r="D7" s="8">
+        <v>36.31</v>
+      </c>
+      <c r="E7" s="8">
+        <v>43.28</v>
+      </c>
+      <c r="F7" s="8">
+        <v>50.25</v>
+      </c>
+      <c r="G7" s="8">
+        <v>57.22</v>
+      </c>
+      <c r="H7" s="8">
+        <v>66.7</v>
+      </c>
+      <c r="I7" s="8">
+        <v>76.17</v>
+      </c>
+      <c r="J7" s="8">
+        <v>85.65</v>
+      </c>
+      <c r="K7" s="8">
+        <v>111.9</v>
+      </c>
+      <c r="M7" s="9">
+        <v>3</v>
+      </c>
+      <c r="N7" s="8">
+        <v>138.15</v>
+      </c>
+      <c r="O7" s="8">
+        <v>187.66</v>
+      </c>
+      <c r="P7" s="8">
+        <v>237.17</v>
+      </c>
+      <c r="Q7" s="8">
+        <v>286.68</v>
+      </c>
+      <c r="R7" s="8">
+        <v>336.18</v>
+      </c>
+      <c r="S7" s="8">
+        <v>527.12</v>
+      </c>
+      <c r="T7" s="8">
+        <v>718.06</v>
+      </c>
+      <c r="U7" s="8">
+        <v>909</v>
+      </c>
+      <c r="V7" s="8">
+        <v>1099.94</v>
+      </c>
+      <c r="W7" s="8">
+        <v>1290.8800000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A8" s="5">
+        <v>4</v>
+      </c>
+      <c r="B8" s="8">
+        <v>15.11</v>
+      </c>
+      <c r="C8" s="8">
+        <v>27.54</v>
+      </c>
+      <c r="D8" s="8">
+        <v>39.97</v>
+      </c>
+      <c r="E8" s="8">
+        <v>47.38</v>
+      </c>
+      <c r="F8" s="8">
+        <v>54.8</v>
+      </c>
+      <c r="G8" s="8">
+        <v>62.22</v>
+      </c>
+      <c r="H8" s="8">
+        <v>72.3</v>
+      </c>
+      <c r="I8" s="8">
+        <v>82.39</v>
+      </c>
+      <c r="J8" s="8">
+        <v>92.47</v>
+      </c>
+      <c r="K8" s="8">
+        <v>115.31</v>
+      </c>
+      <c r="M8" s="9">
+        <v>4</v>
+      </c>
+      <c r="N8" s="8">
+        <v>138.15</v>
+      </c>
+      <c r="O8" s="8">
+        <v>187.66</v>
+      </c>
+      <c r="P8" s="8">
+        <v>237.17</v>
+      </c>
+      <c r="Q8" s="8">
+        <v>286.68</v>
+      </c>
+      <c r="R8" s="8">
+        <v>336.18</v>
+      </c>
+      <c r="S8" s="8">
+        <v>527.12</v>
+      </c>
+      <c r="T8" s="8">
+        <v>718.06</v>
+      </c>
+      <c r="U8" s="8">
+        <v>909</v>
+      </c>
+      <c r="V8" s="8">
+        <v>1099.94</v>
+      </c>
+      <c r="W8" s="8">
+        <v>1290.8800000000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A9" s="5">
+        <v>5</v>
+      </c>
+      <c r="B9" s="8">
+        <v>16.739999999999998</v>
+      </c>
+      <c r="C9" s="8">
+        <v>29.99</v>
+      </c>
+      <c r="D9" s="8">
+        <v>43.25</v>
+      </c>
+      <c r="E9" s="8">
+        <v>51</v>
+      </c>
+      <c r="F9" s="8">
+        <v>58.74</v>
+      </c>
+      <c r="G9" s="8">
+        <v>66.489999999999995</v>
+      </c>
+      <c r="H9" s="8">
+        <v>76.42</v>
+      </c>
+      <c r="I9" s="8">
+        <v>86.36</v>
+      </c>
+      <c r="J9" s="8">
+        <v>96.3</v>
+      </c>
+      <c r="K9" s="8">
+        <v>117.23</v>
+      </c>
+      <c r="M9" s="9">
+        <v>5</v>
+      </c>
+      <c r="N9" s="8">
+        <v>138.15</v>
+      </c>
+      <c r="O9" s="8">
+        <v>187.66</v>
+      </c>
+      <c r="P9" s="8">
+        <v>237.17</v>
+      </c>
+      <c r="Q9" s="8">
+        <v>286.68</v>
+      </c>
+      <c r="R9" s="8">
+        <v>336.18</v>
+      </c>
+      <c r="S9" s="8">
+        <v>527.12</v>
+      </c>
+      <c r="T9" s="8">
+        <v>718.06</v>
+      </c>
+      <c r="U9" s="8">
+        <v>909</v>
+      </c>
+      <c r="V9" s="8">
+        <v>1099.94</v>
+      </c>
+      <c r="W9" s="8">
+        <v>1290.8800000000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A10" s="5">
+        <v>6</v>
+      </c>
+      <c r="B10" s="8">
+        <v>18.37</v>
+      </c>
+      <c r="C10" s="8">
+        <v>32.450000000000003</v>
+      </c>
+      <c r="D10" s="8">
+        <v>46.53</v>
+      </c>
+      <c r="E10" s="8">
+        <v>54.61</v>
+      </c>
+      <c r="F10" s="8">
+        <v>62.68</v>
+      </c>
+      <c r="G10" s="8">
+        <v>70.760000000000005</v>
+      </c>
+      <c r="H10" s="8">
+        <v>80.55</v>
+      </c>
+      <c r="I10" s="8">
+        <v>90.33</v>
+      </c>
+      <c r="J10" s="8">
+        <v>100.12</v>
+      </c>
+      <c r="K10" s="8">
+        <v>119.14</v>
+      </c>
+      <c r="M10" s="9">
+        <v>6</v>
+      </c>
+      <c r="N10" s="8">
+        <v>138.15</v>
+      </c>
+      <c r="O10" s="8">
+        <v>187.66</v>
+      </c>
+      <c r="P10" s="8">
+        <v>237.17</v>
+      </c>
+      <c r="Q10" s="8">
+        <v>286.68</v>
+      </c>
+      <c r="R10" s="8">
+        <v>336.18</v>
+      </c>
+      <c r="S10" s="8">
+        <v>527.12</v>
+      </c>
+      <c r="T10" s="8">
+        <v>718.06</v>
+      </c>
+      <c r="U10" s="8">
+        <v>909</v>
+      </c>
+      <c r="V10" s="8">
+        <v>1099.94</v>
+      </c>
+      <c r="W10" s="8">
+        <v>1290.8800000000001</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A11" s="5">
+        <v>7</v>
+      </c>
+      <c r="B11" s="8">
+        <v>20.64</v>
+      </c>
+      <c r="C11" s="8">
+        <v>35.64</v>
+      </c>
+      <c r="D11" s="8">
+        <v>50.65</v>
+      </c>
+      <c r="E11" s="8">
+        <v>58.7</v>
+      </c>
+      <c r="F11" s="8">
+        <v>66.75</v>
+      </c>
+      <c r="G11" s="8">
+        <v>74.8</v>
+      </c>
+      <c r="H11" s="8">
+        <v>84.67</v>
+      </c>
+      <c r="I11" s="8">
+        <v>94.55</v>
+      </c>
+      <c r="J11" s="8">
+        <v>104.43</v>
+      </c>
+      <c r="K11" s="8">
+        <v>121.29</v>
+      </c>
+      <c r="M11" s="9">
+        <v>7</v>
+      </c>
+      <c r="N11" s="8">
+        <v>138.15</v>
+      </c>
+      <c r="O11" s="8">
+        <v>187.66</v>
+      </c>
+      <c r="P11" s="8">
+        <v>237.17</v>
+      </c>
+      <c r="Q11" s="8">
+        <v>286.68</v>
+      </c>
+      <c r="R11" s="8">
+        <v>336.18</v>
+      </c>
+      <c r="S11" s="8">
+        <v>527.12</v>
+      </c>
+      <c r="T11" s="8">
+        <v>718.06</v>
+      </c>
+      <c r="U11" s="8">
+        <v>909</v>
+      </c>
+      <c r="V11" s="8">
+        <v>1099.94</v>
+      </c>
+      <c r="W11" s="8">
+        <v>1290.8800000000001</v>
+      </c>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A12" s="5">
+        <v>8</v>
+      </c>
+      <c r="B12" s="8">
+        <v>22.9</v>
+      </c>
+      <c r="C12" s="8">
+        <v>38.840000000000003</v>
+      </c>
+      <c r="D12" s="8">
+        <v>54.77</v>
+      </c>
+      <c r="E12" s="8">
+        <v>62.79</v>
+      </c>
+      <c r="F12" s="8">
+        <v>70.81</v>
+      </c>
+      <c r="G12" s="8">
+        <v>78.83</v>
+      </c>
+      <c r="H12" s="8">
+        <v>88.8</v>
+      </c>
+      <c r="I12" s="8">
+        <v>98.76</v>
+      </c>
+      <c r="J12" s="8">
+        <v>108.73</v>
+      </c>
+      <c r="K12" s="8">
+        <v>123.44</v>
+      </c>
+      <c r="M12" s="9">
+        <v>8</v>
+      </c>
+      <c r="N12" s="8">
+        <v>138.15</v>
+      </c>
+      <c r="O12" s="8">
+        <v>187.66</v>
+      </c>
+      <c r="P12" s="8">
+        <v>237.17</v>
+      </c>
+      <c r="Q12" s="8">
+        <v>286.68</v>
+      </c>
+      <c r="R12" s="8">
+        <v>336.18</v>
+      </c>
+      <c r="S12" s="8">
+        <v>527.12</v>
+      </c>
+      <c r="T12" s="8">
+        <v>718.06</v>
+      </c>
+      <c r="U12" s="8">
+        <v>909</v>
+      </c>
+      <c r="V12" s="8">
+        <v>1099.94</v>
+      </c>
+      <c r="W12" s="8">
+        <v>1290.8800000000001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A13" s="5">
+        <v>9</v>
+      </c>
+      <c r="B13" s="8">
+        <v>25.16</v>
+      </c>
+      <c r="C13" s="8">
+        <v>42.03</v>
+      </c>
+      <c r="D13" s="8">
+        <v>58.9</v>
+      </c>
+      <c r="E13" s="8">
+        <v>66.89</v>
+      </c>
+      <c r="F13" s="8">
+        <v>74.88</v>
+      </c>
+      <c r="G13" s="8">
+        <v>82.87</v>
+      </c>
+      <c r="H13" s="8">
+        <v>92.92</v>
+      </c>
+      <c r="I13" s="8">
+        <v>102.98</v>
+      </c>
+      <c r="J13" s="8">
+        <v>113.03</v>
+      </c>
+      <c r="K13" s="8">
+        <v>125.59</v>
+      </c>
+      <c r="M13" s="9">
+        <v>9</v>
+      </c>
+      <c r="N13" s="8">
+        <v>138.15</v>
+      </c>
+      <c r="O13" s="8">
+        <v>187.66</v>
+      </c>
+      <c r="P13" s="8">
+        <v>237.17</v>
+      </c>
+      <c r="Q13" s="8">
+        <v>286.68</v>
+      </c>
+      <c r="R13" s="8">
+        <v>336.18</v>
+      </c>
+      <c r="S13" s="8">
+        <v>527.12</v>
+      </c>
+      <c r="T13" s="8">
+        <v>718.06</v>
+      </c>
+      <c r="U13" s="8">
+        <v>909</v>
+      </c>
+      <c r="V13" s="8">
+        <v>1099.94</v>
+      </c>
+      <c r="W13" s="8">
+        <v>1290.8800000000001</v>
+      </c>
+    </row>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A14" s="5">
+        <v>10</v>
+      </c>
+      <c r="B14" s="8">
+        <v>26.79</v>
+      </c>
+      <c r="C14" s="8">
+        <v>43.34</v>
+      </c>
+      <c r="D14" s="8">
+        <v>59.89</v>
+      </c>
+      <c r="E14" s="8">
+        <v>67.56</v>
+      </c>
+      <c r="F14" s="8">
+        <v>75.22</v>
+      </c>
+      <c r="G14" s="8">
+        <v>82.89</v>
+      </c>
+      <c r="H14" s="8">
+        <v>93.18</v>
+      </c>
+      <c r="I14" s="8">
+        <v>103.47</v>
+      </c>
+      <c r="J14" s="8">
+        <v>113.76</v>
+      </c>
+      <c r="K14" s="8">
+        <v>125.96</v>
+      </c>
+      <c r="M14" s="9">
+        <v>10</v>
+      </c>
+      <c r="N14" s="8">
+        <v>138.15</v>
+      </c>
+      <c r="O14" s="8">
+        <v>187.66</v>
+      </c>
+      <c r="P14" s="8">
+        <v>237.17</v>
+      </c>
+      <c r="Q14" s="8">
+        <v>286.68</v>
+      </c>
+      <c r="R14" s="8">
+        <v>336.18</v>
+      </c>
+      <c r="S14" s="8">
+        <v>527.12</v>
+      </c>
+      <c r="T14" s="8">
+        <v>718.06</v>
+      </c>
+      <c r="U14" s="8">
+        <v>909</v>
+      </c>
+      <c r="V14" s="8">
+        <v>1099.94</v>
+      </c>
+      <c r="W14" s="8">
+        <v>1290.8800000000001</v>
+      </c>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A15" s="5">
+        <v>11</v>
+      </c>
+      <c r="B15" s="8">
+        <v>28.41</v>
+      </c>
+      <c r="C15" s="8">
+        <v>44.65</v>
+      </c>
+      <c r="D15" s="8">
+        <v>60.89</v>
+      </c>
+      <c r="E15" s="8">
+        <v>68.23</v>
+      </c>
+      <c r="F15" s="8">
+        <v>75.569999999999993</v>
+      </c>
+      <c r="G15" s="8">
+        <v>82.91</v>
+      </c>
+      <c r="H15" s="8">
+        <v>93.44</v>
+      </c>
+      <c r="I15" s="8">
+        <v>103.97</v>
+      </c>
+      <c r="J15" s="8">
+        <v>114.5</v>
+      </c>
+      <c r="K15" s="8">
+        <v>126.32</v>
+      </c>
+      <c r="M15" s="9">
+        <v>11</v>
+      </c>
+      <c r="N15" s="8">
+        <v>138.15</v>
+      </c>
+      <c r="O15" s="8">
+        <v>187.66</v>
+      </c>
+      <c r="P15" s="8">
+        <v>237.17</v>
+      </c>
+      <c r="Q15" s="8">
+        <v>286.68</v>
+      </c>
+      <c r="R15" s="8">
+        <v>336.18</v>
+      </c>
+      <c r="S15" s="8">
+        <v>527.12</v>
+      </c>
+      <c r="T15" s="8">
+        <v>718.06</v>
+      </c>
+      <c r="U15" s="8">
+        <v>909</v>
+      </c>
+      <c r="V15" s="8">
+        <v>1099.94</v>
+      </c>
+      <c r="W15" s="8">
+        <v>1290.8800000000001</v>
+      </c>
+    </row>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A16" s="5">
+        <v>12</v>
+      </c>
+      <c r="B16" s="8">
+        <v>30.04</v>
+      </c>
+      <c r="C16" s="8">
+        <v>45.96</v>
+      </c>
+      <c r="D16" s="8">
+        <v>61.88</v>
+      </c>
+      <c r="E16" s="8">
+        <v>68.900000000000006</v>
+      </c>
+      <c r="F16" s="8">
+        <v>75.91</v>
+      </c>
+      <c r="G16" s="8">
+        <v>82.93</v>
+      </c>
+      <c r="H16" s="8">
+        <v>93.7</v>
+      </c>
+      <c r="I16" s="8">
+        <v>104.46</v>
+      </c>
+      <c r="J16" s="8">
+        <v>115.23</v>
+      </c>
+      <c r="K16" s="8">
+        <v>126.69</v>
+      </c>
+      <c r="M16" s="9">
+        <v>12</v>
+      </c>
+      <c r="N16" s="8">
+        <v>138.15</v>
+      </c>
+      <c r="O16" s="8">
+        <v>187.66</v>
+      </c>
+      <c r="P16" s="8">
+        <v>237.17</v>
+      </c>
+      <c r="Q16" s="8">
+        <v>286.68</v>
+      </c>
+      <c r="R16" s="8">
+        <v>336.18</v>
+      </c>
+      <c r="S16" s="8">
+        <v>527.12</v>
+      </c>
+      <c r="T16" s="8">
+        <v>718.06</v>
+      </c>
+      <c r="U16" s="8">
+        <v>909</v>
+      </c>
+      <c r="V16" s="8">
+        <v>1099.94</v>
+      </c>
+      <c r="W16" s="8">
+        <v>1290.8800000000001</v>
+      </c>
+    </row>
+    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A17" s="5">
+        <v>13</v>
+      </c>
+      <c r="B17" s="8">
+        <v>31.66</v>
+      </c>
+      <c r="C17" s="8">
+        <v>47.27</v>
+      </c>
+      <c r="D17" s="8">
+        <v>62.88</v>
+      </c>
+      <c r="E17" s="8">
+        <v>69.569999999999993</v>
+      </c>
+      <c r="F17" s="8">
+        <v>76.260000000000005</v>
+      </c>
+      <c r="G17" s="8">
+        <v>82.95</v>
+      </c>
+      <c r="H17" s="8">
+        <v>93.95</v>
+      </c>
+      <c r="I17" s="8">
+        <v>104.96</v>
+      </c>
+      <c r="J17" s="8">
+        <v>115.96</v>
+      </c>
+      <c r="K17" s="8">
+        <v>127.06</v>
+      </c>
+      <c r="M17" s="9">
+        <v>13</v>
+      </c>
+      <c r="N17" s="8">
+        <v>138.15</v>
+      </c>
+      <c r="O17" s="8">
+        <v>187.66</v>
+      </c>
+      <c r="P17" s="8">
+        <v>237.17</v>
+      </c>
+      <c r="Q17" s="8">
+        <v>286.68</v>
+      </c>
+      <c r="R17" s="8">
+        <v>336.18</v>
+      </c>
+      <c r="S17" s="8">
+        <v>527.12</v>
+      </c>
+      <c r="T17" s="8">
+        <v>718.06</v>
+      </c>
+      <c r="U17" s="8">
+        <v>909</v>
+      </c>
+      <c r="V17" s="8">
+        <v>1099.94</v>
+      </c>
+      <c r="W17" s="8">
+        <v>1290.8800000000001</v>
+      </c>
+    </row>
+    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A18" s="5">
+        <v>14</v>
+      </c>
+      <c r="B18" s="8">
+        <v>33.29</v>
+      </c>
+      <c r="C18" s="8">
+        <v>48.58</v>
+      </c>
+      <c r="D18" s="8">
+        <v>63.87</v>
+      </c>
+      <c r="E18" s="8">
+        <v>70.239999999999995</v>
+      </c>
+      <c r="F18" s="8">
+        <v>76.599999999999994</v>
+      </c>
+      <c r="G18" s="8">
+        <v>82.97</v>
+      </c>
+      <c r="H18" s="8">
+        <v>94.21</v>
+      </c>
+      <c r="I18" s="8">
+        <v>105.45</v>
+      </c>
+      <c r="J18" s="8">
+        <v>116.69</v>
+      </c>
+      <c r="K18" s="8">
+        <v>127.42</v>
+      </c>
+      <c r="M18" s="9">
+        <v>14</v>
+      </c>
+      <c r="N18" s="8">
+        <v>138.15</v>
+      </c>
+      <c r="O18" s="8">
+        <v>187.66</v>
+      </c>
+      <c r="P18" s="8">
+        <v>237.17</v>
+      </c>
+      <c r="Q18" s="8">
+        <v>286.68</v>
+      </c>
+      <c r="R18" s="8">
+        <v>336.18</v>
+      </c>
+      <c r="S18" s="8">
+        <v>527.12</v>
+      </c>
+      <c r="T18" s="8">
+        <v>718.06</v>
+      </c>
+      <c r="U18" s="8">
+        <v>909</v>
+      </c>
+      <c r="V18" s="8">
+        <v>1099.94</v>
+      </c>
+      <c r="W18" s="8">
+        <v>1290.8800000000001</v>
+      </c>
+    </row>
+    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A19" s="5">
+        <v>15</v>
+      </c>
+      <c r="B19" s="8">
+        <v>34.909999999999997</v>
+      </c>
+      <c r="C19" s="8">
+        <v>49.89</v>
+      </c>
+      <c r="D19" s="8">
+        <v>64.87</v>
+      </c>
+      <c r="E19" s="8">
+        <v>70.91</v>
+      </c>
+      <c r="F19" s="8">
+        <v>76.95</v>
+      </c>
+      <c r="G19" s="8">
+        <v>82.99</v>
+      </c>
+      <c r="H19" s="8">
+        <v>94.47</v>
+      </c>
+      <c r="I19" s="8">
+        <v>105.95</v>
+      </c>
+      <c r="J19" s="8">
+        <v>117.43</v>
+      </c>
+      <c r="K19" s="8">
+        <v>127.79</v>
+      </c>
+      <c r="M19" s="9">
+        <v>15</v>
+      </c>
+      <c r="N19" s="8">
+        <v>138.15</v>
+      </c>
+      <c r="O19" s="8">
+        <v>187.66</v>
+      </c>
+      <c r="P19" s="8">
+        <v>237.17</v>
+      </c>
+      <c r="Q19" s="8">
+        <v>286.68</v>
+      </c>
+      <c r="R19" s="8">
+        <v>336.18</v>
+      </c>
+      <c r="S19" s="8">
+        <v>527.12</v>
+      </c>
+      <c r="T19" s="8">
+        <v>718.06</v>
+      </c>
+      <c r="U19" s="8">
+        <v>909</v>
+      </c>
+      <c r="V19" s="8">
+        <v>1099.94</v>
+      </c>
+      <c r="W19" s="8">
+        <v>1290.8800000000001</v>
+      </c>
+    </row>
+    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A20" s="5">
+        <v>16</v>
+      </c>
+      <c r="B20" s="8">
+        <v>36.54</v>
+      </c>
+      <c r="C20" s="8">
+        <v>51.2</v>
+      </c>
+      <c r="D20" s="8">
+        <v>65.86</v>
+      </c>
+      <c r="E20" s="8">
+        <v>71.58</v>
+      </c>
+      <c r="F20" s="8">
+        <v>77.290000000000006</v>
+      </c>
+      <c r="G20" s="8">
+        <v>83.01</v>
+      </c>
+      <c r="H20" s="8">
+        <v>94.73</v>
+      </c>
+      <c r="I20" s="8">
+        <v>106.44</v>
+      </c>
+      <c r="J20" s="8">
+        <v>118.16</v>
+      </c>
+      <c r="K20" s="8">
+        <v>128.16</v>
+      </c>
+      <c r="M20" s="9">
+        <v>16</v>
+      </c>
+      <c r="N20" s="8">
+        <v>138.15</v>
+      </c>
+      <c r="O20" s="8">
+        <v>187.66</v>
+      </c>
+      <c r="P20" s="8">
+        <v>237.17</v>
+      </c>
+      <c r="Q20" s="8">
+        <v>286.68</v>
+      </c>
+      <c r="R20" s="8">
+        <v>336.18</v>
+      </c>
+      <c r="S20" s="8">
+        <v>527.12</v>
+      </c>
+      <c r="T20" s="8">
+        <v>718.06</v>
+      </c>
+      <c r="U20" s="8">
+        <v>909</v>
+      </c>
+      <c r="V20" s="8">
+        <v>1099.94</v>
+      </c>
+      <c r="W20" s="8">
+        <v>1290.8800000000001</v>
+      </c>
+    </row>
+    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A21" s="5">
+        <v>17</v>
+      </c>
+      <c r="B21" s="8">
+        <v>38.17</v>
+      </c>
+      <c r="C21" s="8">
+        <v>52.51</v>
+      </c>
+      <c r="D21" s="8">
+        <v>66.86</v>
+      </c>
+      <c r="E21" s="8">
+        <v>72.25</v>
+      </c>
+      <c r="F21" s="8">
+        <v>77.64</v>
+      </c>
+      <c r="G21" s="8">
+        <v>83.03</v>
+      </c>
+      <c r="H21" s="8">
+        <v>94.98</v>
+      </c>
+      <c r="I21" s="8">
+        <v>106.94</v>
+      </c>
+      <c r="J21" s="8">
+        <v>118.89</v>
+      </c>
+      <c r="K21" s="8">
+        <v>128.52000000000001</v>
+      </c>
+      <c r="M21" s="9">
+        <v>17</v>
+      </c>
+      <c r="N21" s="8">
+        <v>138.15</v>
+      </c>
+      <c r="O21" s="8">
+        <v>187.66</v>
+      </c>
+      <c r="P21" s="8">
+        <v>237.17</v>
+      </c>
+      <c r="Q21" s="8">
+        <v>286.68</v>
+      </c>
+      <c r="R21" s="8">
+        <v>336.18</v>
+      </c>
+      <c r="S21" s="8">
+        <v>527.12</v>
+      </c>
+      <c r="T21" s="8">
+        <v>718.06</v>
+      </c>
+      <c r="U21" s="8">
+        <v>909</v>
+      </c>
+      <c r="V21" s="8">
+        <v>1099.94</v>
+      </c>
+      <c r="W21" s="8">
+        <v>1290.8800000000001</v>
+      </c>
+    </row>
+    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A22" s="5">
+        <v>18</v>
+      </c>
+      <c r="B22" s="8">
+        <v>39.79</v>
+      </c>
+      <c r="C22" s="8">
+        <v>53.82</v>
+      </c>
+      <c r="D22" s="8">
+        <v>67.849999999999994</v>
+      </c>
+      <c r="E22" s="8">
+        <v>72.92</v>
+      </c>
+      <c r="F22" s="8">
+        <v>77.98</v>
+      </c>
+      <c r="G22" s="8">
+        <v>83.05</v>
+      </c>
+      <c r="H22" s="8">
+        <v>95.24</v>
+      </c>
+      <c r="I22" s="8">
+        <v>107.43</v>
+      </c>
+      <c r="J22" s="8">
+        <v>119.62</v>
+      </c>
+      <c r="K22" s="8">
+        <v>128.88999999999999</v>
+      </c>
+      <c r="M22" s="9">
+        <v>18</v>
+      </c>
+      <c r="N22" s="8">
+        <v>138.15</v>
+      </c>
+      <c r="O22" s="8">
+        <v>187.66</v>
+      </c>
+      <c r="P22" s="8">
+        <v>237.17</v>
+      </c>
+      <c r="Q22" s="8">
+        <v>286.68</v>
+      </c>
+      <c r="R22" s="8">
+        <v>336.18</v>
+      </c>
+      <c r="S22" s="8">
+        <v>527.12</v>
+      </c>
+      <c r="T22" s="8">
+        <v>718.06</v>
+      </c>
+      <c r="U22" s="8">
+        <v>909</v>
+      </c>
+      <c r="V22" s="8">
+        <v>1099.94</v>
+      </c>
+      <c r="W22" s="8">
+        <v>1290.8800000000001</v>
+      </c>
+    </row>
+    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A23" s="5">
+        <v>19</v>
+      </c>
+      <c r="B23" s="8">
+        <v>41.42</v>
+      </c>
+      <c r="C23" s="8">
+        <v>55.13</v>
+      </c>
+      <c r="D23" s="8">
+        <v>68.849999999999994</v>
+      </c>
+      <c r="E23" s="8">
+        <v>73.59</v>
+      </c>
+      <c r="F23" s="8">
+        <v>78.33</v>
+      </c>
+      <c r="G23" s="8">
+        <v>83.07</v>
+      </c>
+      <c r="H23" s="8">
+        <v>95.5</v>
+      </c>
+      <c r="I23" s="8">
+        <v>107.93</v>
+      </c>
+      <c r="J23" s="8">
+        <v>120.36</v>
+      </c>
+      <c r="K23" s="8">
+        <v>129.25</v>
+      </c>
+      <c r="M23" s="9">
+        <v>19</v>
+      </c>
+      <c r="N23" s="8">
+        <v>138.15</v>
+      </c>
+      <c r="O23" s="8">
+        <v>187.66</v>
+      </c>
+      <c r="P23" s="8">
+        <v>237.17</v>
+      </c>
+      <c r="Q23" s="8">
+        <v>286.68</v>
+      </c>
+      <c r="R23" s="8">
+        <v>336.18</v>
+      </c>
+      <c r="S23" s="8">
+        <v>527.12</v>
+      </c>
+      <c r="T23" s="8">
+        <v>718.06</v>
+      </c>
+      <c r="U23" s="8">
+        <v>909</v>
+      </c>
+      <c r="V23" s="8">
+        <v>1099.94</v>
+      </c>
+      <c r="W23" s="8">
+        <v>1290.8800000000001</v>
+      </c>
+    </row>
+    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A24" s="5">
+        <v>20</v>
+      </c>
+      <c r="B24" s="8">
+        <v>43.04</v>
+      </c>
+      <c r="C24" s="8">
+        <v>56.44</v>
+      </c>
+      <c r="D24" s="8">
+        <v>69.84</v>
+      </c>
+      <c r="E24" s="8">
+        <v>74.260000000000005</v>
+      </c>
+      <c r="F24" s="8">
+        <v>78.680000000000007</v>
+      </c>
+      <c r="G24" s="8">
+        <v>83.09</v>
+      </c>
+      <c r="H24" s="8">
+        <v>95.76</v>
+      </c>
+      <c r="I24" s="8">
+        <v>108.42</v>
+      </c>
+      <c r="J24" s="8">
+        <v>121.09</v>
+      </c>
+      <c r="K24" s="8">
+        <v>129.62</v>
+      </c>
+      <c r="M24" s="9">
+        <v>20</v>
+      </c>
+      <c r="N24" s="8">
+        <v>138.15</v>
+      </c>
+      <c r="O24" s="8">
+        <v>187.66</v>
+      </c>
+      <c r="P24" s="8">
+        <v>237.17</v>
+      </c>
+      <c r="Q24" s="8">
+        <v>286.68</v>
+      </c>
+      <c r="R24" s="8">
+        <v>336.18</v>
+      </c>
+      <c r="S24" s="8">
+        <v>527.12</v>
+      </c>
+      <c r="T24" s="8">
+        <v>718.06</v>
+      </c>
+      <c r="U24" s="8">
+        <v>909</v>
+      </c>
+      <c r="V24" s="8">
+        <v>1099.94</v>
+      </c>
+      <c r="W24" s="8">
+        <v>1290.8800000000001</v>
+      </c>
+    </row>
+    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A25" s="5">
+        <v>21</v>
+      </c>
+      <c r="B25" s="8">
+        <v>44.67</v>
+      </c>
+      <c r="C25" s="8">
+        <v>57.75</v>
+      </c>
+      <c r="D25" s="8">
+        <v>70.84</v>
+      </c>
+      <c r="E25" s="8">
+        <v>74.930000000000007</v>
+      </c>
+      <c r="F25" s="8">
+        <v>79.02</v>
+      </c>
+      <c r="G25" s="8">
+        <v>83.11</v>
+      </c>
+      <c r="H25" s="8">
+        <v>96.02</v>
+      </c>
+      <c r="I25" s="8">
+        <v>108.92</v>
+      </c>
+      <c r="J25" s="8">
+        <v>121.82</v>
+      </c>
+      <c r="K25" s="8">
+        <v>129.99</v>
+      </c>
+      <c r="M25" s="9">
+        <v>21</v>
+      </c>
+      <c r="N25" s="8">
+        <v>138.15</v>
+      </c>
+      <c r="O25" s="8">
+        <v>187.66</v>
+      </c>
+      <c r="P25" s="8">
+        <v>237.17</v>
+      </c>
+      <c r="Q25" s="8">
+        <v>286.68</v>
+      </c>
+      <c r="R25" s="8">
+        <v>336.18</v>
+      </c>
+      <c r="S25" s="8">
+        <v>527.12</v>
+      </c>
+      <c r="T25" s="8">
+        <v>718.06</v>
+      </c>
+      <c r="U25" s="8">
+        <v>909</v>
+      </c>
+      <c r="V25" s="8">
+        <v>1099.94</v>
+      </c>
+      <c r="W25" s="8">
+        <v>1290.8800000000001</v>
+      </c>
+    </row>
+    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A26" s="5">
+        <v>22</v>
+      </c>
+      <c r="B26" s="8">
+        <v>46.3</v>
+      </c>
+      <c r="C26" s="8">
+        <v>59.06</v>
+      </c>
+      <c r="D26" s="8">
+        <v>71.83</v>
+      </c>
+      <c r="E26" s="8">
+        <v>75.599999999999994</v>
+      </c>
+      <c r="F26" s="8">
+        <v>79.37</v>
+      </c>
+      <c r="G26" s="8">
+        <v>83.13</v>
+      </c>
+      <c r="H26" s="8">
+        <v>96.27</v>
+      </c>
+      <c r="I26" s="8">
+        <v>109.41</v>
+      </c>
+      <c r="J26" s="8">
+        <v>122.55</v>
+      </c>
+      <c r="K26" s="8">
+        <v>130.35</v>
+      </c>
+      <c r="M26" s="9">
+        <v>22</v>
+      </c>
+      <c r="N26" s="8">
+        <v>138.15</v>
+      </c>
+      <c r="O26" s="8">
+        <v>187.66</v>
+      </c>
+      <c r="P26" s="8">
+        <v>237.17</v>
+      </c>
+      <c r="Q26" s="8">
+        <v>286.68</v>
+      </c>
+      <c r="R26" s="8">
+        <v>336.18</v>
+      </c>
+      <c r="S26" s="8">
+        <v>527.12</v>
+      </c>
+      <c r="T26" s="8">
+        <v>718.06</v>
+      </c>
+      <c r="U26" s="8">
+        <v>909</v>
+      </c>
+      <c r="V26" s="8">
+        <v>1099.94</v>
+      </c>
+      <c r="W26" s="8">
+        <v>1290.8800000000001</v>
+      </c>
+    </row>
+    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A27" s="5">
+        <v>23</v>
+      </c>
+      <c r="B27" s="8">
+        <v>47.92</v>
+      </c>
+      <c r="C27" s="8">
+        <v>60.37</v>
+      </c>
+      <c r="D27" s="8">
+        <v>72.83</v>
+      </c>
+      <c r="E27" s="8">
+        <v>76.27</v>
+      </c>
+      <c r="F27" s="8">
+        <v>79.709999999999994</v>
+      </c>
+      <c r="G27" s="8">
+        <v>83.15</v>
+      </c>
+      <c r="H27" s="8">
+        <v>96.53</v>
+      </c>
+      <c r="I27" s="8">
+        <v>109.91</v>
+      </c>
+      <c r="J27" s="8">
+        <v>123.29</v>
+      </c>
+      <c r="K27" s="8">
+        <v>130.72</v>
+      </c>
+      <c r="M27" s="9">
+        <v>23</v>
+      </c>
+      <c r="N27" s="8">
+        <v>138.15</v>
+      </c>
+      <c r="O27" s="8">
+        <v>187.66</v>
+      </c>
+      <c r="P27" s="8">
+        <v>237.17</v>
+      </c>
+      <c r="Q27" s="8">
+        <v>286.68</v>
+      </c>
+      <c r="R27" s="8">
+        <v>336.18</v>
+      </c>
+      <c r="S27" s="8">
+        <v>527.12</v>
+      </c>
+      <c r="T27" s="8">
+        <v>718.06</v>
+      </c>
+      <c r="U27" s="8">
+        <v>909</v>
+      </c>
+      <c r="V27" s="8">
+        <v>1099.94</v>
+      </c>
+      <c r="W27" s="8">
+        <v>1290.8800000000001</v>
+      </c>
+    </row>
+    <row r="28" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A28" s="5">
+        <v>24</v>
+      </c>
+      <c r="B28" s="8">
+        <v>49.55</v>
+      </c>
+      <c r="C28" s="8">
+        <v>61.69</v>
+      </c>
+      <c r="D28" s="8">
+        <v>73.819999999999993</v>
+      </c>
+      <c r="E28" s="8">
+        <v>76.94</v>
+      </c>
+      <c r="F28" s="8">
+        <v>80.06</v>
+      </c>
+      <c r="G28" s="8">
+        <v>83.17</v>
+      </c>
+      <c r="H28" s="8">
+        <v>96.79</v>
+      </c>
+      <c r="I28" s="8">
+        <v>110.4</v>
+      </c>
+      <c r="J28" s="8">
+        <v>124.02</v>
+      </c>
+      <c r="K28" s="8">
+        <v>131.09</v>
+      </c>
+      <c r="M28" s="9">
+        <v>24</v>
+      </c>
+      <c r="N28" s="8">
+        <v>138.15</v>
+      </c>
+      <c r="O28" s="8">
+        <v>187.66</v>
+      </c>
+      <c r="P28" s="8">
+        <v>237.17</v>
+      </c>
+      <c r="Q28" s="8">
+        <v>286.68</v>
+      </c>
+      <c r="R28" s="8">
+        <v>336.18</v>
+      </c>
+      <c r="S28" s="8">
+        <v>527.12</v>
+      </c>
+      <c r="T28" s="8">
+        <v>718.06</v>
+      </c>
+      <c r="U28" s="8">
+        <v>909</v>
+      </c>
+      <c r="V28" s="8">
+        <v>1099.94</v>
+      </c>
+      <c r="W28" s="8">
+        <v>1290.8800000000001</v>
+      </c>
+    </row>
+    <row r="29" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A29" s="5">
+        <v>25</v>
+      </c>
+      <c r="B29" s="8">
+        <v>51.17</v>
+      </c>
+      <c r="C29" s="8">
+        <v>63</v>
+      </c>
+      <c r="D29" s="8">
+        <v>74.819999999999993</v>
+      </c>
+      <c r="E29" s="8">
+        <v>77.61</v>
+      </c>
+      <c r="F29" s="8">
+        <v>80.400000000000006</v>
+      </c>
+      <c r="G29" s="8">
+        <v>83.19</v>
+      </c>
+      <c r="H29" s="8">
+        <v>97.05</v>
+      </c>
+      <c r="I29" s="8">
+        <v>110.9</v>
+      </c>
+      <c r="J29" s="8">
+        <v>124.75</v>
+      </c>
+      <c r="K29" s="8">
+        <v>131.44999999999999</v>
+      </c>
+      <c r="M29" s="9">
+        <v>25</v>
+      </c>
+      <c r="N29" s="8">
+        <v>138.15</v>
+      </c>
+      <c r="O29" s="8">
+        <v>187.66</v>
+      </c>
+      <c r="P29" s="8">
+        <v>237.17</v>
+      </c>
+      <c r="Q29" s="8">
+        <v>286.68</v>
+      </c>
+      <c r="R29" s="8">
+        <v>336.18</v>
+      </c>
+      <c r="S29" s="8">
+        <v>527.12</v>
+      </c>
+      <c r="T29" s="8">
+        <v>718.06</v>
+      </c>
+      <c r="U29" s="8">
+        <v>909</v>
+      </c>
+      <c r="V29" s="8">
+        <v>1099.94</v>
+      </c>
+      <c r="W29" s="8">
+        <v>1290.8800000000001</v>
+      </c>
+    </row>
+    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A30" s="5">
+        <v>26</v>
+      </c>
+      <c r="B30" s="8">
+        <v>52.8</v>
+      </c>
+      <c r="C30" s="8">
+        <v>64.31</v>
+      </c>
+      <c r="D30" s="8">
+        <v>75.81</v>
+      </c>
+      <c r="E30" s="8">
+        <v>78.28</v>
+      </c>
+      <c r="F30" s="8">
+        <v>80.75</v>
+      </c>
+      <c r="G30" s="8">
+        <v>83.21</v>
+      </c>
+      <c r="H30" s="8">
+        <v>97.3</v>
+      </c>
+      <c r="I30" s="8">
+        <v>111.39</v>
+      </c>
+      <c r="J30" s="8">
+        <v>125.48</v>
+      </c>
+      <c r="K30" s="8">
+        <v>131.82</v>
+      </c>
+      <c r="M30" s="9">
+        <v>26</v>
+      </c>
+      <c r="N30" s="8">
+        <v>138.15</v>
+      </c>
+      <c r="O30" s="8">
+        <v>187.66</v>
+      </c>
+      <c r="P30" s="8">
+        <v>237.17</v>
+      </c>
+      <c r="Q30" s="8">
+        <v>286.68</v>
+      </c>
+      <c r="R30" s="8">
+        <v>336.18</v>
+      </c>
+      <c r="S30" s="8">
+        <v>527.12</v>
+      </c>
+      <c r="T30" s="8">
+        <v>718.06</v>
+      </c>
+      <c r="U30" s="8">
+        <v>909</v>
+      </c>
+      <c r="V30" s="8">
+        <v>1099.94</v>
+      </c>
+      <c r="W30" s="8">
+        <v>1290.8800000000001</v>
+      </c>
+    </row>
+    <row r="31" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A31" s="5">
+        <v>27</v>
+      </c>
+      <c r="B31" s="8">
+        <v>54.43</v>
+      </c>
+      <c r="C31" s="8">
+        <v>65.62</v>
+      </c>
+      <c r="D31" s="8">
+        <v>76.81</v>
+      </c>
+      <c r="E31" s="8">
+        <v>78.95</v>
+      </c>
+      <c r="F31" s="8">
+        <v>81.09</v>
+      </c>
+      <c r="G31" s="8">
+        <v>83.23</v>
+      </c>
+      <c r="H31" s="8">
+        <v>97.56</v>
+      </c>
+      <c r="I31" s="8">
+        <v>111.89</v>
+      </c>
+      <c r="J31" s="8">
+        <v>126.22</v>
+      </c>
+      <c r="K31" s="8">
+        <v>132.18</v>
+      </c>
+      <c r="M31" s="9">
+        <v>27</v>
+      </c>
+      <c r="N31" s="8">
+        <v>138.15</v>
+      </c>
+      <c r="O31" s="8">
+        <v>187.66</v>
+      </c>
+      <c r="P31" s="8">
+        <v>237.17</v>
+      </c>
+      <c r="Q31" s="8">
+        <v>286.68</v>
+      </c>
+      <c r="R31" s="8">
+        <v>336.18</v>
+      </c>
+      <c r="S31" s="8">
+        <v>527.12</v>
+      </c>
+      <c r="T31" s="8">
+        <v>718.06</v>
+      </c>
+      <c r="U31" s="8">
+        <v>909</v>
+      </c>
+      <c r="V31" s="8">
+        <v>1099.94</v>
+      </c>
+      <c r="W31" s="8">
+        <v>1290.8800000000001</v>
+      </c>
+    </row>
+    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A32" s="5">
+        <v>28</v>
+      </c>
+      <c r="B32" s="8">
+        <v>56.05</v>
+      </c>
+      <c r="C32" s="8">
+        <v>66.930000000000007</v>
+      </c>
+      <c r="D32" s="8">
+        <v>77.8</v>
+      </c>
+      <c r="E32" s="8">
+        <v>79.62</v>
+      </c>
+      <c r="F32" s="8">
+        <v>81.44</v>
+      </c>
+      <c r="G32" s="8">
+        <v>83.25</v>
+      </c>
+      <c r="H32" s="8">
+        <v>97.82</v>
+      </c>
+      <c r="I32" s="8">
+        <v>112.38</v>
+      </c>
+      <c r="J32" s="8">
+        <v>126.95</v>
+      </c>
+      <c r="K32" s="8">
+        <v>132.55000000000001</v>
+      </c>
+      <c r="M32" s="9">
+        <v>28</v>
+      </c>
+      <c r="N32" s="8">
+        <v>138.15</v>
+      </c>
+      <c r="O32" s="8">
+        <v>187.66</v>
+      </c>
+      <c r="P32" s="8">
+        <v>237.17</v>
+      </c>
+      <c r="Q32" s="8">
+        <v>286.68</v>
+      </c>
+      <c r="R32" s="8">
+        <v>336.18</v>
+      </c>
+      <c r="S32" s="8">
+        <v>527.12</v>
+      </c>
+      <c r="T32" s="8">
+        <v>718.06</v>
+      </c>
+      <c r="U32" s="8">
+        <v>909</v>
+      </c>
+      <c r="V32" s="8">
+        <v>1099.94</v>
+      </c>
+      <c r="W32" s="8">
+        <v>1290.8800000000001</v>
+      </c>
+    </row>
+    <row r="33" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A33" s="5">
+        <v>29</v>
+      </c>
+      <c r="B33" s="8">
+        <v>57.68</v>
+      </c>
+      <c r="C33" s="8">
+        <v>68.239999999999995</v>
+      </c>
+      <c r="D33" s="8">
+        <v>78.8</v>
+      </c>
+      <c r="E33" s="8">
+        <v>80.290000000000006</v>
+      </c>
+      <c r="F33" s="8">
+        <v>81.78</v>
+      </c>
+      <c r="G33" s="8">
+        <v>83.27</v>
+      </c>
+      <c r="H33" s="8">
+        <v>98.08</v>
+      </c>
+      <c r="I33" s="8">
+        <v>112.88</v>
+      </c>
+      <c r="J33" s="8">
+        <v>127.68</v>
+      </c>
+      <c r="K33" s="8">
+        <v>132.91999999999999</v>
+      </c>
+      <c r="M33" s="9">
+        <v>29</v>
+      </c>
+      <c r="N33" s="8">
+        <v>138.15</v>
+      </c>
+      <c r="O33" s="8">
+        <v>187.66</v>
+      </c>
+      <c r="P33" s="8">
+        <v>237.17</v>
+      </c>
+      <c r="Q33" s="8">
+        <v>286.68</v>
+      </c>
+      <c r="R33" s="8">
+        <v>336.18</v>
+      </c>
+      <c r="S33" s="8">
+        <v>527.12</v>
+      </c>
+      <c r="T33" s="8">
+        <v>718.06</v>
+      </c>
+      <c r="U33" s="8">
+        <v>909</v>
+      </c>
+      <c r="V33" s="8">
+        <v>1099.94</v>
+      </c>
+      <c r="W33" s="8">
+        <v>1290.8800000000001</v>
+      </c>
+    </row>
+    <row r="34" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A34" s="5">
+        <v>30</v>
+      </c>
+      <c r="B34" s="8">
+        <v>59.3</v>
+      </c>
+      <c r="C34" s="8">
+        <v>69.55</v>
+      </c>
+      <c r="D34" s="8">
+        <v>79.790000000000006</v>
+      </c>
+      <c r="E34" s="8">
+        <v>80.959999999999994</v>
+      </c>
+      <c r="F34" s="8">
+        <v>82.13</v>
+      </c>
+      <c r="G34" s="8">
+        <v>83.29</v>
+      </c>
+      <c r="H34" s="8">
+        <v>98.33</v>
+      </c>
+      <c r="I34" s="8">
+        <v>113.37</v>
+      </c>
+      <c r="J34" s="8">
+        <v>128.41</v>
+      </c>
+      <c r="K34" s="8">
+        <v>133.28</v>
+      </c>
+      <c r="M34" s="9">
+        <v>30</v>
+      </c>
+      <c r="N34" s="8">
+        <v>138.15</v>
+      </c>
+      <c r="O34" s="8">
+        <v>187.66</v>
+      </c>
+      <c r="P34" s="8">
+        <v>237.17</v>
+      </c>
+      <c r="Q34" s="8">
+        <v>286.68</v>
+      </c>
+      <c r="R34" s="8">
+        <v>336.18</v>
+      </c>
+      <c r="S34" s="8">
+        <v>527.12</v>
+      </c>
+      <c r="T34" s="8">
+        <v>718.06</v>
+      </c>
+      <c r="U34" s="8">
+        <v>909</v>
+      </c>
+      <c r="V34" s="8">
+        <v>1099.94</v>
+      </c>
+      <c r="W34" s="8">
+        <v>1290.8800000000001</v>
+      </c>
+    </row>
+    <row r="35" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A35" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B35" s="8">
+        <v>35.809999999999988</v>
+      </c>
+      <c r="C35" s="8">
+        <v>48.883666666666663</v>
+      </c>
+      <c r="D35" s="8">
+        <v>61.957666666666647</v>
+      </c>
+      <c r="E35" s="8">
+        <v>67.278999999999996</v>
+      </c>
+      <c r="F35" s="8">
+        <v>72.598333333333343</v>
+      </c>
+      <c r="G35" s="8">
+        <v>77.917999999999992</v>
+      </c>
+      <c r="H35" s="8">
+        <v>89.66166666666669</v>
+      </c>
+      <c r="I35" s="8">
+        <v>101.40400000000001</v>
+      </c>
+      <c r="J35" s="8">
+        <v>113.14733333333332</v>
+      </c>
+      <c r="K35" s="8">
+        <v>125.64999999999999</v>
+      </c>
+      <c r="M35" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="N35" s="10">
+        <v>138.15000000000006</v>
+      </c>
+      <c r="O35" s="10">
+        <v>187.65999999999991</v>
+      </c>
+      <c r="P35" s="10">
+        <v>237.17000000000004</v>
+      </c>
+      <c r="Q35" s="10">
+        <v>286.68000000000012</v>
+      </c>
+      <c r="R35" s="10">
+        <v>336.18000000000012</v>
+      </c>
+      <c r="S35" s="10">
+        <v>527.12000000000035</v>
+      </c>
+      <c r="T35" s="10">
+        <v>718.06000000000006</v>
+      </c>
+      <c r="U35" s="10">
+        <v>909</v>
+      </c>
+      <c r="V35" s="10">
+        <v>1099.9399999999996</v>
+      </c>
+      <c r="W35" s="10">
+        <v>1290.8800000000003</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B2:K2"/>
+    <mergeCell ref="M1:W1"/>
+    <mergeCell ref="N2:W2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{612EBB24-0E24-4D37-B6A7-8B4DA2BD1A51}">
   <dimension ref="A1:W35"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.08984375" customWidth="1"/>
-    <col min="13" max="23" width="11.08984375" customWidth="1"/>
+    <col min="1" max="1" width="11.140625" customWidth="1"/>
+    <col min="13" max="23" width="11.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>30</v>
       </c>
@@ -762,7 +3092,7 @@
       <c r="V1" s="14"/>
       <c r="W1" s="15"/>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -794,7 +3124,7 @@
       <c r="V2" s="12"/>
       <c r="W2" s="12"/>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>2</v>
       </c>
@@ -862,7 +3192,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>3</v>
       </c>
@@ -930,7 +3260,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
         <v>1</v>
       </c>
@@ -998,7 +3328,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
         <v>2</v>
       </c>
@@ -1066,7 +3396,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
         <v>3</v>
       </c>
@@ -1134,7 +3464,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
         <v>4</v>
       </c>
@@ -1202,7 +3532,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
         <v>5</v>
       </c>
@@ -1270,7 +3600,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A10" s="5">
         <v>6</v>
       </c>
@@ -1338,7 +3668,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A11" s="5">
         <v>7</v>
       </c>
@@ -1406,7 +3736,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A12" s="5">
         <v>8</v>
       </c>
@@ -1474,7 +3804,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A13" s="5">
         <v>9</v>
       </c>
@@ -1542,7 +3872,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A14" s="5">
         <v>10</v>
       </c>
@@ -1610,7 +3940,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A15" s="5">
         <v>11</v>
       </c>
@@ -1678,7 +4008,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A16" s="5">
         <v>12</v>
       </c>
@@ -1746,7 +4076,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A17" s="5">
         <v>13</v>
       </c>
@@ -1814,7 +4144,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A18" s="5">
         <v>14</v>
       </c>
@@ -1882,7 +4212,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A19" s="5">
         <v>15</v>
       </c>
@@ -1950,7 +4280,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A20" s="5">
         <v>16</v>
       </c>
@@ -2018,7 +4348,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A21" s="5">
         <v>17</v>
       </c>
@@ -2086,7 +4416,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A22" s="5">
         <v>18</v>
       </c>
@@ -2154,7 +4484,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A23" s="5">
         <v>19</v>
       </c>
@@ -2222,7 +4552,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A24" s="5">
         <v>20</v>
       </c>
@@ -2290,7 +4620,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A25" s="5">
         <v>21</v>
       </c>
@@ -2358,7 +4688,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A26" s="5">
         <v>22</v>
       </c>
@@ -2426,7 +4756,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A27" s="5">
         <v>23</v>
       </c>
@@ -2494,7 +4824,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A28" s="5">
         <v>24</v>
       </c>
@@ -2562,7 +4892,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A29" s="5">
         <v>25</v>
       </c>
@@ -2630,7 +4960,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A30" s="5">
         <v>26</v>
       </c>
@@ -2698,7 +5028,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A31" s="5">
         <v>27</v>
       </c>
@@ -2766,7 +5096,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A32" s="5">
         <v>28</v>
       </c>
@@ -2834,7 +5164,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="33" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A33" s="5">
         <v>29</v>
       </c>
@@ -2902,7 +5232,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="34" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A34" s="5">
         <v>30</v>
       </c>
@@ -2970,7 +5300,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="35" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
         <v>14</v>
       </c>
@@ -3048,16 +5378,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A2E7E46-B70B-4DB0-97AE-2138287FA00A}">
   <dimension ref="A1:W35"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.08984375" customWidth="1"/>
-    <col min="13" max="23" width="11.08984375" customWidth="1"/>
+    <col min="1" max="1" width="11.140625" customWidth="1"/>
+    <col min="13" max="23" width="11.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>28</v>
       </c>
@@ -3085,7 +5415,7 @@
       <c r="V1" s="14"/>
       <c r="W1" s="15"/>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -3117,7 +5447,7 @@
       <c r="V2" s="12"/>
       <c r="W2" s="12"/>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>2</v>
       </c>
@@ -3185,7 +5515,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>3</v>
       </c>
@@ -3253,7 +5583,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
         <v>1</v>
       </c>
@@ -3321,7 +5651,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
         <v>2</v>
       </c>
@@ -3389,7 +5719,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
         <v>3</v>
       </c>
@@ -3457,7 +5787,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
         <v>4</v>
       </c>
@@ -3525,7 +5855,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
         <v>5</v>
       </c>
@@ -3593,7 +5923,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A10" s="5">
         <v>6</v>
       </c>
@@ -3661,7 +5991,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A11" s="5">
         <v>7</v>
       </c>
@@ -3729,7 +6059,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A12" s="5">
         <v>8</v>
       </c>
@@ -3797,7 +6127,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A13" s="5">
         <v>9</v>
       </c>
@@ -3865,7 +6195,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A14" s="5">
         <v>10</v>
       </c>
@@ -3933,7 +6263,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A15" s="5">
         <v>11</v>
       </c>
@@ -4001,7 +6331,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A16" s="5">
         <v>12</v>
       </c>
@@ -4069,7 +6399,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A17" s="5">
         <v>13</v>
       </c>
@@ -4137,7 +6467,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A18" s="5">
         <v>14</v>
       </c>
@@ -4205,7 +6535,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A19" s="5">
         <v>15</v>
       </c>
@@ -4273,7 +6603,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A20" s="5">
         <v>16</v>
       </c>
@@ -4341,7 +6671,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A21" s="5">
         <v>17</v>
       </c>
@@ -4409,7 +6739,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A22" s="5">
         <v>18</v>
       </c>
@@ -4477,7 +6807,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A23" s="5">
         <v>19</v>
       </c>
@@ -4545,7 +6875,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A24" s="5">
         <v>20</v>
       </c>
@@ -4613,7 +6943,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A25" s="5">
         <v>21</v>
       </c>
@@ -4681,7 +7011,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A26" s="5">
         <v>22</v>
       </c>
@@ -4749,7 +7079,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A27" s="5">
         <v>23</v>
       </c>
@@ -4817,7 +7147,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A28" s="5">
         <v>24</v>
       </c>
@@ -4885,7 +7215,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A29" s="5">
         <v>25</v>
       </c>
@@ -4953,7 +7283,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A30" s="5">
         <v>26</v>
       </c>
@@ -5021,7 +7351,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A31" s="5">
         <v>27</v>
       </c>
@@ -5089,7 +7419,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A32" s="5">
         <v>28</v>
       </c>
@@ -5157,7 +7487,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="33" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A33" s="5">
         <v>29</v>
       </c>
@@ -5225,7 +7555,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="34" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A34" s="5">
         <v>30</v>
       </c>
@@ -5293,7 +7623,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="35" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
         <v>14</v>
       </c>
@@ -5371,16 +7701,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D32525DC-1FAE-40FA-B3A1-6E6C0B62B72E}">
   <dimension ref="A1:W35"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.1796875" customWidth="1"/>
-    <col min="13" max="23" width="11.1796875" customWidth="1"/>
+    <col min="1" max="1" width="11.140625" customWidth="1"/>
+    <col min="13" max="23" width="11.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>26</v>
       </c>
@@ -5408,7 +7738,7 @@
       <c r="V1" s="14"/>
       <c r="W1" s="15"/>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -5440,7 +7770,7 @@
       <c r="V2" s="12"/>
       <c r="W2" s="12"/>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>2</v>
       </c>
@@ -5508,7 +7838,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>3</v>
       </c>
@@ -5576,7 +7906,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
         <v>1</v>
       </c>
@@ -5644,7 +7974,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
         <v>2</v>
       </c>
@@ -5712,7 +8042,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
         <v>3</v>
       </c>
@@ -5780,7 +8110,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
         <v>4</v>
       </c>
@@ -5848,7 +8178,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
         <v>5</v>
       </c>
@@ -5916,7 +8246,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A10" s="5">
         <v>6</v>
       </c>
@@ -5984,7 +8314,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A11" s="5">
         <v>7</v>
       </c>
@@ -6052,7 +8382,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A12" s="5">
         <v>8</v>
       </c>
@@ -6120,7 +8450,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A13" s="5">
         <v>9</v>
       </c>
@@ -6188,7 +8518,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A14" s="5">
         <v>10</v>
       </c>
@@ -6256,7 +8586,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A15" s="5">
         <v>11</v>
       </c>
@@ -6324,7 +8654,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A16" s="5">
         <v>12</v>
       </c>
@@ -6392,7 +8722,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A17" s="5">
         <v>13</v>
       </c>
@@ -6460,7 +8790,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A18" s="5">
         <v>14</v>
       </c>
@@ -6528,7 +8858,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A19" s="5">
         <v>15</v>
       </c>
@@ -6596,7 +8926,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A20" s="5">
         <v>16</v>
       </c>
@@ -6664,7 +8994,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A21" s="5">
         <v>17</v>
       </c>
@@ -6732,7 +9062,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A22" s="5">
         <v>18</v>
       </c>
@@ -6800,7 +9130,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A23" s="5">
         <v>19</v>
       </c>
@@ -6868,7 +9198,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A24" s="5">
         <v>20</v>
       </c>
@@ -6936,7 +9266,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A25" s="5">
         <v>21</v>
       </c>
@@ -7004,7 +9334,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A26" s="5">
         <v>22</v>
       </c>
@@ -7072,7 +9402,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A27" s="5">
         <v>23</v>
       </c>
@@ -7140,7 +9470,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A28" s="5">
         <v>24</v>
       </c>
@@ -7208,7 +9538,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A29" s="5">
         <v>25</v>
       </c>
@@ -7276,7 +9606,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A30" s="5">
         <v>26</v>
       </c>
@@ -7344,7 +9674,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A31" s="5">
         <v>27</v>
       </c>
@@ -7412,7 +9742,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A32" s="5">
         <v>28</v>
       </c>
@@ -7480,7 +9810,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="33" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A33" s="5">
         <v>29</v>
       </c>
@@ -7548,7 +9878,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="34" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A34" s="5">
         <v>30</v>
       </c>
@@ -7616,7 +9946,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="35" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
         <v>14</v>
       </c>
@@ -7694,15 +10024,15 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <sheetPr codeName="Sheet9">
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
   <dimension ref="H31"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="31" spans="8:8" x14ac:dyDescent="0.35">
+    <row r="31" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H31" s="1"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 Update NAIC content history - 2026-06-02
</commit_message>
<xml_diff>
--- a/docs/content_history/pbr-2026-vm20-table-f-g-current-spreads.xlsx
+++ b/docs/content_history/pbr-2026-vm20-table-f-g-current-spreads.xlsx
@@ -1,23 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\PBR\VM20_VM22_ProductSupport\PBR Production Web Data\Current Year\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF0A3062-E358-4E67-AC54-79F2A4C44FD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B217903-9369-45E9-9ACD-B41ABCB3658B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="795" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="795" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="April_2026" sheetId="27" r:id="rId1"/>
-    <sheet name="March_2026" sheetId="26" r:id="rId2"/>
-    <sheet name="February_2026" sheetId="25" r:id="rId3"/>
-    <sheet name="January_2026" sheetId="24" r:id="rId4"/>
-    <sheet name="LEGAL DISCLAIMER" sheetId="11" r:id="rId5"/>
+    <sheet name="May_2026" sheetId="28" r:id="rId1"/>
+    <sheet name="April_2026" sheetId="27" r:id="rId2"/>
+    <sheet name="March_2026" sheetId="26" r:id="rId3"/>
+    <sheet name="February_2026" sheetId="25" r:id="rId4"/>
+    <sheet name="January_2026" sheetId="24" r:id="rId5"/>
+    <sheet name="LEGAL DISCLAIMER" sheetId="11" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="36">
   <si>
     <t>WAL</t>
   </si>
@@ -136,6 +137,12 @@
   </si>
   <si>
     <t>Table G. (04/30/2026) Below Investment Grade Current Benchmark Spreads (in bps)</t>
+  </si>
+  <si>
+    <t>Table F (05/29/2026)  Investment Grade Current Benchmark Spreads (in bps)</t>
+  </si>
+  <si>
+    <t>Table G. (05/29/2026) Below Investment Grade Current Benchmark Spreads (in bps)</t>
   </si>
 </sst>
 </file>
@@ -412,7 +419,7 @@
                   <a14:compatExt spid="_x0000_s4104"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000008100000}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0400-000008100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -733,6 +740,2329 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89E0380B-3232-4FC8-8E48-B6A283DD6300}">
+  <dimension ref="A1:W35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.140625" customWidth="1"/>
+    <col min="13" max="23" width="11.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="M1" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="N1" s="14"/>
+      <c r="O1" s="14"/>
+      <c r="P1" s="14"/>
+      <c r="Q1" s="14"/>
+      <c r="R1" s="14"/>
+      <c r="S1" s="14"/>
+      <c r="T1" s="14"/>
+      <c r="U1" s="14"/>
+      <c r="V1" s="14"/>
+      <c r="W1" s="15"/>
+    </row>
+    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12"/>
+      <c r="K2" s="12"/>
+      <c r="M2" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="N2" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="O2" s="12"/>
+      <c r="P2" s="12"/>
+      <c r="Q2" s="12"/>
+      <c r="R2" s="12"/>
+      <c r="S2" s="12"/>
+      <c r="T2" s="12"/>
+      <c r="U2" s="12"/>
+      <c r="V2" s="12"/>
+      <c r="W2" s="12"/>
+    </row>
+    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="5">
+        <v>1</v>
+      </c>
+      <c r="C3" s="5">
+        <v>2</v>
+      </c>
+      <c r="D3" s="5">
+        <v>3</v>
+      </c>
+      <c r="E3" s="5">
+        <v>4</v>
+      </c>
+      <c r="F3" s="5">
+        <v>5</v>
+      </c>
+      <c r="G3" s="5">
+        <v>6</v>
+      </c>
+      <c r="H3" s="5">
+        <v>7</v>
+      </c>
+      <c r="I3" s="5">
+        <v>8</v>
+      </c>
+      <c r="J3" s="5">
+        <v>9</v>
+      </c>
+      <c r="K3" s="5">
+        <v>10</v>
+      </c>
+      <c r="M3" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="N3" s="5">
+        <v>11</v>
+      </c>
+      <c r="O3" s="5">
+        <v>12</v>
+      </c>
+      <c r="P3" s="5">
+        <v>13</v>
+      </c>
+      <c r="Q3" s="5">
+        <v>14</v>
+      </c>
+      <c r="R3" s="5">
+        <v>15</v>
+      </c>
+      <c r="S3" s="5">
+        <v>16</v>
+      </c>
+      <c r="T3" s="5">
+        <v>17</v>
+      </c>
+      <c r="U3" s="5">
+        <v>18</v>
+      </c>
+      <c r="V3" s="5">
+        <v>19</v>
+      </c>
+      <c r="W3" s="5">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="M4" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="P4" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q4" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="R4" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="S4" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="T4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="U4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="V4" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="W4" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A5" s="5">
+        <v>1</v>
+      </c>
+      <c r="B5" s="8">
+        <v>13.93</v>
+      </c>
+      <c r="C5" s="8">
+        <v>17.79</v>
+      </c>
+      <c r="D5" s="8">
+        <v>21.64</v>
+      </c>
+      <c r="E5" s="8">
+        <v>27.03</v>
+      </c>
+      <c r="F5" s="8">
+        <v>32.43</v>
+      </c>
+      <c r="G5" s="8">
+        <v>37.82</v>
+      </c>
+      <c r="H5" s="8">
+        <v>45</v>
+      </c>
+      <c r="I5" s="8">
+        <v>52.19</v>
+      </c>
+      <c r="J5" s="8">
+        <v>59.38</v>
+      </c>
+      <c r="K5" s="8">
+        <v>92.44</v>
+      </c>
+      <c r="M5" s="9">
+        <v>1</v>
+      </c>
+      <c r="N5" s="8">
+        <v>125.51</v>
+      </c>
+      <c r="O5" s="8">
+        <v>174.86</v>
+      </c>
+      <c r="P5" s="8">
+        <v>224.21</v>
+      </c>
+      <c r="Q5" s="8">
+        <v>273.56</v>
+      </c>
+      <c r="R5" s="8">
+        <v>322.91000000000003</v>
+      </c>
+      <c r="S5" s="8">
+        <v>527.94000000000005</v>
+      </c>
+      <c r="T5" s="8">
+        <v>732.97</v>
+      </c>
+      <c r="U5" s="8">
+        <v>938</v>
+      </c>
+      <c r="V5" s="8">
+        <v>1143.03</v>
+      </c>
+      <c r="W5" s="8">
+        <v>1348.06</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A6" s="5">
+        <v>2</v>
+      </c>
+      <c r="B6" s="8">
+        <v>12.94</v>
+      </c>
+      <c r="C6" s="8">
+        <v>19.41</v>
+      </c>
+      <c r="D6" s="8">
+        <v>25.88</v>
+      </c>
+      <c r="E6" s="8">
+        <v>31.85</v>
+      </c>
+      <c r="F6" s="8">
+        <v>37.81</v>
+      </c>
+      <c r="G6" s="8">
+        <v>43.78</v>
+      </c>
+      <c r="H6" s="8">
+        <v>51.61</v>
+      </c>
+      <c r="I6" s="8">
+        <v>59.44</v>
+      </c>
+      <c r="J6" s="8">
+        <v>67.28</v>
+      </c>
+      <c r="K6" s="8">
+        <v>96.39</v>
+      </c>
+      <c r="M6" s="9">
+        <v>2</v>
+      </c>
+      <c r="N6" s="8">
+        <v>125.51</v>
+      </c>
+      <c r="O6" s="8">
+        <v>174.86</v>
+      </c>
+      <c r="P6" s="8">
+        <v>224.21</v>
+      </c>
+      <c r="Q6" s="8">
+        <v>273.56</v>
+      </c>
+      <c r="R6" s="8">
+        <v>322.91000000000003</v>
+      </c>
+      <c r="S6" s="8">
+        <v>527.94000000000005</v>
+      </c>
+      <c r="T6" s="8">
+        <v>732.97</v>
+      </c>
+      <c r="U6" s="8">
+        <v>938</v>
+      </c>
+      <c r="V6" s="8">
+        <v>1143.03</v>
+      </c>
+      <c r="W6" s="8">
+        <v>1348.06</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A7" s="5">
+        <v>3</v>
+      </c>
+      <c r="B7" s="8">
+        <v>11.96</v>
+      </c>
+      <c r="C7" s="8">
+        <v>21.04</v>
+      </c>
+      <c r="D7" s="8">
+        <v>30.12</v>
+      </c>
+      <c r="E7" s="8">
+        <v>36.659999999999997</v>
+      </c>
+      <c r="F7" s="8">
+        <v>43.2</v>
+      </c>
+      <c r="G7" s="8">
+        <v>49.74</v>
+      </c>
+      <c r="H7" s="8">
+        <v>58.22</v>
+      </c>
+      <c r="I7" s="8">
+        <v>66.7</v>
+      </c>
+      <c r="J7" s="8">
+        <v>75.180000000000007</v>
+      </c>
+      <c r="K7" s="8">
+        <v>100.34</v>
+      </c>
+      <c r="M7" s="9">
+        <v>3</v>
+      </c>
+      <c r="N7" s="8">
+        <v>125.51</v>
+      </c>
+      <c r="O7" s="8">
+        <v>174.86</v>
+      </c>
+      <c r="P7" s="8">
+        <v>224.21</v>
+      </c>
+      <c r="Q7" s="8">
+        <v>273.56</v>
+      </c>
+      <c r="R7" s="8">
+        <v>322.91000000000003</v>
+      </c>
+      <c r="S7" s="8">
+        <v>527.94000000000005</v>
+      </c>
+      <c r="T7" s="8">
+        <v>732.97</v>
+      </c>
+      <c r="U7" s="8">
+        <v>938</v>
+      </c>
+      <c r="V7" s="8">
+        <v>1143.03</v>
+      </c>
+      <c r="W7" s="8">
+        <v>1348.06</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A8" s="5">
+        <v>4</v>
+      </c>
+      <c r="B8" s="8">
+        <v>10.97</v>
+      </c>
+      <c r="C8" s="8">
+        <v>22.67</v>
+      </c>
+      <c r="D8" s="8">
+        <v>34.36</v>
+      </c>
+      <c r="E8" s="8">
+        <v>41.47</v>
+      </c>
+      <c r="F8" s="8">
+        <v>48.59</v>
+      </c>
+      <c r="G8" s="8">
+        <v>55.7</v>
+      </c>
+      <c r="H8" s="8">
+        <v>64.819999999999993</v>
+      </c>
+      <c r="I8" s="8">
+        <v>73.95</v>
+      </c>
+      <c r="J8" s="8">
+        <v>83.08</v>
+      </c>
+      <c r="K8" s="8">
+        <v>104.29</v>
+      </c>
+      <c r="M8" s="9">
+        <v>4</v>
+      </c>
+      <c r="N8" s="8">
+        <v>125.51</v>
+      </c>
+      <c r="O8" s="8">
+        <v>174.86</v>
+      </c>
+      <c r="P8" s="8">
+        <v>224.21</v>
+      </c>
+      <c r="Q8" s="8">
+        <v>273.56</v>
+      </c>
+      <c r="R8" s="8">
+        <v>322.91000000000003</v>
+      </c>
+      <c r="S8" s="8">
+        <v>527.94000000000005</v>
+      </c>
+      <c r="T8" s="8">
+        <v>732.97</v>
+      </c>
+      <c r="U8" s="8">
+        <v>938</v>
+      </c>
+      <c r="V8" s="8">
+        <v>1143.03</v>
+      </c>
+      <c r="W8" s="8">
+        <v>1348.06</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A9" s="5">
+        <v>5</v>
+      </c>
+      <c r="B9" s="8">
+        <v>12.13</v>
+      </c>
+      <c r="C9" s="8">
+        <v>24.72</v>
+      </c>
+      <c r="D9" s="8">
+        <v>37.31</v>
+      </c>
+      <c r="E9" s="8">
+        <v>44.88</v>
+      </c>
+      <c r="F9" s="8">
+        <v>52.45</v>
+      </c>
+      <c r="G9" s="8">
+        <v>60.03</v>
+      </c>
+      <c r="H9" s="8">
+        <v>69.040000000000006</v>
+      </c>
+      <c r="I9" s="8">
+        <v>78.06</v>
+      </c>
+      <c r="J9" s="8">
+        <v>87.07</v>
+      </c>
+      <c r="K9" s="8">
+        <v>106.29</v>
+      </c>
+      <c r="M9" s="9">
+        <v>5</v>
+      </c>
+      <c r="N9" s="8">
+        <v>125.51</v>
+      </c>
+      <c r="O9" s="8">
+        <v>174.86</v>
+      </c>
+      <c r="P9" s="8">
+        <v>224.21</v>
+      </c>
+      <c r="Q9" s="8">
+        <v>273.56</v>
+      </c>
+      <c r="R9" s="8">
+        <v>322.91000000000003</v>
+      </c>
+      <c r="S9" s="8">
+        <v>527.94000000000005</v>
+      </c>
+      <c r="T9" s="8">
+        <v>732.97</v>
+      </c>
+      <c r="U9" s="8">
+        <v>938</v>
+      </c>
+      <c r="V9" s="8">
+        <v>1143.03</v>
+      </c>
+      <c r="W9" s="8">
+        <v>1348.06</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A10" s="5">
+        <v>6</v>
+      </c>
+      <c r="B10" s="8">
+        <v>13.29</v>
+      </c>
+      <c r="C10" s="8">
+        <v>26.77</v>
+      </c>
+      <c r="D10" s="8">
+        <v>40.25</v>
+      </c>
+      <c r="E10" s="8">
+        <v>48.29</v>
+      </c>
+      <c r="F10" s="8">
+        <v>56.32</v>
+      </c>
+      <c r="G10" s="8">
+        <v>64.36</v>
+      </c>
+      <c r="H10" s="8">
+        <v>73.260000000000005</v>
+      </c>
+      <c r="I10" s="8">
+        <v>82.16</v>
+      </c>
+      <c r="J10" s="8">
+        <v>91.07</v>
+      </c>
+      <c r="K10" s="8">
+        <v>108.29</v>
+      </c>
+      <c r="M10" s="9">
+        <v>6</v>
+      </c>
+      <c r="N10" s="8">
+        <v>125.51</v>
+      </c>
+      <c r="O10" s="8">
+        <v>174.86</v>
+      </c>
+      <c r="P10" s="8">
+        <v>224.21</v>
+      </c>
+      <c r="Q10" s="8">
+        <v>273.56</v>
+      </c>
+      <c r="R10" s="8">
+        <v>322.91000000000003</v>
+      </c>
+      <c r="S10" s="8">
+        <v>527.94000000000005</v>
+      </c>
+      <c r="T10" s="8">
+        <v>732.97</v>
+      </c>
+      <c r="U10" s="8">
+        <v>938</v>
+      </c>
+      <c r="V10" s="8">
+        <v>1143.03</v>
+      </c>
+      <c r="W10" s="8">
+        <v>1348.06</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A11" s="5">
+        <v>7</v>
+      </c>
+      <c r="B11" s="8">
+        <v>15.36</v>
+      </c>
+      <c r="C11" s="8">
+        <v>30.06</v>
+      </c>
+      <c r="D11" s="8">
+        <v>44.76</v>
+      </c>
+      <c r="E11" s="8">
+        <v>52.61</v>
+      </c>
+      <c r="F11" s="8">
+        <v>60.47</v>
+      </c>
+      <c r="G11" s="8">
+        <v>68.33</v>
+      </c>
+      <c r="H11" s="8">
+        <v>77.37</v>
+      </c>
+      <c r="I11" s="8">
+        <v>86.41</v>
+      </c>
+      <c r="J11" s="8">
+        <v>95.45</v>
+      </c>
+      <c r="K11" s="8">
+        <v>110.48</v>
+      </c>
+      <c r="M11" s="9">
+        <v>7</v>
+      </c>
+      <c r="N11" s="8">
+        <v>125.51</v>
+      </c>
+      <c r="O11" s="8">
+        <v>174.86</v>
+      </c>
+      <c r="P11" s="8">
+        <v>224.21</v>
+      </c>
+      <c r="Q11" s="8">
+        <v>273.56</v>
+      </c>
+      <c r="R11" s="8">
+        <v>322.91000000000003</v>
+      </c>
+      <c r="S11" s="8">
+        <v>527.94000000000005</v>
+      </c>
+      <c r="T11" s="8">
+        <v>732.97</v>
+      </c>
+      <c r="U11" s="8">
+        <v>938</v>
+      </c>
+      <c r="V11" s="8">
+        <v>1143.03</v>
+      </c>
+      <c r="W11" s="8">
+        <v>1348.06</v>
+      </c>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A12" s="5">
+        <v>8</v>
+      </c>
+      <c r="B12" s="8">
+        <v>17.440000000000001</v>
+      </c>
+      <c r="C12" s="8">
+        <v>33.35</v>
+      </c>
+      <c r="D12" s="8">
+        <v>49.27</v>
+      </c>
+      <c r="E12" s="8">
+        <v>56.94</v>
+      </c>
+      <c r="F12" s="8">
+        <v>64.62</v>
+      </c>
+      <c r="G12" s="8">
+        <v>72.290000000000006</v>
+      </c>
+      <c r="H12" s="8">
+        <v>81.47</v>
+      </c>
+      <c r="I12" s="8">
+        <v>90.65</v>
+      </c>
+      <c r="J12" s="8">
+        <v>99.83</v>
+      </c>
+      <c r="K12" s="8">
+        <v>112.67</v>
+      </c>
+      <c r="M12" s="9">
+        <v>8</v>
+      </c>
+      <c r="N12" s="8">
+        <v>125.51</v>
+      </c>
+      <c r="O12" s="8">
+        <v>174.86</v>
+      </c>
+      <c r="P12" s="8">
+        <v>224.21</v>
+      </c>
+      <c r="Q12" s="8">
+        <v>273.56</v>
+      </c>
+      <c r="R12" s="8">
+        <v>322.91000000000003</v>
+      </c>
+      <c r="S12" s="8">
+        <v>527.94000000000005</v>
+      </c>
+      <c r="T12" s="8">
+        <v>732.97</v>
+      </c>
+      <c r="U12" s="8">
+        <v>938</v>
+      </c>
+      <c r="V12" s="8">
+        <v>1143.03</v>
+      </c>
+      <c r="W12" s="8">
+        <v>1348.06</v>
+      </c>
+    </row>
+    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A13" s="5">
+        <v>9</v>
+      </c>
+      <c r="B13" s="8">
+        <v>19.510000000000002</v>
+      </c>
+      <c r="C13" s="8">
+        <v>36.64</v>
+      </c>
+      <c r="D13" s="8">
+        <v>53.77</v>
+      </c>
+      <c r="E13" s="8">
+        <v>61.27</v>
+      </c>
+      <c r="F13" s="8">
+        <v>68.77</v>
+      </c>
+      <c r="G13" s="8">
+        <v>76.260000000000005</v>
+      </c>
+      <c r="H13" s="8">
+        <v>85.58</v>
+      </c>
+      <c r="I13" s="8">
+        <v>94.9</v>
+      </c>
+      <c r="J13" s="8">
+        <v>104.21</v>
+      </c>
+      <c r="K13" s="8">
+        <v>114.86</v>
+      </c>
+      <c r="M13" s="9">
+        <v>9</v>
+      </c>
+      <c r="N13" s="8">
+        <v>125.51</v>
+      </c>
+      <c r="O13" s="8">
+        <v>174.86</v>
+      </c>
+      <c r="P13" s="8">
+        <v>224.21</v>
+      </c>
+      <c r="Q13" s="8">
+        <v>273.56</v>
+      </c>
+      <c r="R13" s="8">
+        <v>322.91000000000003</v>
+      </c>
+      <c r="S13" s="8">
+        <v>527.94000000000005</v>
+      </c>
+      <c r="T13" s="8">
+        <v>732.97</v>
+      </c>
+      <c r="U13" s="8">
+        <v>938</v>
+      </c>
+      <c r="V13" s="8">
+        <v>1143.03</v>
+      </c>
+      <c r="W13" s="8">
+        <v>1348.06</v>
+      </c>
+    </row>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A14" s="5">
+        <v>10</v>
+      </c>
+      <c r="B14" s="8">
+        <v>21.07</v>
+      </c>
+      <c r="C14" s="8">
+        <v>37.92</v>
+      </c>
+      <c r="D14" s="8">
+        <v>54.77</v>
+      </c>
+      <c r="E14" s="8">
+        <v>61.9</v>
+      </c>
+      <c r="F14" s="8">
+        <v>69.040000000000006</v>
+      </c>
+      <c r="G14" s="8">
+        <v>76.180000000000007</v>
+      </c>
+      <c r="H14" s="8">
+        <v>85.74</v>
+      </c>
+      <c r="I14" s="8">
+        <v>95.3</v>
+      </c>
+      <c r="J14" s="8">
+        <v>104.86</v>
+      </c>
+      <c r="K14" s="8">
+        <v>115.19</v>
+      </c>
+      <c r="M14" s="9">
+        <v>10</v>
+      </c>
+      <c r="N14" s="8">
+        <v>125.51</v>
+      </c>
+      <c r="O14" s="8">
+        <v>174.86</v>
+      </c>
+      <c r="P14" s="8">
+        <v>224.21</v>
+      </c>
+      <c r="Q14" s="8">
+        <v>273.56</v>
+      </c>
+      <c r="R14" s="8">
+        <v>322.91000000000003</v>
+      </c>
+      <c r="S14" s="8">
+        <v>527.94000000000005</v>
+      </c>
+      <c r="T14" s="8">
+        <v>732.97</v>
+      </c>
+      <c r="U14" s="8">
+        <v>938</v>
+      </c>
+      <c r="V14" s="8">
+        <v>1143.03</v>
+      </c>
+      <c r="W14" s="8">
+        <v>1348.06</v>
+      </c>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A15" s="5">
+        <v>11</v>
+      </c>
+      <c r="B15" s="8">
+        <v>22.63</v>
+      </c>
+      <c r="C15" s="8">
+        <v>39.19</v>
+      </c>
+      <c r="D15" s="8">
+        <v>55.76</v>
+      </c>
+      <c r="E15" s="8">
+        <v>62.54</v>
+      </c>
+      <c r="F15" s="8">
+        <v>69.319999999999993</v>
+      </c>
+      <c r="G15" s="8">
+        <v>76.099999999999994</v>
+      </c>
+      <c r="H15" s="8">
+        <v>85.9</v>
+      </c>
+      <c r="I15" s="8">
+        <v>95.71</v>
+      </c>
+      <c r="J15" s="8">
+        <v>105.51</v>
+      </c>
+      <c r="K15" s="8">
+        <v>115.51</v>
+      </c>
+      <c r="M15" s="9">
+        <v>11</v>
+      </c>
+      <c r="N15" s="8">
+        <v>125.51</v>
+      </c>
+      <c r="O15" s="8">
+        <v>174.86</v>
+      </c>
+      <c r="P15" s="8">
+        <v>224.21</v>
+      </c>
+      <c r="Q15" s="8">
+        <v>273.56</v>
+      </c>
+      <c r="R15" s="8">
+        <v>322.91000000000003</v>
+      </c>
+      <c r="S15" s="8">
+        <v>527.94000000000005</v>
+      </c>
+      <c r="T15" s="8">
+        <v>732.97</v>
+      </c>
+      <c r="U15" s="8">
+        <v>938</v>
+      </c>
+      <c r="V15" s="8">
+        <v>1143.03</v>
+      </c>
+      <c r="W15" s="8">
+        <v>1348.06</v>
+      </c>
+    </row>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A16" s="5">
+        <v>12</v>
+      </c>
+      <c r="B16" s="8">
+        <v>24.18</v>
+      </c>
+      <c r="C16" s="8">
+        <v>40.47</v>
+      </c>
+      <c r="D16" s="8">
+        <v>56.76</v>
+      </c>
+      <c r="E16" s="8">
+        <v>63.17</v>
+      </c>
+      <c r="F16" s="8">
+        <v>69.59</v>
+      </c>
+      <c r="G16" s="8">
+        <v>76.010000000000005</v>
+      </c>
+      <c r="H16" s="8">
+        <v>86.06</v>
+      </c>
+      <c r="I16" s="8">
+        <v>96.11</v>
+      </c>
+      <c r="J16" s="8">
+        <v>106.16</v>
+      </c>
+      <c r="K16" s="8">
+        <v>115.84</v>
+      </c>
+      <c r="M16" s="9">
+        <v>12</v>
+      </c>
+      <c r="N16" s="8">
+        <v>125.51</v>
+      </c>
+      <c r="O16" s="8">
+        <v>174.86</v>
+      </c>
+      <c r="P16" s="8">
+        <v>224.21</v>
+      </c>
+      <c r="Q16" s="8">
+        <v>273.56</v>
+      </c>
+      <c r="R16" s="8">
+        <v>322.91000000000003</v>
+      </c>
+      <c r="S16" s="8">
+        <v>527.94000000000005</v>
+      </c>
+      <c r="T16" s="8">
+        <v>732.97</v>
+      </c>
+      <c r="U16" s="8">
+        <v>938</v>
+      </c>
+      <c r="V16" s="8">
+        <v>1143.03</v>
+      </c>
+      <c r="W16" s="8">
+        <v>1348.06</v>
+      </c>
+    </row>
+    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A17" s="5">
+        <v>13</v>
+      </c>
+      <c r="B17" s="8">
+        <v>25.74</v>
+      </c>
+      <c r="C17" s="8">
+        <v>41.74</v>
+      </c>
+      <c r="D17" s="8">
+        <v>57.75</v>
+      </c>
+      <c r="E17" s="8">
+        <v>63.81</v>
+      </c>
+      <c r="F17" s="8">
+        <v>69.87</v>
+      </c>
+      <c r="G17" s="8">
+        <v>75.930000000000007</v>
+      </c>
+      <c r="H17" s="8">
+        <v>86.22</v>
+      </c>
+      <c r="I17" s="8">
+        <v>96.52</v>
+      </c>
+      <c r="J17" s="8">
+        <v>106.81</v>
+      </c>
+      <c r="K17" s="8">
+        <v>116.16</v>
+      </c>
+      <c r="M17" s="9">
+        <v>13</v>
+      </c>
+      <c r="N17" s="8">
+        <v>125.51</v>
+      </c>
+      <c r="O17" s="8">
+        <v>174.86</v>
+      </c>
+      <c r="P17" s="8">
+        <v>224.21</v>
+      </c>
+      <c r="Q17" s="8">
+        <v>273.56</v>
+      </c>
+      <c r="R17" s="8">
+        <v>322.91000000000003</v>
+      </c>
+      <c r="S17" s="8">
+        <v>527.94000000000005</v>
+      </c>
+      <c r="T17" s="8">
+        <v>732.97</v>
+      </c>
+      <c r="U17" s="8">
+        <v>938</v>
+      </c>
+      <c r="V17" s="8">
+        <v>1143.03</v>
+      </c>
+      <c r="W17" s="8">
+        <v>1348.06</v>
+      </c>
+    </row>
+    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A18" s="5">
+        <v>14</v>
+      </c>
+      <c r="B18" s="8">
+        <v>27.3</v>
+      </c>
+      <c r="C18" s="8">
+        <v>43.02</v>
+      </c>
+      <c r="D18" s="8">
+        <v>58.74</v>
+      </c>
+      <c r="E18" s="8">
+        <v>64.44</v>
+      </c>
+      <c r="F18" s="8">
+        <v>70.14</v>
+      </c>
+      <c r="G18" s="8">
+        <v>75.84</v>
+      </c>
+      <c r="H18" s="8">
+        <v>86.38</v>
+      </c>
+      <c r="I18" s="8">
+        <v>96.92</v>
+      </c>
+      <c r="J18" s="8">
+        <v>107.46</v>
+      </c>
+      <c r="K18" s="8">
+        <v>116.49</v>
+      </c>
+      <c r="M18" s="9">
+        <v>14</v>
+      </c>
+      <c r="N18" s="8">
+        <v>125.51</v>
+      </c>
+      <c r="O18" s="8">
+        <v>174.86</v>
+      </c>
+      <c r="P18" s="8">
+        <v>224.21</v>
+      </c>
+      <c r="Q18" s="8">
+        <v>273.56</v>
+      </c>
+      <c r="R18" s="8">
+        <v>322.91000000000003</v>
+      </c>
+      <c r="S18" s="8">
+        <v>527.94000000000005</v>
+      </c>
+      <c r="T18" s="8">
+        <v>732.97</v>
+      </c>
+      <c r="U18" s="8">
+        <v>938</v>
+      </c>
+      <c r="V18" s="8">
+        <v>1143.03</v>
+      </c>
+      <c r="W18" s="8">
+        <v>1348.06</v>
+      </c>
+    </row>
+    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A19" s="5">
+        <v>15</v>
+      </c>
+      <c r="B19" s="8">
+        <v>28.85</v>
+      </c>
+      <c r="C19" s="8">
+        <v>44.3</v>
+      </c>
+      <c r="D19" s="8">
+        <v>59.74</v>
+      </c>
+      <c r="E19" s="8">
+        <v>65.08</v>
+      </c>
+      <c r="F19" s="8">
+        <v>70.42</v>
+      </c>
+      <c r="G19" s="8">
+        <v>75.760000000000005</v>
+      </c>
+      <c r="H19" s="8">
+        <v>86.54</v>
+      </c>
+      <c r="I19" s="8">
+        <v>97.33</v>
+      </c>
+      <c r="J19" s="8">
+        <v>108.11</v>
+      </c>
+      <c r="K19" s="8">
+        <v>116.81</v>
+      </c>
+      <c r="M19" s="9">
+        <v>15</v>
+      </c>
+      <c r="N19" s="8">
+        <v>125.51</v>
+      </c>
+      <c r="O19" s="8">
+        <v>174.86</v>
+      </c>
+      <c r="P19" s="8">
+        <v>224.21</v>
+      </c>
+      <c r="Q19" s="8">
+        <v>273.56</v>
+      </c>
+      <c r="R19" s="8">
+        <v>322.91000000000003</v>
+      </c>
+      <c r="S19" s="8">
+        <v>527.94000000000005</v>
+      </c>
+      <c r="T19" s="8">
+        <v>732.97</v>
+      </c>
+      <c r="U19" s="8">
+        <v>938</v>
+      </c>
+      <c r="V19" s="8">
+        <v>1143.03</v>
+      </c>
+      <c r="W19" s="8">
+        <v>1348.06</v>
+      </c>
+    </row>
+    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A20" s="5">
+        <v>16</v>
+      </c>
+      <c r="B20" s="8">
+        <v>30.41</v>
+      </c>
+      <c r="C20" s="8">
+        <v>45.57</v>
+      </c>
+      <c r="D20" s="8">
+        <v>60.73</v>
+      </c>
+      <c r="E20" s="8">
+        <v>65.709999999999994</v>
+      </c>
+      <c r="F20" s="8">
+        <v>70.69</v>
+      </c>
+      <c r="G20" s="8">
+        <v>75.67</v>
+      </c>
+      <c r="H20" s="8">
+        <v>86.7</v>
+      </c>
+      <c r="I20" s="8">
+        <v>97.73</v>
+      </c>
+      <c r="J20" s="8">
+        <v>108.76</v>
+      </c>
+      <c r="K20" s="8">
+        <v>117.14</v>
+      </c>
+      <c r="M20" s="9">
+        <v>16</v>
+      </c>
+      <c r="N20" s="8">
+        <v>125.51</v>
+      </c>
+      <c r="O20" s="8">
+        <v>174.86</v>
+      </c>
+      <c r="P20" s="8">
+        <v>224.21</v>
+      </c>
+      <c r="Q20" s="8">
+        <v>273.56</v>
+      </c>
+      <c r="R20" s="8">
+        <v>322.91000000000003</v>
+      </c>
+      <c r="S20" s="8">
+        <v>527.94000000000005</v>
+      </c>
+      <c r="T20" s="8">
+        <v>732.97</v>
+      </c>
+      <c r="U20" s="8">
+        <v>938</v>
+      </c>
+      <c r="V20" s="8">
+        <v>1143.03</v>
+      </c>
+      <c r="W20" s="8">
+        <v>1348.06</v>
+      </c>
+    </row>
+    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A21" s="5">
+        <v>17</v>
+      </c>
+      <c r="B21" s="8">
+        <v>31.97</v>
+      </c>
+      <c r="C21" s="8">
+        <v>46.85</v>
+      </c>
+      <c r="D21" s="8">
+        <v>61.73</v>
+      </c>
+      <c r="E21" s="8">
+        <v>66.349999999999994</v>
+      </c>
+      <c r="F21" s="8">
+        <v>70.97</v>
+      </c>
+      <c r="G21" s="8">
+        <v>75.59</v>
+      </c>
+      <c r="H21" s="8">
+        <v>86.86</v>
+      </c>
+      <c r="I21" s="8">
+        <v>98.14</v>
+      </c>
+      <c r="J21" s="8">
+        <v>109.41</v>
+      </c>
+      <c r="K21" s="8">
+        <v>117.46</v>
+      </c>
+      <c r="M21" s="9">
+        <v>17</v>
+      </c>
+      <c r="N21" s="8">
+        <v>125.51</v>
+      </c>
+      <c r="O21" s="8">
+        <v>174.86</v>
+      </c>
+      <c r="P21" s="8">
+        <v>224.21</v>
+      </c>
+      <c r="Q21" s="8">
+        <v>273.56</v>
+      </c>
+      <c r="R21" s="8">
+        <v>322.91000000000003</v>
+      </c>
+      <c r="S21" s="8">
+        <v>527.94000000000005</v>
+      </c>
+      <c r="T21" s="8">
+        <v>732.97</v>
+      </c>
+      <c r="U21" s="8">
+        <v>938</v>
+      </c>
+      <c r="V21" s="8">
+        <v>1143.03</v>
+      </c>
+      <c r="W21" s="8">
+        <v>1348.06</v>
+      </c>
+    </row>
+    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A22" s="5">
+        <v>18</v>
+      </c>
+      <c r="B22" s="8">
+        <v>33.520000000000003</v>
+      </c>
+      <c r="C22" s="8">
+        <v>48.12</v>
+      </c>
+      <c r="D22" s="8">
+        <v>62.72</v>
+      </c>
+      <c r="E22" s="8">
+        <v>66.98</v>
+      </c>
+      <c r="F22" s="8">
+        <v>71.239999999999995</v>
+      </c>
+      <c r="G22" s="8">
+        <v>75.5</v>
+      </c>
+      <c r="H22" s="8">
+        <v>87.02</v>
+      </c>
+      <c r="I22" s="8">
+        <v>98.54</v>
+      </c>
+      <c r="J22" s="8">
+        <v>110.06</v>
+      </c>
+      <c r="K22" s="8">
+        <v>117.79</v>
+      </c>
+      <c r="M22" s="9">
+        <v>18</v>
+      </c>
+      <c r="N22" s="8">
+        <v>125.51</v>
+      </c>
+      <c r="O22" s="8">
+        <v>174.86</v>
+      </c>
+      <c r="P22" s="8">
+        <v>224.21</v>
+      </c>
+      <c r="Q22" s="8">
+        <v>273.56</v>
+      </c>
+      <c r="R22" s="8">
+        <v>322.91000000000003</v>
+      </c>
+      <c r="S22" s="8">
+        <v>527.94000000000005</v>
+      </c>
+      <c r="T22" s="8">
+        <v>732.97</v>
+      </c>
+      <c r="U22" s="8">
+        <v>938</v>
+      </c>
+      <c r="V22" s="8">
+        <v>1143.03</v>
+      </c>
+      <c r="W22" s="8">
+        <v>1348.06</v>
+      </c>
+    </row>
+    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A23" s="5">
+        <v>19</v>
+      </c>
+      <c r="B23" s="8">
+        <v>35.08</v>
+      </c>
+      <c r="C23" s="8">
+        <v>49.4</v>
+      </c>
+      <c r="D23" s="8">
+        <v>63.72</v>
+      </c>
+      <c r="E23" s="8">
+        <v>67.62</v>
+      </c>
+      <c r="F23" s="8">
+        <v>71.52</v>
+      </c>
+      <c r="G23" s="8">
+        <v>75.42</v>
+      </c>
+      <c r="H23" s="8">
+        <v>87.18</v>
+      </c>
+      <c r="I23" s="8">
+        <v>98.95</v>
+      </c>
+      <c r="J23" s="8">
+        <v>110.71</v>
+      </c>
+      <c r="K23" s="8">
+        <v>118.11</v>
+      </c>
+      <c r="M23" s="9">
+        <v>19</v>
+      </c>
+      <c r="N23" s="8">
+        <v>125.51</v>
+      </c>
+      <c r="O23" s="8">
+        <v>174.86</v>
+      </c>
+      <c r="P23" s="8">
+        <v>224.21</v>
+      </c>
+      <c r="Q23" s="8">
+        <v>273.56</v>
+      </c>
+      <c r="R23" s="8">
+        <v>322.91000000000003</v>
+      </c>
+      <c r="S23" s="8">
+        <v>527.94000000000005</v>
+      </c>
+      <c r="T23" s="8">
+        <v>732.97</v>
+      </c>
+      <c r="U23" s="8">
+        <v>938</v>
+      </c>
+      <c r="V23" s="8">
+        <v>1143.03</v>
+      </c>
+      <c r="W23" s="8">
+        <v>1348.06</v>
+      </c>
+    </row>
+    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A24" s="5">
+        <v>20</v>
+      </c>
+      <c r="B24" s="8">
+        <v>36.64</v>
+      </c>
+      <c r="C24" s="8">
+        <v>50.67</v>
+      </c>
+      <c r="D24" s="8">
+        <v>64.709999999999994</v>
+      </c>
+      <c r="E24" s="8">
+        <v>68.25</v>
+      </c>
+      <c r="F24" s="8">
+        <v>71.790000000000006</v>
+      </c>
+      <c r="G24" s="8">
+        <v>75.34</v>
+      </c>
+      <c r="H24" s="8">
+        <v>87.34</v>
+      </c>
+      <c r="I24" s="8">
+        <v>99.35</v>
+      </c>
+      <c r="J24" s="8">
+        <v>111.36</v>
+      </c>
+      <c r="K24" s="8">
+        <v>118.44</v>
+      </c>
+      <c r="M24" s="9">
+        <v>20</v>
+      </c>
+      <c r="N24" s="8">
+        <v>125.51</v>
+      </c>
+      <c r="O24" s="8">
+        <v>174.86</v>
+      </c>
+      <c r="P24" s="8">
+        <v>224.21</v>
+      </c>
+      <c r="Q24" s="8">
+        <v>273.56</v>
+      </c>
+      <c r="R24" s="8">
+        <v>322.91000000000003</v>
+      </c>
+      <c r="S24" s="8">
+        <v>527.94000000000005</v>
+      </c>
+      <c r="T24" s="8">
+        <v>732.97</v>
+      </c>
+      <c r="U24" s="8">
+        <v>938</v>
+      </c>
+      <c r="V24" s="8">
+        <v>1143.03</v>
+      </c>
+      <c r="W24" s="8">
+        <v>1348.06</v>
+      </c>
+    </row>
+    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A25" s="5">
+        <v>21</v>
+      </c>
+      <c r="B25" s="8">
+        <v>38.19</v>
+      </c>
+      <c r="C25" s="8">
+        <v>51.95</v>
+      </c>
+      <c r="D25" s="8">
+        <v>65.7</v>
+      </c>
+      <c r="E25" s="8">
+        <v>68.89</v>
+      </c>
+      <c r="F25" s="8">
+        <v>72.069999999999993</v>
+      </c>
+      <c r="G25" s="8">
+        <v>75.25</v>
+      </c>
+      <c r="H25" s="8">
+        <v>87.5</v>
+      </c>
+      <c r="I25" s="8">
+        <v>99.76</v>
+      </c>
+      <c r="J25" s="8">
+        <v>112.01</v>
+      </c>
+      <c r="K25" s="8">
+        <v>118.76</v>
+      </c>
+      <c r="M25" s="9">
+        <v>21</v>
+      </c>
+      <c r="N25" s="8">
+        <v>125.51</v>
+      </c>
+      <c r="O25" s="8">
+        <v>174.86</v>
+      </c>
+      <c r="P25" s="8">
+        <v>224.21</v>
+      </c>
+      <c r="Q25" s="8">
+        <v>273.56</v>
+      </c>
+      <c r="R25" s="8">
+        <v>322.91000000000003</v>
+      </c>
+      <c r="S25" s="8">
+        <v>527.94000000000005</v>
+      </c>
+      <c r="T25" s="8">
+        <v>732.97</v>
+      </c>
+      <c r="U25" s="8">
+        <v>938</v>
+      </c>
+      <c r="V25" s="8">
+        <v>1143.03</v>
+      </c>
+      <c r="W25" s="8">
+        <v>1348.06</v>
+      </c>
+    </row>
+    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A26" s="5">
+        <v>22</v>
+      </c>
+      <c r="B26" s="8">
+        <v>39.75</v>
+      </c>
+      <c r="C26" s="8">
+        <v>53.22</v>
+      </c>
+      <c r="D26" s="8">
+        <v>66.7</v>
+      </c>
+      <c r="E26" s="8">
+        <v>69.52</v>
+      </c>
+      <c r="F26" s="8">
+        <v>72.34</v>
+      </c>
+      <c r="G26" s="8">
+        <v>75.17</v>
+      </c>
+      <c r="H26" s="8">
+        <v>87.66</v>
+      </c>
+      <c r="I26" s="8">
+        <v>100.16</v>
+      </c>
+      <c r="J26" s="8">
+        <v>112.66</v>
+      </c>
+      <c r="K26" s="8">
+        <v>119.08</v>
+      </c>
+      <c r="M26" s="9">
+        <v>22</v>
+      </c>
+      <c r="N26" s="8">
+        <v>125.51</v>
+      </c>
+      <c r="O26" s="8">
+        <v>174.86</v>
+      </c>
+      <c r="P26" s="8">
+        <v>224.21</v>
+      </c>
+      <c r="Q26" s="8">
+        <v>273.56</v>
+      </c>
+      <c r="R26" s="8">
+        <v>322.91000000000003</v>
+      </c>
+      <c r="S26" s="8">
+        <v>527.94000000000005</v>
+      </c>
+      <c r="T26" s="8">
+        <v>732.97</v>
+      </c>
+      <c r="U26" s="8">
+        <v>938</v>
+      </c>
+      <c r="V26" s="8">
+        <v>1143.03</v>
+      </c>
+      <c r="W26" s="8">
+        <v>1348.06</v>
+      </c>
+    </row>
+    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A27" s="5">
+        <v>23</v>
+      </c>
+      <c r="B27" s="8">
+        <v>41.31</v>
+      </c>
+      <c r="C27" s="8">
+        <v>54.5</v>
+      </c>
+      <c r="D27" s="8">
+        <v>67.69</v>
+      </c>
+      <c r="E27" s="8">
+        <v>70.16</v>
+      </c>
+      <c r="F27" s="8">
+        <v>72.62</v>
+      </c>
+      <c r="G27" s="8">
+        <v>75.08</v>
+      </c>
+      <c r="H27" s="8">
+        <v>87.82</v>
+      </c>
+      <c r="I27" s="8">
+        <v>100.57</v>
+      </c>
+      <c r="J27" s="8">
+        <v>113.31</v>
+      </c>
+      <c r="K27" s="8">
+        <v>119.41</v>
+      </c>
+      <c r="M27" s="9">
+        <v>23</v>
+      </c>
+      <c r="N27" s="8">
+        <v>125.51</v>
+      </c>
+      <c r="O27" s="8">
+        <v>174.86</v>
+      </c>
+      <c r="P27" s="8">
+        <v>224.21</v>
+      </c>
+      <c r="Q27" s="8">
+        <v>273.56</v>
+      </c>
+      <c r="R27" s="8">
+        <v>322.91000000000003</v>
+      </c>
+      <c r="S27" s="8">
+        <v>527.94000000000005</v>
+      </c>
+      <c r="T27" s="8">
+        <v>732.97</v>
+      </c>
+      <c r="U27" s="8">
+        <v>938</v>
+      </c>
+      <c r="V27" s="8">
+        <v>1143.03</v>
+      </c>
+      <c r="W27" s="8">
+        <v>1348.06</v>
+      </c>
+    </row>
+    <row r="28" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A28" s="5">
+        <v>24</v>
+      </c>
+      <c r="B28" s="8">
+        <v>42.86</v>
+      </c>
+      <c r="C28" s="8">
+        <v>55.77</v>
+      </c>
+      <c r="D28" s="8">
+        <v>68.69</v>
+      </c>
+      <c r="E28" s="8">
+        <v>70.790000000000006</v>
+      </c>
+      <c r="F28" s="8">
+        <v>72.89</v>
+      </c>
+      <c r="G28" s="8">
+        <v>75</v>
+      </c>
+      <c r="H28" s="8">
+        <v>87.98</v>
+      </c>
+      <c r="I28" s="8">
+        <v>100.97</v>
+      </c>
+      <c r="J28" s="8">
+        <v>113.96</v>
+      </c>
+      <c r="K28" s="8">
+        <v>119.73</v>
+      </c>
+      <c r="M28" s="9">
+        <v>24</v>
+      </c>
+      <c r="N28" s="8">
+        <v>125.51</v>
+      </c>
+      <c r="O28" s="8">
+        <v>174.86</v>
+      </c>
+      <c r="P28" s="8">
+        <v>224.21</v>
+      </c>
+      <c r="Q28" s="8">
+        <v>273.56</v>
+      </c>
+      <c r="R28" s="8">
+        <v>322.91000000000003</v>
+      </c>
+      <c r="S28" s="8">
+        <v>527.94000000000005</v>
+      </c>
+      <c r="T28" s="8">
+        <v>732.97</v>
+      </c>
+      <c r="U28" s="8">
+        <v>938</v>
+      </c>
+      <c r="V28" s="8">
+        <v>1143.03</v>
+      </c>
+      <c r="W28" s="8">
+        <v>1348.06</v>
+      </c>
+    </row>
+    <row r="29" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A29" s="5">
+        <v>25</v>
+      </c>
+      <c r="B29" s="8">
+        <v>44.42</v>
+      </c>
+      <c r="C29" s="8">
+        <v>57.05</v>
+      </c>
+      <c r="D29" s="8">
+        <v>69.680000000000007</v>
+      </c>
+      <c r="E29" s="8">
+        <v>71.430000000000007</v>
+      </c>
+      <c r="F29" s="8">
+        <v>73.17</v>
+      </c>
+      <c r="G29" s="8">
+        <v>74.91</v>
+      </c>
+      <c r="H29" s="8">
+        <v>88.14</v>
+      </c>
+      <c r="I29" s="8">
+        <v>101.38</v>
+      </c>
+      <c r="J29" s="8">
+        <v>114.61</v>
+      </c>
+      <c r="K29" s="8">
+        <v>120.06</v>
+      </c>
+      <c r="M29" s="9">
+        <v>25</v>
+      </c>
+      <c r="N29" s="8">
+        <v>125.51</v>
+      </c>
+      <c r="O29" s="8">
+        <v>174.86</v>
+      </c>
+      <c r="P29" s="8">
+        <v>224.21</v>
+      </c>
+      <c r="Q29" s="8">
+        <v>273.56</v>
+      </c>
+      <c r="R29" s="8">
+        <v>322.91000000000003</v>
+      </c>
+      <c r="S29" s="8">
+        <v>527.94000000000005</v>
+      </c>
+      <c r="T29" s="8">
+        <v>732.97</v>
+      </c>
+      <c r="U29" s="8">
+        <v>938</v>
+      </c>
+      <c r="V29" s="8">
+        <v>1143.03</v>
+      </c>
+      <c r="W29" s="8">
+        <v>1348.06</v>
+      </c>
+    </row>
+    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A30" s="5">
+        <v>26</v>
+      </c>
+      <c r="B30" s="8">
+        <v>45.98</v>
+      </c>
+      <c r="C30" s="8">
+        <v>58.33</v>
+      </c>
+      <c r="D30" s="8">
+        <v>70.680000000000007</v>
+      </c>
+      <c r="E30" s="8">
+        <v>72.06</v>
+      </c>
+      <c r="F30" s="8">
+        <v>73.44</v>
+      </c>
+      <c r="G30" s="8">
+        <v>74.83</v>
+      </c>
+      <c r="H30" s="8">
+        <v>88.3</v>
+      </c>
+      <c r="I30" s="8">
+        <v>101.78</v>
+      </c>
+      <c r="J30" s="8">
+        <v>115.26</v>
+      </c>
+      <c r="K30" s="8">
+        <v>120.38</v>
+      </c>
+      <c r="M30" s="9">
+        <v>26</v>
+      </c>
+      <c r="N30" s="8">
+        <v>125.51</v>
+      </c>
+      <c r="O30" s="8">
+        <v>174.86</v>
+      </c>
+      <c r="P30" s="8">
+        <v>224.21</v>
+      </c>
+      <c r="Q30" s="8">
+        <v>273.56</v>
+      </c>
+      <c r="R30" s="8">
+        <v>322.91000000000003</v>
+      </c>
+      <c r="S30" s="8">
+        <v>527.94000000000005</v>
+      </c>
+      <c r="T30" s="8">
+        <v>732.97</v>
+      </c>
+      <c r="U30" s="8">
+        <v>938</v>
+      </c>
+      <c r="V30" s="8">
+        <v>1143.03</v>
+      </c>
+      <c r="W30" s="8">
+        <v>1348.06</v>
+      </c>
+    </row>
+    <row r="31" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A31" s="5">
+        <v>27</v>
+      </c>
+      <c r="B31" s="8">
+        <v>47.53</v>
+      </c>
+      <c r="C31" s="8">
+        <v>59.6</v>
+      </c>
+      <c r="D31" s="8">
+        <v>71.67</v>
+      </c>
+      <c r="E31" s="8">
+        <v>72.7</v>
+      </c>
+      <c r="F31" s="8">
+        <v>73.72</v>
+      </c>
+      <c r="G31" s="8">
+        <v>74.739999999999995</v>
+      </c>
+      <c r="H31" s="8">
+        <v>88.47</v>
+      </c>
+      <c r="I31" s="8">
+        <v>102.19</v>
+      </c>
+      <c r="J31" s="8">
+        <v>115.91</v>
+      </c>
+      <c r="K31" s="8">
+        <v>120.71</v>
+      </c>
+      <c r="M31" s="9">
+        <v>27</v>
+      </c>
+      <c r="N31" s="8">
+        <v>125.51</v>
+      </c>
+      <c r="O31" s="8">
+        <v>174.86</v>
+      </c>
+      <c r="P31" s="8">
+        <v>224.21</v>
+      </c>
+      <c r="Q31" s="8">
+        <v>273.56</v>
+      </c>
+      <c r="R31" s="8">
+        <v>322.91000000000003</v>
+      </c>
+      <c r="S31" s="8">
+        <v>527.94000000000005</v>
+      </c>
+      <c r="T31" s="8">
+        <v>732.97</v>
+      </c>
+      <c r="U31" s="8">
+        <v>938</v>
+      </c>
+      <c r="V31" s="8">
+        <v>1143.03</v>
+      </c>
+      <c r="W31" s="8">
+        <v>1348.06</v>
+      </c>
+    </row>
+    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A32" s="5">
+        <v>28</v>
+      </c>
+      <c r="B32" s="8">
+        <v>49.09</v>
+      </c>
+      <c r="C32" s="8">
+        <v>60.88</v>
+      </c>
+      <c r="D32" s="8">
+        <v>72.66</v>
+      </c>
+      <c r="E32" s="8">
+        <v>73.33</v>
+      </c>
+      <c r="F32" s="8">
+        <v>73.989999999999995</v>
+      </c>
+      <c r="G32" s="8">
+        <v>74.66</v>
+      </c>
+      <c r="H32" s="8">
+        <v>88.63</v>
+      </c>
+      <c r="I32" s="8">
+        <v>102.59</v>
+      </c>
+      <c r="J32" s="8">
+        <v>116.56</v>
+      </c>
+      <c r="K32" s="8">
+        <v>121.03</v>
+      </c>
+      <c r="M32" s="9">
+        <v>28</v>
+      </c>
+      <c r="N32" s="8">
+        <v>125.51</v>
+      </c>
+      <c r="O32" s="8">
+        <v>174.86</v>
+      </c>
+      <c r="P32" s="8">
+        <v>224.21</v>
+      </c>
+      <c r="Q32" s="8">
+        <v>273.56</v>
+      </c>
+      <c r="R32" s="8">
+        <v>322.91000000000003</v>
+      </c>
+      <c r="S32" s="8">
+        <v>527.94000000000005</v>
+      </c>
+      <c r="T32" s="8">
+        <v>732.97</v>
+      </c>
+      <c r="U32" s="8">
+        <v>938</v>
+      </c>
+      <c r="V32" s="8">
+        <v>1143.03</v>
+      </c>
+      <c r="W32" s="8">
+        <v>1348.06</v>
+      </c>
+    </row>
+    <row r="33" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A33" s="5">
+        <v>29</v>
+      </c>
+      <c r="B33" s="8">
+        <v>50.65</v>
+      </c>
+      <c r="C33" s="8">
+        <v>62.15</v>
+      </c>
+      <c r="D33" s="8">
+        <v>73.66</v>
+      </c>
+      <c r="E33" s="8">
+        <v>73.959999999999994</v>
+      </c>
+      <c r="F33" s="8">
+        <v>74.27</v>
+      </c>
+      <c r="G33" s="8">
+        <v>74.58</v>
+      </c>
+      <c r="H33" s="8">
+        <v>88.79</v>
+      </c>
+      <c r="I33" s="8">
+        <v>103</v>
+      </c>
+      <c r="J33" s="8">
+        <v>117.21</v>
+      </c>
+      <c r="K33" s="8">
+        <v>121.36</v>
+      </c>
+      <c r="M33" s="9">
+        <v>29</v>
+      </c>
+      <c r="N33" s="8">
+        <v>125.51</v>
+      </c>
+      <c r="O33" s="8">
+        <v>174.86</v>
+      </c>
+      <c r="P33" s="8">
+        <v>224.21</v>
+      </c>
+      <c r="Q33" s="8">
+        <v>273.56</v>
+      </c>
+      <c r="R33" s="8">
+        <v>322.91000000000003</v>
+      </c>
+      <c r="S33" s="8">
+        <v>527.94000000000005</v>
+      </c>
+      <c r="T33" s="8">
+        <v>732.97</v>
+      </c>
+      <c r="U33" s="8">
+        <v>938</v>
+      </c>
+      <c r="V33" s="8">
+        <v>1143.03</v>
+      </c>
+      <c r="W33" s="8">
+        <v>1348.06</v>
+      </c>
+    </row>
+    <row r="34" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A34" s="5">
+        <v>30</v>
+      </c>
+      <c r="B34" s="8">
+        <v>52.2</v>
+      </c>
+      <c r="C34" s="8">
+        <v>63.43</v>
+      </c>
+      <c r="D34" s="8">
+        <v>74.650000000000006</v>
+      </c>
+      <c r="E34" s="8">
+        <v>74.599999999999994</v>
+      </c>
+      <c r="F34" s="8">
+        <v>74.55</v>
+      </c>
+      <c r="G34" s="8">
+        <v>74.489999999999995</v>
+      </c>
+      <c r="H34" s="8">
+        <v>88.95</v>
+      </c>
+      <c r="I34" s="8">
+        <v>103.4</v>
+      </c>
+      <c r="J34" s="8">
+        <v>117.86</v>
+      </c>
+      <c r="K34" s="8">
+        <v>121.68</v>
+      </c>
+      <c r="M34" s="9">
+        <v>30</v>
+      </c>
+      <c r="N34" s="8">
+        <v>125.51</v>
+      </c>
+      <c r="O34" s="8">
+        <v>174.86</v>
+      </c>
+      <c r="P34" s="8">
+        <v>224.21</v>
+      </c>
+      <c r="Q34" s="8">
+        <v>273.56</v>
+      </c>
+      <c r="R34" s="8">
+        <v>322.91000000000003</v>
+      </c>
+      <c r="S34" s="8">
+        <v>527.94000000000005</v>
+      </c>
+      <c r="T34" s="8">
+        <v>732.97</v>
+      </c>
+      <c r="U34" s="8">
+        <v>938</v>
+      </c>
+      <c r="V34" s="8">
+        <v>1143.03</v>
+      </c>
+      <c r="W34" s="8">
+        <v>1348.06</v>
+      </c>
+    </row>
+    <row r="35" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A35" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B35" s="8">
+        <v>29.896666666666668</v>
+      </c>
+      <c r="C35" s="8">
+        <v>43.219333333333338</v>
+      </c>
+      <c r="D35" s="8">
+        <v>56.542333333333353</v>
+      </c>
+      <c r="E35" s="8">
+        <v>61.143000000000001</v>
+      </c>
+      <c r="F35" s="8">
+        <v>65.74366666666667</v>
+      </c>
+      <c r="G35" s="8">
+        <v>70.345333333333329</v>
+      </c>
+      <c r="H35" s="8">
+        <v>81.351666666666659</v>
+      </c>
+      <c r="I35" s="8">
+        <v>92.362000000000023</v>
+      </c>
+      <c r="J35" s="8">
+        <v>103.37033333333333</v>
+      </c>
+      <c r="K35" s="8">
+        <v>114.43966666666668</v>
+      </c>
+      <c r="M35" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="N35" s="10">
+        <v>125.51000000000009</v>
+      </c>
+      <c r="O35" s="10">
+        <v>174.86</v>
+      </c>
+      <c r="P35" s="10">
+        <v>224.21</v>
+      </c>
+      <c r="Q35" s="10">
+        <v>273.56000000000017</v>
+      </c>
+      <c r="R35" s="10">
+        <v>322.90999999999991</v>
+      </c>
+      <c r="S35" s="10">
+        <v>527.9400000000004</v>
+      </c>
+      <c r="T35" s="10">
+        <v>732.97</v>
+      </c>
+      <c r="U35" s="10">
+        <v>938</v>
+      </c>
+      <c r="V35" s="10">
+        <v>1143.0299999999995</v>
+      </c>
+      <c r="W35" s="10">
+        <v>1348.06</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B2:K2"/>
+    <mergeCell ref="M1:W1"/>
+    <mergeCell ref="N2:W2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3EEC94F4-4E93-438D-92F8-5C9CBA48C22A}">
   <dimension ref="A1:W35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3055,7 +5385,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{612EBB24-0E24-4D37-B6A7-8B4DA2BD1A51}">
   <dimension ref="A1:W35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5378,7 +7708,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A2E7E46-B70B-4DB0-97AE-2138287FA00A}">
   <dimension ref="A1:W35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -7701,7 +10031,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D32525DC-1FAE-40FA-B3A1-6E6C0B62B72E}">
   <dimension ref="A1:W35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -10024,7 +12354,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <sheetPr codeName="Sheet9">
     <tabColor rgb="FFFFFF00"/>

</xml_diff>

<commit_message>
📊 Update NAIC content history - 2026-07-02
</commit_message>
<xml_diff>
--- a/docs/content_history/pbr-2026-vm20-table-f-g-current-spreads.xlsx
+++ b/docs/content_history/pbr-2026-vm20-table-f-g-current-spreads.xlsx
@@ -1,24 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\PBR\VM20_VM22_ProductSupport\PBR Production Web Data\Current Year\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B217903-9369-45E9-9ACD-B41ABCB3658B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AE96921-D258-4EBB-BD8B-D2333E983B4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="795" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="795" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="May_2026" sheetId="28" r:id="rId1"/>
-    <sheet name="April_2026" sheetId="27" r:id="rId2"/>
-    <sheet name="March_2026" sheetId="26" r:id="rId3"/>
-    <sheet name="February_2026" sheetId="25" r:id="rId4"/>
-    <sheet name="January_2026" sheetId="24" r:id="rId5"/>
-    <sheet name="LEGAL DISCLAIMER" sheetId="11" r:id="rId6"/>
+    <sheet name="June_2026" sheetId="29" r:id="rId1"/>
+    <sheet name="May_2026" sheetId="28" r:id="rId2"/>
+    <sheet name="April_2026" sheetId="27" r:id="rId3"/>
+    <sheet name="March_2026" sheetId="26" r:id="rId4"/>
+    <sheet name="February_2026" sheetId="25" r:id="rId5"/>
+    <sheet name="January_2026" sheetId="24" r:id="rId6"/>
+    <sheet name="LEGAL DISCLAIMER" sheetId="11" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="38">
   <si>
     <t>WAL</t>
   </si>
@@ -143,6 +144,12 @@
   </si>
   <si>
     <t>Table G. (05/29/2026) Below Investment Grade Current Benchmark Spreads (in bps)</t>
+  </si>
+  <si>
+    <t>Table F (06/30/2026)  Investment Grade Current Benchmark Spreads (in bps)</t>
+  </si>
+  <si>
+    <t>Table G. (06/30/2026) Below Investment Grade Current Benchmark Spreads (in bps)</t>
   </si>
 </sst>
 </file>
@@ -419,7 +426,7 @@
                   <a14:compatExt spid="_x0000_s4104"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0400-000008100000}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0500-000008100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -740,6 +747,2329 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{918B0DAF-F95D-4AE3-B8B6-445C4F5FB350}">
+  <dimension ref="A1:W35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.140625" customWidth="1"/>
+    <col min="13" max="23" width="11.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="M1" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="N1" s="14"/>
+      <c r="O1" s="14"/>
+      <c r="P1" s="14"/>
+      <c r="Q1" s="14"/>
+      <c r="R1" s="14"/>
+      <c r="S1" s="14"/>
+      <c r="T1" s="14"/>
+      <c r="U1" s="14"/>
+      <c r="V1" s="14"/>
+      <c r="W1" s="15"/>
+    </row>
+    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12"/>
+      <c r="K2" s="12"/>
+      <c r="M2" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="N2" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="O2" s="12"/>
+      <c r="P2" s="12"/>
+      <c r="Q2" s="12"/>
+      <c r="R2" s="12"/>
+      <c r="S2" s="12"/>
+      <c r="T2" s="12"/>
+      <c r="U2" s="12"/>
+      <c r="V2" s="12"/>
+      <c r="W2" s="12"/>
+    </row>
+    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="5">
+        <v>1</v>
+      </c>
+      <c r="C3" s="5">
+        <v>2</v>
+      </c>
+      <c r="D3" s="5">
+        <v>3</v>
+      </c>
+      <c r="E3" s="5">
+        <v>4</v>
+      </c>
+      <c r="F3" s="5">
+        <v>5</v>
+      </c>
+      <c r="G3" s="5">
+        <v>6</v>
+      </c>
+      <c r="H3" s="5">
+        <v>7</v>
+      </c>
+      <c r="I3" s="5">
+        <v>8</v>
+      </c>
+      <c r="J3" s="5">
+        <v>9</v>
+      </c>
+      <c r="K3" s="5">
+        <v>10</v>
+      </c>
+      <c r="M3" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="N3" s="5">
+        <v>11</v>
+      </c>
+      <c r="O3" s="5">
+        <v>12</v>
+      </c>
+      <c r="P3" s="5">
+        <v>13</v>
+      </c>
+      <c r="Q3" s="5">
+        <v>14</v>
+      </c>
+      <c r="R3" s="5">
+        <v>15</v>
+      </c>
+      <c r="S3" s="5">
+        <v>16</v>
+      </c>
+      <c r="T3" s="5">
+        <v>17</v>
+      </c>
+      <c r="U3" s="5">
+        <v>18</v>
+      </c>
+      <c r="V3" s="5">
+        <v>19</v>
+      </c>
+      <c r="W3" s="5">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="M4" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="P4" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q4" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="R4" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="S4" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="T4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="U4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="V4" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="W4" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A5" s="5">
+        <v>1</v>
+      </c>
+      <c r="B5" s="8">
+        <v>0.1</v>
+      </c>
+      <c r="C5" s="8">
+        <v>10.92</v>
+      </c>
+      <c r="D5" s="8">
+        <v>21.73</v>
+      </c>
+      <c r="E5" s="8">
+        <v>26.34</v>
+      </c>
+      <c r="F5" s="8">
+        <v>30.94</v>
+      </c>
+      <c r="G5" s="8">
+        <v>35.549999999999997</v>
+      </c>
+      <c r="H5" s="8">
+        <v>42.04</v>
+      </c>
+      <c r="I5" s="8">
+        <v>48.53</v>
+      </c>
+      <c r="J5" s="8">
+        <v>55.02</v>
+      </c>
+      <c r="K5" s="8">
+        <v>90.85</v>
+      </c>
+      <c r="M5" s="9">
+        <v>1</v>
+      </c>
+      <c r="N5" s="8">
+        <v>126.67</v>
+      </c>
+      <c r="O5" s="8">
+        <v>175.53</v>
+      </c>
+      <c r="P5" s="8">
+        <v>224.39</v>
+      </c>
+      <c r="Q5" s="8">
+        <v>273.24</v>
+      </c>
+      <c r="R5" s="8">
+        <v>322.10000000000002</v>
+      </c>
+      <c r="S5" s="8">
+        <v>538.05999999999995</v>
+      </c>
+      <c r="T5" s="8">
+        <v>754.03</v>
+      </c>
+      <c r="U5" s="8">
+        <v>970</v>
+      </c>
+      <c r="V5" s="8">
+        <v>1185.97</v>
+      </c>
+      <c r="W5" s="8">
+        <v>1401.94</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A6" s="5">
+        <v>2</v>
+      </c>
+      <c r="B6" s="8">
+        <v>4.72</v>
+      </c>
+      <c r="C6" s="8">
+        <v>15.68</v>
+      </c>
+      <c r="D6" s="8">
+        <v>26.63</v>
+      </c>
+      <c r="E6" s="8">
+        <v>31.95</v>
+      </c>
+      <c r="F6" s="8">
+        <v>37.270000000000003</v>
+      </c>
+      <c r="G6" s="8">
+        <v>42.59</v>
+      </c>
+      <c r="H6" s="8">
+        <v>49.95</v>
+      </c>
+      <c r="I6" s="8">
+        <v>57.31</v>
+      </c>
+      <c r="J6" s="8">
+        <v>64.680000000000007</v>
+      </c>
+      <c r="K6" s="8">
+        <v>95.68</v>
+      </c>
+      <c r="M6" s="9">
+        <v>2</v>
+      </c>
+      <c r="N6" s="8">
+        <v>126.67</v>
+      </c>
+      <c r="O6" s="8">
+        <v>175.53</v>
+      </c>
+      <c r="P6" s="8">
+        <v>224.39</v>
+      </c>
+      <c r="Q6" s="8">
+        <v>273.24</v>
+      </c>
+      <c r="R6" s="8">
+        <v>322.10000000000002</v>
+      </c>
+      <c r="S6" s="8">
+        <v>538.05999999999995</v>
+      </c>
+      <c r="T6" s="8">
+        <v>754.03</v>
+      </c>
+      <c r="U6" s="8">
+        <v>970</v>
+      </c>
+      <c r="V6" s="8">
+        <v>1185.97</v>
+      </c>
+      <c r="W6" s="8">
+        <v>1401.94</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A7" s="5">
+        <v>3</v>
+      </c>
+      <c r="B7" s="8">
+        <v>9.34</v>
+      </c>
+      <c r="C7" s="8">
+        <v>20.440000000000001</v>
+      </c>
+      <c r="D7" s="8">
+        <v>31.53</v>
+      </c>
+      <c r="E7" s="8">
+        <v>37.57</v>
+      </c>
+      <c r="F7" s="8">
+        <v>43.6</v>
+      </c>
+      <c r="G7" s="8">
+        <v>49.63</v>
+      </c>
+      <c r="H7" s="8">
+        <v>57.87</v>
+      </c>
+      <c r="I7" s="8">
+        <v>66.099999999999994</v>
+      </c>
+      <c r="J7" s="8">
+        <v>74.33</v>
+      </c>
+      <c r="K7" s="8">
+        <v>100.5</v>
+      </c>
+      <c r="M7" s="9">
+        <v>3</v>
+      </c>
+      <c r="N7" s="8">
+        <v>126.67</v>
+      </c>
+      <c r="O7" s="8">
+        <v>175.53</v>
+      </c>
+      <c r="P7" s="8">
+        <v>224.39</v>
+      </c>
+      <c r="Q7" s="8">
+        <v>273.24</v>
+      </c>
+      <c r="R7" s="8">
+        <v>322.10000000000002</v>
+      </c>
+      <c r="S7" s="8">
+        <v>538.05999999999995</v>
+      </c>
+      <c r="T7" s="8">
+        <v>754.03</v>
+      </c>
+      <c r="U7" s="8">
+        <v>970</v>
+      </c>
+      <c r="V7" s="8">
+        <v>1185.97</v>
+      </c>
+      <c r="W7" s="8">
+        <v>1401.94</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A8" s="5">
+        <v>4</v>
+      </c>
+      <c r="B8" s="8">
+        <v>13.96</v>
+      </c>
+      <c r="C8" s="8">
+        <v>25.2</v>
+      </c>
+      <c r="D8" s="8">
+        <v>36.43</v>
+      </c>
+      <c r="E8" s="8">
+        <v>43.18</v>
+      </c>
+      <c r="F8" s="8">
+        <v>49.93</v>
+      </c>
+      <c r="G8" s="8">
+        <v>56.68</v>
+      </c>
+      <c r="H8" s="8">
+        <v>65.78</v>
+      </c>
+      <c r="I8" s="8">
+        <v>74.88</v>
+      </c>
+      <c r="J8" s="8">
+        <v>83.99</v>
+      </c>
+      <c r="K8" s="8">
+        <v>105.33</v>
+      </c>
+      <c r="M8" s="9">
+        <v>4</v>
+      </c>
+      <c r="N8" s="8">
+        <v>126.67</v>
+      </c>
+      <c r="O8" s="8">
+        <v>175.53</v>
+      </c>
+      <c r="P8" s="8">
+        <v>224.39</v>
+      </c>
+      <c r="Q8" s="8">
+        <v>273.24</v>
+      </c>
+      <c r="R8" s="8">
+        <v>322.10000000000002</v>
+      </c>
+      <c r="S8" s="8">
+        <v>538.05999999999995</v>
+      </c>
+      <c r="T8" s="8">
+        <v>754.03</v>
+      </c>
+      <c r="U8" s="8">
+        <v>970</v>
+      </c>
+      <c r="V8" s="8">
+        <v>1185.97</v>
+      </c>
+      <c r="W8" s="8">
+        <v>1401.94</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A9" s="5">
+        <v>5</v>
+      </c>
+      <c r="B9" s="8">
+        <v>15.91</v>
+      </c>
+      <c r="C9" s="8">
+        <v>28.5</v>
+      </c>
+      <c r="D9" s="8">
+        <v>41.09</v>
+      </c>
+      <c r="E9" s="8">
+        <v>47.94</v>
+      </c>
+      <c r="F9" s="8">
+        <v>54.79</v>
+      </c>
+      <c r="G9" s="8">
+        <v>61.64</v>
+      </c>
+      <c r="H9" s="8">
+        <v>70.760000000000005</v>
+      </c>
+      <c r="I9" s="8">
+        <v>79.87</v>
+      </c>
+      <c r="J9" s="8">
+        <v>88.99</v>
+      </c>
+      <c r="K9" s="8">
+        <v>107.83</v>
+      </c>
+      <c r="M9" s="9">
+        <v>5</v>
+      </c>
+      <c r="N9" s="8">
+        <v>126.67</v>
+      </c>
+      <c r="O9" s="8">
+        <v>175.53</v>
+      </c>
+      <c r="P9" s="8">
+        <v>224.39</v>
+      </c>
+      <c r="Q9" s="8">
+        <v>273.24</v>
+      </c>
+      <c r="R9" s="8">
+        <v>322.10000000000002</v>
+      </c>
+      <c r="S9" s="8">
+        <v>538.05999999999995</v>
+      </c>
+      <c r="T9" s="8">
+        <v>754.03</v>
+      </c>
+      <c r="U9" s="8">
+        <v>970</v>
+      </c>
+      <c r="V9" s="8">
+        <v>1185.97</v>
+      </c>
+      <c r="W9" s="8">
+        <v>1401.94</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A10" s="5">
+        <v>6</v>
+      </c>
+      <c r="B10" s="8">
+        <v>17.850000000000001</v>
+      </c>
+      <c r="C10" s="8">
+        <v>31.8</v>
+      </c>
+      <c r="D10" s="8">
+        <v>45.75</v>
+      </c>
+      <c r="E10" s="8">
+        <v>52.7</v>
+      </c>
+      <c r="F10" s="8">
+        <v>59.65</v>
+      </c>
+      <c r="G10" s="8">
+        <v>66.599999999999994</v>
+      </c>
+      <c r="H10" s="8">
+        <v>75.73</v>
+      </c>
+      <c r="I10" s="8">
+        <v>84.86</v>
+      </c>
+      <c r="J10" s="8">
+        <v>93.99</v>
+      </c>
+      <c r="K10" s="8">
+        <v>110.33</v>
+      </c>
+      <c r="M10" s="9">
+        <v>6</v>
+      </c>
+      <c r="N10" s="8">
+        <v>126.67</v>
+      </c>
+      <c r="O10" s="8">
+        <v>175.53</v>
+      </c>
+      <c r="P10" s="8">
+        <v>224.39</v>
+      </c>
+      <c r="Q10" s="8">
+        <v>273.24</v>
+      </c>
+      <c r="R10" s="8">
+        <v>322.10000000000002</v>
+      </c>
+      <c r="S10" s="8">
+        <v>538.05999999999995</v>
+      </c>
+      <c r="T10" s="8">
+        <v>754.03</v>
+      </c>
+      <c r="U10" s="8">
+        <v>970</v>
+      </c>
+      <c r="V10" s="8">
+        <v>1185.97</v>
+      </c>
+      <c r="W10" s="8">
+        <v>1401.94</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A11" s="5">
+        <v>7</v>
+      </c>
+      <c r="B11" s="8">
+        <v>21.08</v>
+      </c>
+      <c r="C11" s="8">
+        <v>35.65</v>
+      </c>
+      <c r="D11" s="8">
+        <v>50.21</v>
+      </c>
+      <c r="E11" s="8">
+        <v>57.08</v>
+      </c>
+      <c r="F11" s="8">
+        <v>63.96</v>
+      </c>
+      <c r="G11" s="8">
+        <v>70.83</v>
+      </c>
+      <c r="H11" s="8">
+        <v>80.16</v>
+      </c>
+      <c r="I11" s="8">
+        <v>89.48</v>
+      </c>
+      <c r="J11" s="8">
+        <v>98.81</v>
+      </c>
+      <c r="K11" s="8">
+        <v>112.74</v>
+      </c>
+      <c r="M11" s="9">
+        <v>7</v>
+      </c>
+      <c r="N11" s="8">
+        <v>126.67</v>
+      </c>
+      <c r="O11" s="8">
+        <v>175.53</v>
+      </c>
+      <c r="P11" s="8">
+        <v>224.39</v>
+      </c>
+      <c r="Q11" s="8">
+        <v>273.24</v>
+      </c>
+      <c r="R11" s="8">
+        <v>322.10000000000002</v>
+      </c>
+      <c r="S11" s="8">
+        <v>538.05999999999995</v>
+      </c>
+      <c r="T11" s="8">
+        <v>754.03</v>
+      </c>
+      <c r="U11" s="8">
+        <v>970</v>
+      </c>
+      <c r="V11" s="8">
+        <v>1185.97</v>
+      </c>
+      <c r="W11" s="8">
+        <v>1401.94</v>
+      </c>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A12" s="5">
+        <v>8</v>
+      </c>
+      <c r="B12" s="8">
+        <v>24.31</v>
+      </c>
+      <c r="C12" s="8">
+        <v>39.49</v>
+      </c>
+      <c r="D12" s="8">
+        <v>54.67</v>
+      </c>
+      <c r="E12" s="8">
+        <v>61.47</v>
+      </c>
+      <c r="F12" s="8">
+        <v>68.27</v>
+      </c>
+      <c r="G12" s="8">
+        <v>75.069999999999993</v>
+      </c>
+      <c r="H12" s="8">
+        <v>84.58</v>
+      </c>
+      <c r="I12" s="8">
+        <v>94.1</v>
+      </c>
+      <c r="J12" s="8">
+        <v>103.62</v>
+      </c>
+      <c r="K12" s="8">
+        <v>115.15</v>
+      </c>
+      <c r="M12" s="9">
+        <v>8</v>
+      </c>
+      <c r="N12" s="8">
+        <v>126.67</v>
+      </c>
+      <c r="O12" s="8">
+        <v>175.53</v>
+      </c>
+      <c r="P12" s="8">
+        <v>224.39</v>
+      </c>
+      <c r="Q12" s="8">
+        <v>273.24</v>
+      </c>
+      <c r="R12" s="8">
+        <v>322.10000000000002</v>
+      </c>
+      <c r="S12" s="8">
+        <v>538.05999999999995</v>
+      </c>
+      <c r="T12" s="8">
+        <v>754.03</v>
+      </c>
+      <c r="U12" s="8">
+        <v>970</v>
+      </c>
+      <c r="V12" s="8">
+        <v>1185.97</v>
+      </c>
+      <c r="W12" s="8">
+        <v>1401.94</v>
+      </c>
+    </row>
+    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A13" s="5">
+        <v>9</v>
+      </c>
+      <c r="B13" s="8">
+        <v>27.53</v>
+      </c>
+      <c r="C13" s="8">
+        <v>43.33</v>
+      </c>
+      <c r="D13" s="8">
+        <v>59.13</v>
+      </c>
+      <c r="E13" s="8">
+        <v>65.849999999999994</v>
+      </c>
+      <c r="F13" s="8">
+        <v>72.569999999999993</v>
+      </c>
+      <c r="G13" s="8">
+        <v>79.3</v>
+      </c>
+      <c r="H13" s="8">
+        <v>89.01</v>
+      </c>
+      <c r="I13" s="8">
+        <v>98.72</v>
+      </c>
+      <c r="J13" s="8">
+        <v>108.43</v>
+      </c>
+      <c r="K13" s="8">
+        <v>117.55</v>
+      </c>
+      <c r="M13" s="9">
+        <v>9</v>
+      </c>
+      <c r="N13" s="8">
+        <v>126.67</v>
+      </c>
+      <c r="O13" s="8">
+        <v>175.53</v>
+      </c>
+      <c r="P13" s="8">
+        <v>224.39</v>
+      </c>
+      <c r="Q13" s="8">
+        <v>273.24</v>
+      </c>
+      <c r="R13" s="8">
+        <v>322.10000000000002</v>
+      </c>
+      <c r="S13" s="8">
+        <v>538.05999999999995</v>
+      </c>
+      <c r="T13" s="8">
+        <v>754.03</v>
+      </c>
+      <c r="U13" s="8">
+        <v>970</v>
+      </c>
+      <c r="V13" s="8">
+        <v>1185.97</v>
+      </c>
+      <c r="W13" s="8">
+        <v>1401.94</v>
+      </c>
+    </row>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A14" s="5">
+        <v>10</v>
+      </c>
+      <c r="B14" s="8">
+        <v>29.19</v>
+      </c>
+      <c r="C14" s="8">
+        <v>44.8</v>
+      </c>
+      <c r="D14" s="8">
+        <v>60.4</v>
+      </c>
+      <c r="E14" s="8">
+        <v>66.73</v>
+      </c>
+      <c r="F14" s="8">
+        <v>73.06</v>
+      </c>
+      <c r="G14" s="8">
+        <v>79.39</v>
+      </c>
+      <c r="H14" s="8">
+        <v>89.32</v>
+      </c>
+      <c r="I14" s="8">
+        <v>99.26</v>
+      </c>
+      <c r="J14" s="8">
+        <v>109.19</v>
+      </c>
+      <c r="K14" s="8">
+        <v>117.93</v>
+      </c>
+      <c r="M14" s="9">
+        <v>10</v>
+      </c>
+      <c r="N14" s="8">
+        <v>126.67</v>
+      </c>
+      <c r="O14" s="8">
+        <v>175.53</v>
+      </c>
+      <c r="P14" s="8">
+        <v>224.39</v>
+      </c>
+      <c r="Q14" s="8">
+        <v>273.24</v>
+      </c>
+      <c r="R14" s="8">
+        <v>322.10000000000002</v>
+      </c>
+      <c r="S14" s="8">
+        <v>538.05999999999995</v>
+      </c>
+      <c r="T14" s="8">
+        <v>754.03</v>
+      </c>
+      <c r="U14" s="8">
+        <v>970</v>
+      </c>
+      <c r="V14" s="8">
+        <v>1185.97</v>
+      </c>
+      <c r="W14" s="8">
+        <v>1401.94</v>
+      </c>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A15" s="5">
+        <v>11</v>
+      </c>
+      <c r="B15" s="8">
+        <v>30.85</v>
+      </c>
+      <c r="C15" s="8">
+        <v>46.26</v>
+      </c>
+      <c r="D15" s="8">
+        <v>61.68</v>
+      </c>
+      <c r="E15" s="8">
+        <v>67.61</v>
+      </c>
+      <c r="F15" s="8">
+        <v>73.55</v>
+      </c>
+      <c r="G15" s="8">
+        <v>79.48</v>
+      </c>
+      <c r="H15" s="8">
+        <v>89.64</v>
+      </c>
+      <c r="I15" s="8">
+        <v>99.8</v>
+      </c>
+      <c r="J15" s="8">
+        <v>109.95</v>
+      </c>
+      <c r="K15" s="8">
+        <v>118.31</v>
+      </c>
+      <c r="M15" s="9">
+        <v>11</v>
+      </c>
+      <c r="N15" s="8">
+        <v>126.67</v>
+      </c>
+      <c r="O15" s="8">
+        <v>175.53</v>
+      </c>
+      <c r="P15" s="8">
+        <v>224.39</v>
+      </c>
+      <c r="Q15" s="8">
+        <v>273.24</v>
+      </c>
+      <c r="R15" s="8">
+        <v>322.10000000000002</v>
+      </c>
+      <c r="S15" s="8">
+        <v>538.05999999999995</v>
+      </c>
+      <c r="T15" s="8">
+        <v>754.03</v>
+      </c>
+      <c r="U15" s="8">
+        <v>970</v>
+      </c>
+      <c r="V15" s="8">
+        <v>1185.97</v>
+      </c>
+      <c r="W15" s="8">
+        <v>1401.94</v>
+      </c>
+    </row>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A16" s="5">
+        <v>12</v>
+      </c>
+      <c r="B16" s="8">
+        <v>32.51</v>
+      </c>
+      <c r="C16" s="8">
+        <v>47.73</v>
+      </c>
+      <c r="D16" s="8">
+        <v>62.95</v>
+      </c>
+      <c r="E16" s="8">
+        <v>68.489999999999995</v>
+      </c>
+      <c r="F16" s="8">
+        <v>74.03</v>
+      </c>
+      <c r="G16" s="8">
+        <v>79.569999999999993</v>
+      </c>
+      <c r="H16" s="8">
+        <v>89.95</v>
+      </c>
+      <c r="I16" s="8">
+        <v>100.33</v>
+      </c>
+      <c r="J16" s="8">
+        <v>110.72</v>
+      </c>
+      <c r="K16" s="8">
+        <v>118.69</v>
+      </c>
+      <c r="M16" s="9">
+        <v>12</v>
+      </c>
+      <c r="N16" s="8">
+        <v>126.67</v>
+      </c>
+      <c r="O16" s="8">
+        <v>175.53</v>
+      </c>
+      <c r="P16" s="8">
+        <v>224.39</v>
+      </c>
+      <c r="Q16" s="8">
+        <v>273.24</v>
+      </c>
+      <c r="R16" s="8">
+        <v>322.10000000000002</v>
+      </c>
+      <c r="S16" s="8">
+        <v>538.05999999999995</v>
+      </c>
+      <c r="T16" s="8">
+        <v>754.03</v>
+      </c>
+      <c r="U16" s="8">
+        <v>970</v>
+      </c>
+      <c r="V16" s="8">
+        <v>1185.97</v>
+      </c>
+      <c r="W16" s="8">
+        <v>1401.94</v>
+      </c>
+    </row>
+    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A17" s="5">
+        <v>13</v>
+      </c>
+      <c r="B17" s="8">
+        <v>34.159999999999997</v>
+      </c>
+      <c r="C17" s="8">
+        <v>49.19</v>
+      </c>
+      <c r="D17" s="8">
+        <v>64.23</v>
+      </c>
+      <c r="E17" s="8">
+        <v>69.37</v>
+      </c>
+      <c r="F17" s="8">
+        <v>74.52</v>
+      </c>
+      <c r="G17" s="8">
+        <v>79.66</v>
+      </c>
+      <c r="H17" s="8">
+        <v>90.27</v>
+      </c>
+      <c r="I17" s="8">
+        <v>100.87</v>
+      </c>
+      <c r="J17" s="8">
+        <v>111.48</v>
+      </c>
+      <c r="K17" s="8">
+        <v>119.08</v>
+      </c>
+      <c r="M17" s="9">
+        <v>13</v>
+      </c>
+      <c r="N17" s="8">
+        <v>126.67</v>
+      </c>
+      <c r="O17" s="8">
+        <v>175.53</v>
+      </c>
+      <c r="P17" s="8">
+        <v>224.39</v>
+      </c>
+      <c r="Q17" s="8">
+        <v>273.24</v>
+      </c>
+      <c r="R17" s="8">
+        <v>322.10000000000002</v>
+      </c>
+      <c r="S17" s="8">
+        <v>538.05999999999995</v>
+      </c>
+      <c r="T17" s="8">
+        <v>754.03</v>
+      </c>
+      <c r="U17" s="8">
+        <v>970</v>
+      </c>
+      <c r="V17" s="8">
+        <v>1185.97</v>
+      </c>
+      <c r="W17" s="8">
+        <v>1401.94</v>
+      </c>
+    </row>
+    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A18" s="5">
+        <v>14</v>
+      </c>
+      <c r="B18" s="8">
+        <v>35.82</v>
+      </c>
+      <c r="C18" s="8">
+        <v>50.66</v>
+      </c>
+      <c r="D18" s="8">
+        <v>65.5</v>
+      </c>
+      <c r="E18" s="8">
+        <v>70.25</v>
+      </c>
+      <c r="F18" s="8">
+        <v>75</v>
+      </c>
+      <c r="G18" s="8">
+        <v>79.760000000000005</v>
+      </c>
+      <c r="H18" s="8">
+        <v>90.58</v>
+      </c>
+      <c r="I18" s="8">
+        <v>101.41</v>
+      </c>
+      <c r="J18" s="8">
+        <v>112.24</v>
+      </c>
+      <c r="K18" s="8">
+        <v>119.46</v>
+      </c>
+      <c r="M18" s="9">
+        <v>14</v>
+      </c>
+      <c r="N18" s="8">
+        <v>126.67</v>
+      </c>
+      <c r="O18" s="8">
+        <v>175.53</v>
+      </c>
+      <c r="P18" s="8">
+        <v>224.39</v>
+      </c>
+      <c r="Q18" s="8">
+        <v>273.24</v>
+      </c>
+      <c r="R18" s="8">
+        <v>322.10000000000002</v>
+      </c>
+      <c r="S18" s="8">
+        <v>538.05999999999995</v>
+      </c>
+      <c r="T18" s="8">
+        <v>754.03</v>
+      </c>
+      <c r="U18" s="8">
+        <v>970</v>
+      </c>
+      <c r="V18" s="8">
+        <v>1185.97</v>
+      </c>
+      <c r="W18" s="8">
+        <v>1401.94</v>
+      </c>
+    </row>
+    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A19" s="5">
+        <v>15</v>
+      </c>
+      <c r="B19" s="8">
+        <v>37.479999999999997</v>
+      </c>
+      <c r="C19" s="8">
+        <v>52.13</v>
+      </c>
+      <c r="D19" s="8">
+        <v>66.78</v>
+      </c>
+      <c r="E19" s="8">
+        <v>71.13</v>
+      </c>
+      <c r="F19" s="8">
+        <v>75.489999999999995</v>
+      </c>
+      <c r="G19" s="8">
+        <v>79.849999999999994</v>
+      </c>
+      <c r="H19" s="8">
+        <v>90.9</v>
+      </c>
+      <c r="I19" s="8">
+        <v>101.95</v>
+      </c>
+      <c r="J19" s="8">
+        <v>113</v>
+      </c>
+      <c r="K19" s="8">
+        <v>119.84</v>
+      </c>
+      <c r="M19" s="9">
+        <v>15</v>
+      </c>
+      <c r="N19" s="8">
+        <v>126.67</v>
+      </c>
+      <c r="O19" s="8">
+        <v>175.53</v>
+      </c>
+      <c r="P19" s="8">
+        <v>224.39</v>
+      </c>
+      <c r="Q19" s="8">
+        <v>273.24</v>
+      </c>
+      <c r="R19" s="8">
+        <v>322.10000000000002</v>
+      </c>
+      <c r="S19" s="8">
+        <v>538.05999999999995</v>
+      </c>
+      <c r="T19" s="8">
+        <v>754.03</v>
+      </c>
+      <c r="U19" s="8">
+        <v>970</v>
+      </c>
+      <c r="V19" s="8">
+        <v>1185.97</v>
+      </c>
+      <c r="W19" s="8">
+        <v>1401.94</v>
+      </c>
+    </row>
+    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A20" s="5">
+        <v>16</v>
+      </c>
+      <c r="B20" s="8">
+        <v>39.130000000000003</v>
+      </c>
+      <c r="C20" s="8">
+        <v>53.59</v>
+      </c>
+      <c r="D20" s="8">
+        <v>68.05</v>
+      </c>
+      <c r="E20" s="8">
+        <v>72.010000000000005</v>
+      </c>
+      <c r="F20" s="8">
+        <v>75.98</v>
+      </c>
+      <c r="G20" s="8">
+        <v>79.94</v>
+      </c>
+      <c r="H20" s="8">
+        <v>91.21</v>
+      </c>
+      <c r="I20" s="8">
+        <v>102.49</v>
+      </c>
+      <c r="J20" s="8">
+        <v>113.76</v>
+      </c>
+      <c r="K20" s="8">
+        <v>120.22</v>
+      </c>
+      <c r="M20" s="9">
+        <v>16</v>
+      </c>
+      <c r="N20" s="8">
+        <v>126.67</v>
+      </c>
+      <c r="O20" s="8">
+        <v>175.53</v>
+      </c>
+      <c r="P20" s="8">
+        <v>224.39</v>
+      </c>
+      <c r="Q20" s="8">
+        <v>273.24</v>
+      </c>
+      <c r="R20" s="8">
+        <v>322.10000000000002</v>
+      </c>
+      <c r="S20" s="8">
+        <v>538.05999999999995</v>
+      </c>
+      <c r="T20" s="8">
+        <v>754.03</v>
+      </c>
+      <c r="U20" s="8">
+        <v>970</v>
+      </c>
+      <c r="V20" s="8">
+        <v>1185.97</v>
+      </c>
+      <c r="W20" s="8">
+        <v>1401.94</v>
+      </c>
+    </row>
+    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A21" s="5">
+        <v>17</v>
+      </c>
+      <c r="B21" s="8">
+        <v>40.79</v>
+      </c>
+      <c r="C21" s="8">
+        <v>55.06</v>
+      </c>
+      <c r="D21" s="8">
+        <v>69.319999999999993</v>
+      </c>
+      <c r="E21" s="8">
+        <v>72.89</v>
+      </c>
+      <c r="F21" s="8">
+        <v>76.459999999999994</v>
+      </c>
+      <c r="G21" s="8">
+        <v>80.03</v>
+      </c>
+      <c r="H21" s="8">
+        <v>91.53</v>
+      </c>
+      <c r="I21" s="8">
+        <v>103.02</v>
+      </c>
+      <c r="J21" s="8">
+        <v>114.52</v>
+      </c>
+      <c r="K21" s="8">
+        <v>120.6</v>
+      </c>
+      <c r="M21" s="9">
+        <v>17</v>
+      </c>
+      <c r="N21" s="8">
+        <v>126.67</v>
+      </c>
+      <c r="O21" s="8">
+        <v>175.53</v>
+      </c>
+      <c r="P21" s="8">
+        <v>224.39</v>
+      </c>
+      <c r="Q21" s="8">
+        <v>273.24</v>
+      </c>
+      <c r="R21" s="8">
+        <v>322.10000000000002</v>
+      </c>
+      <c r="S21" s="8">
+        <v>538.05999999999995</v>
+      </c>
+      <c r="T21" s="8">
+        <v>754.03</v>
+      </c>
+      <c r="U21" s="8">
+        <v>970</v>
+      </c>
+      <c r="V21" s="8">
+        <v>1185.97</v>
+      </c>
+      <c r="W21" s="8">
+        <v>1401.94</v>
+      </c>
+    </row>
+    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A22" s="5">
+        <v>18</v>
+      </c>
+      <c r="B22" s="8">
+        <v>42.45</v>
+      </c>
+      <c r="C22" s="8">
+        <v>56.52</v>
+      </c>
+      <c r="D22" s="8">
+        <v>70.599999999999994</v>
+      </c>
+      <c r="E22" s="8">
+        <v>73.77</v>
+      </c>
+      <c r="F22" s="8">
+        <v>76.95</v>
+      </c>
+      <c r="G22" s="8">
+        <v>80.12</v>
+      </c>
+      <c r="H22" s="8">
+        <v>91.84</v>
+      </c>
+      <c r="I22" s="8">
+        <v>103.56</v>
+      </c>
+      <c r="J22" s="8">
+        <v>115.28</v>
+      </c>
+      <c r="K22" s="8">
+        <v>120.98</v>
+      </c>
+      <c r="M22" s="9">
+        <v>18</v>
+      </c>
+      <c r="N22" s="8">
+        <v>126.67</v>
+      </c>
+      <c r="O22" s="8">
+        <v>175.53</v>
+      </c>
+      <c r="P22" s="8">
+        <v>224.39</v>
+      </c>
+      <c r="Q22" s="8">
+        <v>273.24</v>
+      </c>
+      <c r="R22" s="8">
+        <v>322.10000000000002</v>
+      </c>
+      <c r="S22" s="8">
+        <v>538.05999999999995</v>
+      </c>
+      <c r="T22" s="8">
+        <v>754.03</v>
+      </c>
+      <c r="U22" s="8">
+        <v>970</v>
+      </c>
+      <c r="V22" s="8">
+        <v>1185.97</v>
+      </c>
+      <c r="W22" s="8">
+        <v>1401.94</v>
+      </c>
+    </row>
+    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A23" s="5">
+        <v>19</v>
+      </c>
+      <c r="B23" s="8">
+        <v>44.1</v>
+      </c>
+      <c r="C23" s="8">
+        <v>57.99</v>
+      </c>
+      <c r="D23" s="8">
+        <v>71.87</v>
+      </c>
+      <c r="E23" s="8">
+        <v>74.650000000000006</v>
+      </c>
+      <c r="F23" s="8">
+        <v>77.430000000000007</v>
+      </c>
+      <c r="G23" s="8">
+        <v>80.209999999999994</v>
+      </c>
+      <c r="H23" s="8">
+        <v>92.16</v>
+      </c>
+      <c r="I23" s="8">
+        <v>104.1</v>
+      </c>
+      <c r="J23" s="8">
+        <v>116.04</v>
+      </c>
+      <c r="K23" s="8">
+        <v>121.36</v>
+      </c>
+      <c r="M23" s="9">
+        <v>19</v>
+      </c>
+      <c r="N23" s="8">
+        <v>126.67</v>
+      </c>
+      <c r="O23" s="8">
+        <v>175.53</v>
+      </c>
+      <c r="P23" s="8">
+        <v>224.39</v>
+      </c>
+      <c r="Q23" s="8">
+        <v>273.24</v>
+      </c>
+      <c r="R23" s="8">
+        <v>322.10000000000002</v>
+      </c>
+      <c r="S23" s="8">
+        <v>538.05999999999995</v>
+      </c>
+      <c r="T23" s="8">
+        <v>754.03</v>
+      </c>
+      <c r="U23" s="8">
+        <v>970</v>
+      </c>
+      <c r="V23" s="8">
+        <v>1185.97</v>
+      </c>
+      <c r="W23" s="8">
+        <v>1401.94</v>
+      </c>
+    </row>
+    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A24" s="5">
+        <v>20</v>
+      </c>
+      <c r="B24" s="8">
+        <v>45.76</v>
+      </c>
+      <c r="C24" s="8">
+        <v>59.45</v>
+      </c>
+      <c r="D24" s="8">
+        <v>73.150000000000006</v>
+      </c>
+      <c r="E24" s="8">
+        <v>75.53</v>
+      </c>
+      <c r="F24" s="8">
+        <v>77.92</v>
+      </c>
+      <c r="G24" s="8">
+        <v>80.31</v>
+      </c>
+      <c r="H24" s="8">
+        <v>92.47</v>
+      </c>
+      <c r="I24" s="8">
+        <v>104.64</v>
+      </c>
+      <c r="J24" s="8">
+        <v>116.8</v>
+      </c>
+      <c r="K24" s="8">
+        <v>121.74</v>
+      </c>
+      <c r="M24" s="9">
+        <v>20</v>
+      </c>
+      <c r="N24" s="8">
+        <v>126.67</v>
+      </c>
+      <c r="O24" s="8">
+        <v>175.53</v>
+      </c>
+      <c r="P24" s="8">
+        <v>224.39</v>
+      </c>
+      <c r="Q24" s="8">
+        <v>273.24</v>
+      </c>
+      <c r="R24" s="8">
+        <v>322.10000000000002</v>
+      </c>
+      <c r="S24" s="8">
+        <v>538.05999999999995</v>
+      </c>
+      <c r="T24" s="8">
+        <v>754.03</v>
+      </c>
+      <c r="U24" s="8">
+        <v>970</v>
+      </c>
+      <c r="V24" s="8">
+        <v>1185.97</v>
+      </c>
+      <c r="W24" s="8">
+        <v>1401.94</v>
+      </c>
+    </row>
+    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A25" s="5">
+        <v>21</v>
+      </c>
+      <c r="B25" s="8">
+        <v>47.42</v>
+      </c>
+      <c r="C25" s="8">
+        <v>60.92</v>
+      </c>
+      <c r="D25" s="8">
+        <v>74.42</v>
+      </c>
+      <c r="E25" s="8">
+        <v>76.42</v>
+      </c>
+      <c r="F25" s="8">
+        <v>78.41</v>
+      </c>
+      <c r="G25" s="8">
+        <v>80.400000000000006</v>
+      </c>
+      <c r="H25" s="8">
+        <v>92.79</v>
+      </c>
+      <c r="I25" s="8">
+        <v>105.17</v>
+      </c>
+      <c r="J25" s="8">
+        <v>117.56</v>
+      </c>
+      <c r="K25" s="8">
+        <v>122.12</v>
+      </c>
+      <c r="M25" s="9">
+        <v>21</v>
+      </c>
+      <c r="N25" s="8">
+        <v>126.67</v>
+      </c>
+      <c r="O25" s="8">
+        <v>175.53</v>
+      </c>
+      <c r="P25" s="8">
+        <v>224.39</v>
+      </c>
+      <c r="Q25" s="8">
+        <v>273.24</v>
+      </c>
+      <c r="R25" s="8">
+        <v>322.10000000000002</v>
+      </c>
+      <c r="S25" s="8">
+        <v>538.05999999999995</v>
+      </c>
+      <c r="T25" s="8">
+        <v>754.03</v>
+      </c>
+      <c r="U25" s="8">
+        <v>970</v>
+      </c>
+      <c r="V25" s="8">
+        <v>1185.97</v>
+      </c>
+      <c r="W25" s="8">
+        <v>1401.94</v>
+      </c>
+    </row>
+    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A26" s="5">
+        <v>22</v>
+      </c>
+      <c r="B26" s="8">
+        <v>49.07</v>
+      </c>
+      <c r="C26" s="8">
+        <v>62.39</v>
+      </c>
+      <c r="D26" s="8">
+        <v>75.7</v>
+      </c>
+      <c r="E26" s="8">
+        <v>77.3</v>
+      </c>
+      <c r="F26" s="8">
+        <v>78.89</v>
+      </c>
+      <c r="G26" s="8">
+        <v>80.489999999999995</v>
+      </c>
+      <c r="H26" s="8">
+        <v>93.1</v>
+      </c>
+      <c r="I26" s="8">
+        <v>105.71</v>
+      </c>
+      <c r="J26" s="8">
+        <v>118.32</v>
+      </c>
+      <c r="K26" s="8">
+        <v>122.5</v>
+      </c>
+      <c r="M26" s="9">
+        <v>22</v>
+      </c>
+      <c r="N26" s="8">
+        <v>126.67</v>
+      </c>
+      <c r="O26" s="8">
+        <v>175.53</v>
+      </c>
+      <c r="P26" s="8">
+        <v>224.39</v>
+      </c>
+      <c r="Q26" s="8">
+        <v>273.24</v>
+      </c>
+      <c r="R26" s="8">
+        <v>322.10000000000002</v>
+      </c>
+      <c r="S26" s="8">
+        <v>538.05999999999995</v>
+      </c>
+      <c r="T26" s="8">
+        <v>754.03</v>
+      </c>
+      <c r="U26" s="8">
+        <v>970</v>
+      </c>
+      <c r="V26" s="8">
+        <v>1185.97</v>
+      </c>
+      <c r="W26" s="8">
+        <v>1401.94</v>
+      </c>
+    </row>
+    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A27" s="5">
+        <v>23</v>
+      </c>
+      <c r="B27" s="8">
+        <v>50.73</v>
+      </c>
+      <c r="C27" s="8">
+        <v>63.85</v>
+      </c>
+      <c r="D27" s="8">
+        <v>76.97</v>
+      </c>
+      <c r="E27" s="8">
+        <v>78.180000000000007</v>
+      </c>
+      <c r="F27" s="8">
+        <v>79.38</v>
+      </c>
+      <c r="G27" s="8">
+        <v>80.58</v>
+      </c>
+      <c r="H27" s="8">
+        <v>93.41</v>
+      </c>
+      <c r="I27" s="8">
+        <v>106.25</v>
+      </c>
+      <c r="J27" s="8">
+        <v>119.08</v>
+      </c>
+      <c r="K27" s="8">
+        <v>122.88</v>
+      </c>
+      <c r="M27" s="9">
+        <v>23</v>
+      </c>
+      <c r="N27" s="8">
+        <v>126.67</v>
+      </c>
+      <c r="O27" s="8">
+        <v>175.53</v>
+      </c>
+      <c r="P27" s="8">
+        <v>224.39</v>
+      </c>
+      <c r="Q27" s="8">
+        <v>273.24</v>
+      </c>
+      <c r="R27" s="8">
+        <v>322.10000000000002</v>
+      </c>
+      <c r="S27" s="8">
+        <v>538.05999999999995</v>
+      </c>
+      <c r="T27" s="8">
+        <v>754.03</v>
+      </c>
+      <c r="U27" s="8">
+        <v>970</v>
+      </c>
+      <c r="V27" s="8">
+        <v>1185.97</v>
+      </c>
+      <c r="W27" s="8">
+        <v>1401.94</v>
+      </c>
+    </row>
+    <row r="28" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A28" s="5">
+        <v>24</v>
+      </c>
+      <c r="B28" s="8">
+        <v>52.39</v>
+      </c>
+      <c r="C28" s="8">
+        <v>65.319999999999993</v>
+      </c>
+      <c r="D28" s="8">
+        <v>78.25</v>
+      </c>
+      <c r="E28" s="8">
+        <v>79.06</v>
+      </c>
+      <c r="F28" s="8">
+        <v>79.86</v>
+      </c>
+      <c r="G28" s="8">
+        <v>80.67</v>
+      </c>
+      <c r="H28" s="8">
+        <v>93.73</v>
+      </c>
+      <c r="I28" s="8">
+        <v>106.79</v>
+      </c>
+      <c r="J28" s="8">
+        <v>119.84</v>
+      </c>
+      <c r="K28" s="8">
+        <v>123.26</v>
+      </c>
+      <c r="M28" s="9">
+        <v>24</v>
+      </c>
+      <c r="N28" s="8">
+        <v>126.67</v>
+      </c>
+      <c r="O28" s="8">
+        <v>175.53</v>
+      </c>
+      <c r="P28" s="8">
+        <v>224.39</v>
+      </c>
+      <c r="Q28" s="8">
+        <v>273.24</v>
+      </c>
+      <c r="R28" s="8">
+        <v>322.10000000000002</v>
+      </c>
+      <c r="S28" s="8">
+        <v>538.05999999999995</v>
+      </c>
+      <c r="T28" s="8">
+        <v>754.03</v>
+      </c>
+      <c r="U28" s="8">
+        <v>970</v>
+      </c>
+      <c r="V28" s="8">
+        <v>1185.97</v>
+      </c>
+      <c r="W28" s="8">
+        <v>1401.94</v>
+      </c>
+    </row>
+    <row r="29" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A29" s="5">
+        <v>25</v>
+      </c>
+      <c r="B29" s="8">
+        <v>54.04</v>
+      </c>
+      <c r="C29" s="8">
+        <v>66.78</v>
+      </c>
+      <c r="D29" s="8">
+        <v>79.52</v>
+      </c>
+      <c r="E29" s="8">
+        <v>79.94</v>
+      </c>
+      <c r="F29" s="8">
+        <v>80.349999999999994</v>
+      </c>
+      <c r="G29" s="8">
+        <v>80.760000000000005</v>
+      </c>
+      <c r="H29" s="8">
+        <v>94.04</v>
+      </c>
+      <c r="I29" s="8">
+        <v>107.32</v>
+      </c>
+      <c r="J29" s="8">
+        <v>120.6</v>
+      </c>
+      <c r="K29" s="8">
+        <v>123.64</v>
+      </c>
+      <c r="M29" s="9">
+        <v>25</v>
+      </c>
+      <c r="N29" s="8">
+        <v>126.67</v>
+      </c>
+      <c r="O29" s="8">
+        <v>175.53</v>
+      </c>
+      <c r="P29" s="8">
+        <v>224.39</v>
+      </c>
+      <c r="Q29" s="8">
+        <v>273.24</v>
+      </c>
+      <c r="R29" s="8">
+        <v>322.10000000000002</v>
+      </c>
+      <c r="S29" s="8">
+        <v>538.05999999999995</v>
+      </c>
+      <c r="T29" s="8">
+        <v>754.03</v>
+      </c>
+      <c r="U29" s="8">
+        <v>970</v>
+      </c>
+      <c r="V29" s="8">
+        <v>1185.97</v>
+      </c>
+      <c r="W29" s="8">
+        <v>1401.94</v>
+      </c>
+    </row>
+    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A30" s="5">
+        <v>26</v>
+      </c>
+      <c r="B30" s="8">
+        <v>55.7</v>
+      </c>
+      <c r="C30" s="8">
+        <v>68.25</v>
+      </c>
+      <c r="D30" s="8">
+        <v>80.8</v>
+      </c>
+      <c r="E30" s="8">
+        <v>80.819999999999993</v>
+      </c>
+      <c r="F30" s="8">
+        <v>80.84</v>
+      </c>
+      <c r="G30" s="8">
+        <v>80.86</v>
+      </c>
+      <c r="H30" s="8">
+        <v>94.36</v>
+      </c>
+      <c r="I30" s="8">
+        <v>107.86</v>
+      </c>
+      <c r="J30" s="8">
+        <v>121.36</v>
+      </c>
+      <c r="K30" s="8">
+        <v>124.02</v>
+      </c>
+      <c r="M30" s="9">
+        <v>26</v>
+      </c>
+      <c r="N30" s="8">
+        <v>126.67</v>
+      </c>
+      <c r="O30" s="8">
+        <v>175.53</v>
+      </c>
+      <c r="P30" s="8">
+        <v>224.39</v>
+      </c>
+      <c r="Q30" s="8">
+        <v>273.24</v>
+      </c>
+      <c r="R30" s="8">
+        <v>322.10000000000002</v>
+      </c>
+      <c r="S30" s="8">
+        <v>538.05999999999995</v>
+      </c>
+      <c r="T30" s="8">
+        <v>754.03</v>
+      </c>
+      <c r="U30" s="8">
+        <v>970</v>
+      </c>
+      <c r="V30" s="8">
+        <v>1185.97</v>
+      </c>
+      <c r="W30" s="8">
+        <v>1401.94</v>
+      </c>
+    </row>
+    <row r="31" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A31" s="5">
+        <v>27</v>
+      </c>
+      <c r="B31" s="8">
+        <v>57.36</v>
+      </c>
+      <c r="C31" s="8">
+        <v>69.72</v>
+      </c>
+      <c r="D31" s="8">
+        <v>82.07</v>
+      </c>
+      <c r="E31" s="8">
+        <v>81.7</v>
+      </c>
+      <c r="F31" s="8">
+        <v>81.319999999999993</v>
+      </c>
+      <c r="G31" s="8">
+        <v>80.95</v>
+      </c>
+      <c r="H31" s="8">
+        <v>94.67</v>
+      </c>
+      <c r="I31" s="8">
+        <v>108.4</v>
+      </c>
+      <c r="J31" s="8">
+        <v>122.13</v>
+      </c>
+      <c r="K31" s="8">
+        <v>124.4</v>
+      </c>
+      <c r="M31" s="9">
+        <v>27</v>
+      </c>
+      <c r="N31" s="8">
+        <v>126.67</v>
+      </c>
+      <c r="O31" s="8">
+        <v>175.53</v>
+      </c>
+      <c r="P31" s="8">
+        <v>224.39</v>
+      </c>
+      <c r="Q31" s="8">
+        <v>273.24</v>
+      </c>
+      <c r="R31" s="8">
+        <v>322.10000000000002</v>
+      </c>
+      <c r="S31" s="8">
+        <v>538.05999999999995</v>
+      </c>
+      <c r="T31" s="8">
+        <v>754.03</v>
+      </c>
+      <c r="U31" s="8">
+        <v>970</v>
+      </c>
+      <c r="V31" s="8">
+        <v>1185.97</v>
+      </c>
+      <c r="W31" s="8">
+        <v>1401.94</v>
+      </c>
+    </row>
+    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A32" s="5">
+        <v>28</v>
+      </c>
+      <c r="B32" s="8">
+        <v>59.02</v>
+      </c>
+      <c r="C32" s="8">
+        <v>71.180000000000007</v>
+      </c>
+      <c r="D32" s="8">
+        <v>83.35</v>
+      </c>
+      <c r="E32" s="8">
+        <v>82.58</v>
+      </c>
+      <c r="F32" s="8">
+        <v>81.81</v>
+      </c>
+      <c r="G32" s="8">
+        <v>81.040000000000006</v>
+      </c>
+      <c r="H32" s="8">
+        <v>94.99</v>
+      </c>
+      <c r="I32" s="8">
+        <v>108.94</v>
+      </c>
+      <c r="J32" s="8">
+        <v>122.89</v>
+      </c>
+      <c r="K32" s="8">
+        <v>124.78</v>
+      </c>
+      <c r="M32" s="9">
+        <v>28</v>
+      </c>
+      <c r="N32" s="8">
+        <v>126.67</v>
+      </c>
+      <c r="O32" s="8">
+        <v>175.53</v>
+      </c>
+      <c r="P32" s="8">
+        <v>224.39</v>
+      </c>
+      <c r="Q32" s="8">
+        <v>273.24</v>
+      </c>
+      <c r="R32" s="8">
+        <v>322.10000000000002</v>
+      </c>
+      <c r="S32" s="8">
+        <v>538.05999999999995</v>
+      </c>
+      <c r="T32" s="8">
+        <v>754.03</v>
+      </c>
+      <c r="U32" s="8">
+        <v>970</v>
+      </c>
+      <c r="V32" s="8">
+        <v>1185.97</v>
+      </c>
+      <c r="W32" s="8">
+        <v>1401.94</v>
+      </c>
+    </row>
+    <row r="33" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A33" s="5">
+        <v>29</v>
+      </c>
+      <c r="B33" s="8">
+        <v>60.67</v>
+      </c>
+      <c r="C33" s="8">
+        <v>72.650000000000006</v>
+      </c>
+      <c r="D33" s="8">
+        <v>84.62</v>
+      </c>
+      <c r="E33" s="8">
+        <v>83.46</v>
+      </c>
+      <c r="F33" s="8">
+        <v>82.29</v>
+      </c>
+      <c r="G33" s="8">
+        <v>81.13</v>
+      </c>
+      <c r="H33" s="8">
+        <v>95.3</v>
+      </c>
+      <c r="I33" s="8">
+        <v>109.47</v>
+      </c>
+      <c r="J33" s="8">
+        <v>123.65</v>
+      </c>
+      <c r="K33" s="8">
+        <v>125.16</v>
+      </c>
+      <c r="M33" s="9">
+        <v>29</v>
+      </c>
+      <c r="N33" s="8">
+        <v>126.67</v>
+      </c>
+      <c r="O33" s="8">
+        <v>175.53</v>
+      </c>
+      <c r="P33" s="8">
+        <v>224.39</v>
+      </c>
+      <c r="Q33" s="8">
+        <v>273.24</v>
+      </c>
+      <c r="R33" s="8">
+        <v>322.10000000000002</v>
+      </c>
+      <c r="S33" s="8">
+        <v>538.05999999999995</v>
+      </c>
+      <c r="T33" s="8">
+        <v>754.03</v>
+      </c>
+      <c r="U33" s="8">
+        <v>970</v>
+      </c>
+      <c r="V33" s="8">
+        <v>1185.97</v>
+      </c>
+      <c r="W33" s="8">
+        <v>1401.94</v>
+      </c>
+    </row>
+    <row r="34" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A34" s="5">
+        <v>30</v>
+      </c>
+      <c r="B34" s="8">
+        <v>62.33</v>
+      </c>
+      <c r="C34" s="8">
+        <v>74.11</v>
+      </c>
+      <c r="D34" s="8">
+        <v>85.9</v>
+      </c>
+      <c r="E34" s="8">
+        <v>84.34</v>
+      </c>
+      <c r="F34" s="8">
+        <v>82.78</v>
+      </c>
+      <c r="G34" s="8">
+        <v>81.22</v>
+      </c>
+      <c r="H34" s="8">
+        <v>95.62</v>
+      </c>
+      <c r="I34" s="8">
+        <v>110.01</v>
+      </c>
+      <c r="J34" s="8">
+        <v>124.41</v>
+      </c>
+      <c r="K34" s="8">
+        <v>125.54</v>
+      </c>
+      <c r="M34" s="9">
+        <v>30</v>
+      </c>
+      <c r="N34" s="8">
+        <v>126.67</v>
+      </c>
+      <c r="O34" s="8">
+        <v>175.53</v>
+      </c>
+      <c r="P34" s="8">
+        <v>224.39</v>
+      </c>
+      <c r="Q34" s="8">
+        <v>273.24</v>
+      </c>
+      <c r="R34" s="8">
+        <v>322.10000000000002</v>
+      </c>
+      <c r="S34" s="8">
+        <v>538.05999999999995</v>
+      </c>
+      <c r="T34" s="8">
+        <v>754.03</v>
+      </c>
+      <c r="U34" s="8">
+        <v>970</v>
+      </c>
+      <c r="V34" s="8">
+        <v>1185.97</v>
+      </c>
+      <c r="W34" s="8">
+        <v>1401.94</v>
+      </c>
+    </row>
+    <row r="35" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A35" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B35" s="8">
+        <v>36.525666666666666</v>
+      </c>
+      <c r="C35" s="8">
+        <v>49.985333333333337</v>
+      </c>
+      <c r="D35" s="8">
+        <v>63.443333333333342</v>
+      </c>
+      <c r="E35" s="8">
+        <v>67.010333333333335</v>
+      </c>
+      <c r="F35" s="8">
+        <v>70.576666666666654</v>
+      </c>
+      <c r="G35" s="8">
+        <v>74.143666666666661</v>
+      </c>
+      <c r="H35" s="8">
+        <v>85.25866666666667</v>
+      </c>
+      <c r="I35" s="8">
+        <v>96.373333333333363</v>
+      </c>
+      <c r="J35" s="8">
+        <v>107.48933333333335</v>
+      </c>
+      <c r="K35" s="8">
+        <v>117.08233333333332</v>
+      </c>
+      <c r="M35" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="N35" s="10">
+        <v>126.67000000000004</v>
+      </c>
+      <c r="O35" s="10">
+        <v>175.53000000000003</v>
+      </c>
+      <c r="P35" s="10">
+        <v>224.39000000000004</v>
+      </c>
+      <c r="Q35" s="10">
+        <v>273.23999999999984</v>
+      </c>
+      <c r="R35" s="10">
+        <v>322.10000000000019</v>
+      </c>
+      <c r="S35" s="10">
+        <v>538.0599999999996</v>
+      </c>
+      <c r="T35" s="10">
+        <v>754.02999999999986</v>
+      </c>
+      <c r="U35" s="10">
+        <v>970</v>
+      </c>
+      <c r="V35" s="10">
+        <v>1185.9700000000005</v>
+      </c>
+      <c r="W35" s="10">
+        <v>1401.94</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B2:K2"/>
+    <mergeCell ref="M1:W1"/>
+    <mergeCell ref="N2:W2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89E0380B-3232-4FC8-8E48-B6A283DD6300}">
   <dimension ref="A1:W35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3062,7 +5392,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3EEC94F4-4E93-438D-92F8-5C9CBA48C22A}">
   <dimension ref="A1:W35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5385,7 +7715,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{612EBB24-0E24-4D37-B6A7-8B4DA2BD1A51}">
   <dimension ref="A1:W35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -7708,7 +10038,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A2E7E46-B70B-4DB0-97AE-2138287FA00A}">
   <dimension ref="A1:W35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -10031,7 +12361,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D32525DC-1FAE-40FA-B3A1-6E6C0B62B72E}">
   <dimension ref="A1:W35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -12354,7 +14684,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <sheetPr codeName="Sheet9">
     <tabColor rgb="FFFFFF00"/>

</xml_diff>

<commit_message>
📊 Update NAIC content history - 2026-08-05
</commit_message>
<xml_diff>
--- a/docs/content_history/pbr-2026-vm20-table-f-g-current-spreads.xlsx
+++ b/docs/content_history/pbr-2026-vm20-table-f-g-current-spreads.xlsx
@@ -1,25 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\PBR\VM20_VM22_ProductSupport\PBR Production Web Data\Current Year\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AE96921-D258-4EBB-BD8B-D2333E983B4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CE8A278-3314-471C-B5CE-A5002E5EC884}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="795" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" tabRatio="795" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="June_2026" sheetId="29" r:id="rId1"/>
-    <sheet name="May_2026" sheetId="28" r:id="rId2"/>
-    <sheet name="April_2026" sheetId="27" r:id="rId3"/>
-    <sheet name="March_2026" sheetId="26" r:id="rId4"/>
-    <sheet name="February_2026" sheetId="25" r:id="rId5"/>
-    <sheet name="January_2026" sheetId="24" r:id="rId6"/>
-    <sheet name="LEGAL DISCLAIMER" sheetId="11" r:id="rId7"/>
+    <sheet name="July_2026" sheetId="30" r:id="rId1"/>
+    <sheet name="June_2026" sheetId="29" r:id="rId2"/>
+    <sheet name="May_2026" sheetId="28" r:id="rId3"/>
+    <sheet name="April_2026" sheetId="27" r:id="rId4"/>
+    <sheet name="March_2026" sheetId="26" r:id="rId5"/>
+    <sheet name="February_2026" sheetId="25" r:id="rId6"/>
+    <sheet name="January_2026" sheetId="24" r:id="rId7"/>
+    <sheet name="LEGAL DISCLAIMER" sheetId="11" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="40">
   <si>
     <t>WAL</t>
   </si>
@@ -150,6 +151,12 @@
   </si>
   <si>
     <t>Table G. (06/30/2026) Below Investment Grade Current Benchmark Spreads (in bps)</t>
+  </si>
+  <si>
+    <t>Table F (07/31/2026)  Investment Grade Current Benchmark Spreads (in bps)</t>
+  </si>
+  <si>
+    <t>Table G. (07/31/2026) Below Investment Grade Current Benchmark Spreads (in bps)</t>
   </si>
 </sst>
 </file>
@@ -426,7 +433,7 @@
                   <a14:compatExt spid="_x0000_s4104"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0500-000008100000}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0600-000008100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -747,15 +754,2338 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00F3680C-3C4D-44B1-A900-BDF4637D600C}">
+  <dimension ref="A1:W35"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="11.08984375" customWidth="1"/>
+    <col min="13" max="23" width="11.08984375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="M1" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="N1" s="14"/>
+      <c r="O1" s="14"/>
+      <c r="P1" s="14"/>
+      <c r="Q1" s="14"/>
+      <c r="R1" s="14"/>
+      <c r="S1" s="14"/>
+      <c r="T1" s="14"/>
+      <c r="U1" s="14"/>
+      <c r="V1" s="14"/>
+      <c r="W1" s="15"/>
+    </row>
+    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A2" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12"/>
+      <c r="K2" s="12"/>
+      <c r="M2" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="N2" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="O2" s="12"/>
+      <c r="P2" s="12"/>
+      <c r="Q2" s="12"/>
+      <c r="R2" s="12"/>
+      <c r="S2" s="12"/>
+      <c r="T2" s="12"/>
+      <c r="U2" s="12"/>
+      <c r="V2" s="12"/>
+      <c r="W2" s="12"/>
+    </row>
+    <row r="3" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A3" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="5">
+        <v>1</v>
+      </c>
+      <c r="C3" s="5">
+        <v>2</v>
+      </c>
+      <c r="D3" s="5">
+        <v>3</v>
+      </c>
+      <c r="E3" s="5">
+        <v>4</v>
+      </c>
+      <c r="F3" s="5">
+        <v>5</v>
+      </c>
+      <c r="G3" s="5">
+        <v>6</v>
+      </c>
+      <c r="H3" s="5">
+        <v>7</v>
+      </c>
+      <c r="I3" s="5">
+        <v>8</v>
+      </c>
+      <c r="J3" s="5">
+        <v>9</v>
+      </c>
+      <c r="K3" s="5">
+        <v>10</v>
+      </c>
+      <c r="M3" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="N3" s="5">
+        <v>11</v>
+      </c>
+      <c r="O3" s="5">
+        <v>12</v>
+      </c>
+      <c r="P3" s="5">
+        <v>13</v>
+      </c>
+      <c r="Q3" s="5">
+        <v>14</v>
+      </c>
+      <c r="R3" s="5">
+        <v>15</v>
+      </c>
+      <c r="S3" s="5">
+        <v>16</v>
+      </c>
+      <c r="T3" s="5">
+        <v>17</v>
+      </c>
+      <c r="U3" s="5">
+        <v>18</v>
+      </c>
+      <c r="V3" s="5">
+        <v>19</v>
+      </c>
+      <c r="W3" s="5">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A4" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="M4" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="P4" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q4" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="R4" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="S4" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="T4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="U4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="V4" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="W4" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A5" s="5">
+        <v>1</v>
+      </c>
+      <c r="B5" s="8">
+        <v>2.9</v>
+      </c>
+      <c r="C5" s="8">
+        <v>12.76</v>
+      </c>
+      <c r="D5" s="8">
+        <v>22.62</v>
+      </c>
+      <c r="E5" s="8">
+        <v>27.49</v>
+      </c>
+      <c r="F5" s="8">
+        <v>32.36</v>
+      </c>
+      <c r="G5" s="8">
+        <v>37.229999999999997</v>
+      </c>
+      <c r="H5" s="8">
+        <v>45.69</v>
+      </c>
+      <c r="I5" s="8">
+        <v>54.15</v>
+      </c>
+      <c r="J5" s="8">
+        <v>62.62</v>
+      </c>
+      <c r="K5" s="8">
+        <v>100.85</v>
+      </c>
+      <c r="M5" s="9">
+        <v>1</v>
+      </c>
+      <c r="N5" s="8">
+        <v>139.08000000000001</v>
+      </c>
+      <c r="O5" s="8">
+        <v>185.81</v>
+      </c>
+      <c r="P5" s="8">
+        <v>232.54</v>
+      </c>
+      <c r="Q5" s="8">
+        <v>279.27</v>
+      </c>
+      <c r="R5" s="8">
+        <v>325.99</v>
+      </c>
+      <c r="S5" s="8">
+        <v>562</v>
+      </c>
+      <c r="T5" s="8">
+        <v>798</v>
+      </c>
+      <c r="U5" s="8">
+        <v>1034</v>
+      </c>
+      <c r="V5" s="8">
+        <v>1270</v>
+      </c>
+      <c r="W5" s="8">
+        <v>1506</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A6" s="5">
+        <v>2</v>
+      </c>
+      <c r="B6" s="8">
+        <v>7.73</v>
+      </c>
+      <c r="C6" s="8">
+        <v>18.62</v>
+      </c>
+      <c r="D6" s="8">
+        <v>29.51</v>
+      </c>
+      <c r="E6" s="8">
+        <v>34.700000000000003</v>
+      </c>
+      <c r="F6" s="8">
+        <v>39.9</v>
+      </c>
+      <c r="G6" s="8">
+        <v>45.09</v>
+      </c>
+      <c r="H6" s="8">
+        <v>53.78</v>
+      </c>
+      <c r="I6" s="8">
+        <v>62.47</v>
+      </c>
+      <c r="J6" s="8">
+        <v>71.16</v>
+      </c>
+      <c r="K6" s="8">
+        <v>105.12</v>
+      </c>
+      <c r="M6" s="9">
+        <v>2</v>
+      </c>
+      <c r="N6" s="8">
+        <v>139.08000000000001</v>
+      </c>
+      <c r="O6" s="8">
+        <v>185.81</v>
+      </c>
+      <c r="P6" s="8">
+        <v>232.54</v>
+      </c>
+      <c r="Q6" s="8">
+        <v>279.27</v>
+      </c>
+      <c r="R6" s="8">
+        <v>325.99</v>
+      </c>
+      <c r="S6" s="8">
+        <v>562</v>
+      </c>
+      <c r="T6" s="8">
+        <v>798</v>
+      </c>
+      <c r="U6" s="8">
+        <v>1034</v>
+      </c>
+      <c r="V6" s="8">
+        <v>1270</v>
+      </c>
+      <c r="W6" s="8">
+        <v>1506</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A7" s="5">
+        <v>3</v>
+      </c>
+      <c r="B7" s="8">
+        <v>12.57</v>
+      </c>
+      <c r="C7" s="8">
+        <v>24.48</v>
+      </c>
+      <c r="D7" s="8">
+        <v>36.4</v>
+      </c>
+      <c r="E7" s="8">
+        <v>41.92</v>
+      </c>
+      <c r="F7" s="8">
+        <v>47.43</v>
+      </c>
+      <c r="G7" s="8">
+        <v>52.95</v>
+      </c>
+      <c r="H7" s="8">
+        <v>61.86</v>
+      </c>
+      <c r="I7" s="8">
+        <v>70.78</v>
+      </c>
+      <c r="J7" s="8">
+        <v>79.7</v>
+      </c>
+      <c r="K7" s="8">
+        <v>109.39</v>
+      </c>
+      <c r="M7" s="9">
+        <v>3</v>
+      </c>
+      <c r="N7" s="8">
+        <v>139.08000000000001</v>
+      </c>
+      <c r="O7" s="8">
+        <v>185.81</v>
+      </c>
+      <c r="P7" s="8">
+        <v>232.54</v>
+      </c>
+      <c r="Q7" s="8">
+        <v>279.27</v>
+      </c>
+      <c r="R7" s="8">
+        <v>325.99</v>
+      </c>
+      <c r="S7" s="8">
+        <v>562</v>
+      </c>
+      <c r="T7" s="8">
+        <v>798</v>
+      </c>
+      <c r="U7" s="8">
+        <v>1034</v>
+      </c>
+      <c r="V7" s="8">
+        <v>1270</v>
+      </c>
+      <c r="W7" s="8">
+        <v>1506</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A8" s="5">
+        <v>4</v>
+      </c>
+      <c r="B8" s="8">
+        <v>17.399999999999999</v>
+      </c>
+      <c r="C8" s="8">
+        <v>30.34</v>
+      </c>
+      <c r="D8" s="8">
+        <v>43.29</v>
+      </c>
+      <c r="E8" s="8">
+        <v>49.13</v>
+      </c>
+      <c r="F8" s="8">
+        <v>54.97</v>
+      </c>
+      <c r="G8" s="8">
+        <v>60.81</v>
+      </c>
+      <c r="H8" s="8">
+        <v>69.95</v>
+      </c>
+      <c r="I8" s="8">
+        <v>79.09</v>
+      </c>
+      <c r="J8" s="8">
+        <v>88.24</v>
+      </c>
+      <c r="K8" s="8">
+        <v>113.66</v>
+      </c>
+      <c r="M8" s="9">
+        <v>4</v>
+      </c>
+      <c r="N8" s="8">
+        <v>139.08000000000001</v>
+      </c>
+      <c r="O8" s="8">
+        <v>185.81</v>
+      </c>
+      <c r="P8" s="8">
+        <v>232.54</v>
+      </c>
+      <c r="Q8" s="8">
+        <v>279.27</v>
+      </c>
+      <c r="R8" s="8">
+        <v>325.99</v>
+      </c>
+      <c r="S8" s="8">
+        <v>562</v>
+      </c>
+      <c r="T8" s="8">
+        <v>798</v>
+      </c>
+      <c r="U8" s="8">
+        <v>1034</v>
+      </c>
+      <c r="V8" s="8">
+        <v>1270</v>
+      </c>
+      <c r="W8" s="8">
+        <v>1506</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A9" s="5">
+        <v>5</v>
+      </c>
+      <c r="B9" s="8">
+        <v>18.46</v>
+      </c>
+      <c r="C9" s="8">
+        <v>33.380000000000003</v>
+      </c>
+      <c r="D9" s="8">
+        <v>48.29</v>
+      </c>
+      <c r="E9" s="8">
+        <v>54.09</v>
+      </c>
+      <c r="F9" s="8">
+        <v>59.89</v>
+      </c>
+      <c r="G9" s="8">
+        <v>65.7</v>
+      </c>
+      <c r="H9" s="8">
+        <v>74.92</v>
+      </c>
+      <c r="I9" s="8">
+        <v>84.15</v>
+      </c>
+      <c r="J9" s="8">
+        <v>93.38</v>
+      </c>
+      <c r="K9" s="8">
+        <v>116.23</v>
+      </c>
+      <c r="M9" s="9">
+        <v>5</v>
+      </c>
+      <c r="N9" s="8">
+        <v>139.08000000000001</v>
+      </c>
+      <c r="O9" s="8">
+        <v>185.81</v>
+      </c>
+      <c r="P9" s="8">
+        <v>232.54</v>
+      </c>
+      <c r="Q9" s="8">
+        <v>279.27</v>
+      </c>
+      <c r="R9" s="8">
+        <v>325.99</v>
+      </c>
+      <c r="S9" s="8">
+        <v>562</v>
+      </c>
+      <c r="T9" s="8">
+        <v>798</v>
+      </c>
+      <c r="U9" s="8">
+        <v>1034</v>
+      </c>
+      <c r="V9" s="8">
+        <v>1270</v>
+      </c>
+      <c r="W9" s="8">
+        <v>1506</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A10" s="5">
+        <v>6</v>
+      </c>
+      <c r="B10" s="8">
+        <v>19.53</v>
+      </c>
+      <c r="C10" s="8">
+        <v>36.409999999999997</v>
+      </c>
+      <c r="D10" s="8">
+        <v>53.29</v>
+      </c>
+      <c r="E10" s="8">
+        <v>59.05</v>
+      </c>
+      <c r="F10" s="8">
+        <v>64.819999999999993</v>
+      </c>
+      <c r="G10" s="8">
+        <v>70.59</v>
+      </c>
+      <c r="H10" s="8">
+        <v>79.900000000000006</v>
+      </c>
+      <c r="I10" s="8">
+        <v>89.21</v>
+      </c>
+      <c r="J10" s="8">
+        <v>98.52</v>
+      </c>
+      <c r="K10" s="8">
+        <v>118.8</v>
+      </c>
+      <c r="M10" s="9">
+        <v>6</v>
+      </c>
+      <c r="N10" s="8">
+        <v>139.08000000000001</v>
+      </c>
+      <c r="O10" s="8">
+        <v>185.81</v>
+      </c>
+      <c r="P10" s="8">
+        <v>232.54</v>
+      </c>
+      <c r="Q10" s="8">
+        <v>279.27</v>
+      </c>
+      <c r="R10" s="8">
+        <v>325.99</v>
+      </c>
+      <c r="S10" s="8">
+        <v>562</v>
+      </c>
+      <c r="T10" s="8">
+        <v>798</v>
+      </c>
+      <c r="U10" s="8">
+        <v>1034</v>
+      </c>
+      <c r="V10" s="8">
+        <v>1270</v>
+      </c>
+      <c r="W10" s="8">
+        <v>1506</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A11" s="5">
+        <v>7</v>
+      </c>
+      <c r="B11" s="8">
+        <v>23.86</v>
+      </c>
+      <c r="C11" s="8">
+        <v>41</v>
+      </c>
+      <c r="D11" s="8">
+        <v>58.15</v>
+      </c>
+      <c r="E11" s="8">
+        <v>63.73</v>
+      </c>
+      <c r="F11" s="8">
+        <v>69.319999999999993</v>
+      </c>
+      <c r="G11" s="8">
+        <v>74.900000000000006</v>
+      </c>
+      <c r="H11" s="8">
+        <v>84.4</v>
+      </c>
+      <c r="I11" s="8">
+        <v>93.9</v>
+      </c>
+      <c r="J11" s="8">
+        <v>103.4</v>
+      </c>
+      <c r="K11" s="8">
+        <v>121.24</v>
+      </c>
+      <c r="M11" s="9">
+        <v>7</v>
+      </c>
+      <c r="N11" s="8">
+        <v>139.08000000000001</v>
+      </c>
+      <c r="O11" s="8">
+        <v>185.81</v>
+      </c>
+      <c r="P11" s="8">
+        <v>232.54</v>
+      </c>
+      <c r="Q11" s="8">
+        <v>279.27</v>
+      </c>
+      <c r="R11" s="8">
+        <v>325.99</v>
+      </c>
+      <c r="S11" s="8">
+        <v>562</v>
+      </c>
+      <c r="T11" s="8">
+        <v>798</v>
+      </c>
+      <c r="U11" s="8">
+        <v>1034</v>
+      </c>
+      <c r="V11" s="8">
+        <v>1270</v>
+      </c>
+      <c r="W11" s="8">
+        <v>1506</v>
+      </c>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A12" s="5">
+        <v>8</v>
+      </c>
+      <c r="B12" s="8">
+        <v>28.18</v>
+      </c>
+      <c r="C12" s="8">
+        <v>45.6</v>
+      </c>
+      <c r="D12" s="8">
+        <v>63.01</v>
+      </c>
+      <c r="E12" s="8">
+        <v>68.42</v>
+      </c>
+      <c r="F12" s="8">
+        <v>73.819999999999993</v>
+      </c>
+      <c r="G12" s="8">
+        <v>79.22</v>
+      </c>
+      <c r="H12" s="8">
+        <v>88.91</v>
+      </c>
+      <c r="I12" s="8">
+        <v>98.6</v>
+      </c>
+      <c r="J12" s="8">
+        <v>108.28</v>
+      </c>
+      <c r="K12" s="8">
+        <v>123.68</v>
+      </c>
+      <c r="M12" s="9">
+        <v>8</v>
+      </c>
+      <c r="N12" s="8">
+        <v>139.08000000000001</v>
+      </c>
+      <c r="O12" s="8">
+        <v>185.81</v>
+      </c>
+      <c r="P12" s="8">
+        <v>232.54</v>
+      </c>
+      <c r="Q12" s="8">
+        <v>279.27</v>
+      </c>
+      <c r="R12" s="8">
+        <v>325.99</v>
+      </c>
+      <c r="S12" s="8">
+        <v>562</v>
+      </c>
+      <c r="T12" s="8">
+        <v>798</v>
+      </c>
+      <c r="U12" s="8">
+        <v>1034</v>
+      </c>
+      <c r="V12" s="8">
+        <v>1270</v>
+      </c>
+      <c r="W12" s="8">
+        <v>1506</v>
+      </c>
+    </row>
+    <row r="13" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A13" s="5">
+        <v>9</v>
+      </c>
+      <c r="B13" s="8">
+        <v>32.5</v>
+      </c>
+      <c r="C13" s="8">
+        <v>50.19</v>
+      </c>
+      <c r="D13" s="8">
+        <v>67.88</v>
+      </c>
+      <c r="E13" s="8">
+        <v>73.099999999999994</v>
+      </c>
+      <c r="F13" s="8">
+        <v>78.319999999999993</v>
+      </c>
+      <c r="G13" s="8">
+        <v>83.54</v>
+      </c>
+      <c r="H13" s="8">
+        <v>93.41</v>
+      </c>
+      <c r="I13" s="8">
+        <v>103.29</v>
+      </c>
+      <c r="J13" s="8">
+        <v>113.17</v>
+      </c>
+      <c r="K13" s="8">
+        <v>126.12</v>
+      </c>
+      <c r="M13" s="9">
+        <v>9</v>
+      </c>
+      <c r="N13" s="8">
+        <v>139.08000000000001</v>
+      </c>
+      <c r="O13" s="8">
+        <v>185.81</v>
+      </c>
+      <c r="P13" s="8">
+        <v>232.54</v>
+      </c>
+      <c r="Q13" s="8">
+        <v>279.27</v>
+      </c>
+      <c r="R13" s="8">
+        <v>325.99</v>
+      </c>
+      <c r="S13" s="8">
+        <v>562</v>
+      </c>
+      <c r="T13" s="8">
+        <v>798</v>
+      </c>
+      <c r="U13" s="8">
+        <v>1034</v>
+      </c>
+      <c r="V13" s="8">
+        <v>1270</v>
+      </c>
+      <c r="W13" s="8">
+        <v>1506</v>
+      </c>
+    </row>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A14" s="5">
+        <v>10</v>
+      </c>
+      <c r="B14" s="8">
+        <v>34.14</v>
+      </c>
+      <c r="C14" s="8">
+        <v>51.68</v>
+      </c>
+      <c r="D14" s="8">
+        <v>69.22</v>
+      </c>
+      <c r="E14" s="8">
+        <v>74.010000000000005</v>
+      </c>
+      <c r="F14" s="8">
+        <v>78.81</v>
+      </c>
+      <c r="G14" s="8">
+        <v>83.6</v>
+      </c>
+      <c r="H14" s="8">
+        <v>93.71</v>
+      </c>
+      <c r="I14" s="8">
+        <v>103.82</v>
+      </c>
+      <c r="J14" s="8">
+        <v>113.93</v>
+      </c>
+      <c r="K14" s="8">
+        <v>126.51</v>
+      </c>
+      <c r="M14" s="9">
+        <v>10</v>
+      </c>
+      <c r="N14" s="8">
+        <v>139.08000000000001</v>
+      </c>
+      <c r="O14" s="8">
+        <v>185.81</v>
+      </c>
+      <c r="P14" s="8">
+        <v>232.54</v>
+      </c>
+      <c r="Q14" s="8">
+        <v>279.27</v>
+      </c>
+      <c r="R14" s="8">
+        <v>325.99</v>
+      </c>
+      <c r="S14" s="8">
+        <v>562</v>
+      </c>
+      <c r="T14" s="8">
+        <v>798</v>
+      </c>
+      <c r="U14" s="8">
+        <v>1034</v>
+      </c>
+      <c r="V14" s="8">
+        <v>1270</v>
+      </c>
+      <c r="W14" s="8">
+        <v>1506</v>
+      </c>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A15" s="5">
+        <v>11</v>
+      </c>
+      <c r="B15" s="8">
+        <v>35.78</v>
+      </c>
+      <c r="C15" s="8">
+        <v>53.17</v>
+      </c>
+      <c r="D15" s="8">
+        <v>70.56</v>
+      </c>
+      <c r="E15" s="8">
+        <v>74.930000000000007</v>
+      </c>
+      <c r="F15" s="8">
+        <v>79.290000000000006</v>
+      </c>
+      <c r="G15" s="8">
+        <v>83.66</v>
+      </c>
+      <c r="H15" s="8">
+        <v>94.01</v>
+      </c>
+      <c r="I15" s="8">
+        <v>104.35</v>
+      </c>
+      <c r="J15" s="8">
+        <v>114.7</v>
+      </c>
+      <c r="K15" s="8">
+        <v>126.89</v>
+      </c>
+      <c r="M15" s="9">
+        <v>11</v>
+      </c>
+      <c r="N15" s="8">
+        <v>139.08000000000001</v>
+      </c>
+      <c r="O15" s="8">
+        <v>185.81</v>
+      </c>
+      <c r="P15" s="8">
+        <v>232.54</v>
+      </c>
+      <c r="Q15" s="8">
+        <v>279.27</v>
+      </c>
+      <c r="R15" s="8">
+        <v>325.99</v>
+      </c>
+      <c r="S15" s="8">
+        <v>562</v>
+      </c>
+      <c r="T15" s="8">
+        <v>798</v>
+      </c>
+      <c r="U15" s="8">
+        <v>1034</v>
+      </c>
+      <c r="V15" s="8">
+        <v>1270</v>
+      </c>
+      <c r="W15" s="8">
+        <v>1506</v>
+      </c>
+    </row>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A16" s="5">
+        <v>12</v>
+      </c>
+      <c r="B16" s="8">
+        <v>37.409999999999997</v>
+      </c>
+      <c r="C16" s="8">
+        <v>54.66</v>
+      </c>
+      <c r="D16" s="8">
+        <v>71.900000000000006</v>
+      </c>
+      <c r="E16" s="8">
+        <v>75.84</v>
+      </c>
+      <c r="F16" s="8">
+        <v>79.78</v>
+      </c>
+      <c r="G16" s="8">
+        <v>83.73</v>
+      </c>
+      <c r="H16" s="8">
+        <v>94.3</v>
+      </c>
+      <c r="I16" s="8">
+        <v>104.88</v>
+      </c>
+      <c r="J16" s="8">
+        <v>115.46</v>
+      </c>
+      <c r="K16" s="8">
+        <v>127.27</v>
+      </c>
+      <c r="M16" s="9">
+        <v>12</v>
+      </c>
+      <c r="N16" s="8">
+        <v>139.08000000000001</v>
+      </c>
+      <c r="O16" s="8">
+        <v>185.81</v>
+      </c>
+      <c r="P16" s="8">
+        <v>232.54</v>
+      </c>
+      <c r="Q16" s="8">
+        <v>279.27</v>
+      </c>
+      <c r="R16" s="8">
+        <v>325.99</v>
+      </c>
+      <c r="S16" s="8">
+        <v>562</v>
+      </c>
+      <c r="T16" s="8">
+        <v>798</v>
+      </c>
+      <c r="U16" s="8">
+        <v>1034</v>
+      </c>
+      <c r="V16" s="8">
+        <v>1270</v>
+      </c>
+      <c r="W16" s="8">
+        <v>1506</v>
+      </c>
+    </row>
+    <row r="17" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A17" s="5">
+        <v>13</v>
+      </c>
+      <c r="B17" s="8">
+        <v>39.049999999999997</v>
+      </c>
+      <c r="C17" s="8">
+        <v>56.14</v>
+      </c>
+      <c r="D17" s="8">
+        <v>73.239999999999995</v>
+      </c>
+      <c r="E17" s="8">
+        <v>76.75</v>
+      </c>
+      <c r="F17" s="8">
+        <v>80.27</v>
+      </c>
+      <c r="G17" s="8">
+        <v>83.79</v>
+      </c>
+      <c r="H17" s="8">
+        <v>94.6</v>
+      </c>
+      <c r="I17" s="8">
+        <v>105.41</v>
+      </c>
+      <c r="J17" s="8">
+        <v>116.22</v>
+      </c>
+      <c r="K17" s="8">
+        <v>127.65</v>
+      </c>
+      <c r="M17" s="9">
+        <v>13</v>
+      </c>
+      <c r="N17" s="8">
+        <v>139.08000000000001</v>
+      </c>
+      <c r="O17" s="8">
+        <v>185.81</v>
+      </c>
+      <c r="P17" s="8">
+        <v>232.54</v>
+      </c>
+      <c r="Q17" s="8">
+        <v>279.27</v>
+      </c>
+      <c r="R17" s="8">
+        <v>325.99</v>
+      </c>
+      <c r="S17" s="8">
+        <v>562</v>
+      </c>
+      <c r="T17" s="8">
+        <v>798</v>
+      </c>
+      <c r="U17" s="8">
+        <v>1034</v>
+      </c>
+      <c r="V17" s="8">
+        <v>1270</v>
+      </c>
+      <c r="W17" s="8">
+        <v>1506</v>
+      </c>
+    </row>
+    <row r="18" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A18" s="5">
+        <v>14</v>
+      </c>
+      <c r="B18" s="8">
+        <v>40.69</v>
+      </c>
+      <c r="C18" s="8">
+        <v>57.63</v>
+      </c>
+      <c r="D18" s="8">
+        <v>74.58</v>
+      </c>
+      <c r="E18" s="8">
+        <v>77.67</v>
+      </c>
+      <c r="F18" s="8">
+        <v>80.760000000000005</v>
+      </c>
+      <c r="G18" s="8">
+        <v>83.85</v>
+      </c>
+      <c r="H18" s="8">
+        <v>94.9</v>
+      </c>
+      <c r="I18" s="8">
+        <v>105.94</v>
+      </c>
+      <c r="J18" s="8">
+        <v>116.99</v>
+      </c>
+      <c r="K18" s="8">
+        <v>128.03</v>
+      </c>
+      <c r="M18" s="9">
+        <v>14</v>
+      </c>
+      <c r="N18" s="8">
+        <v>139.08000000000001</v>
+      </c>
+      <c r="O18" s="8">
+        <v>185.81</v>
+      </c>
+      <c r="P18" s="8">
+        <v>232.54</v>
+      </c>
+      <c r="Q18" s="8">
+        <v>279.27</v>
+      </c>
+      <c r="R18" s="8">
+        <v>325.99</v>
+      </c>
+      <c r="S18" s="8">
+        <v>562</v>
+      </c>
+      <c r="T18" s="8">
+        <v>798</v>
+      </c>
+      <c r="U18" s="8">
+        <v>1034</v>
+      </c>
+      <c r="V18" s="8">
+        <v>1270</v>
+      </c>
+      <c r="W18" s="8">
+        <v>1506</v>
+      </c>
+    </row>
+    <row r="19" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A19" s="5">
+        <v>15</v>
+      </c>
+      <c r="B19" s="8">
+        <v>42.33</v>
+      </c>
+      <c r="C19" s="8">
+        <v>59.12</v>
+      </c>
+      <c r="D19" s="8">
+        <v>75.92</v>
+      </c>
+      <c r="E19" s="8">
+        <v>78.58</v>
+      </c>
+      <c r="F19" s="8">
+        <v>81.25</v>
+      </c>
+      <c r="G19" s="8">
+        <v>83.92</v>
+      </c>
+      <c r="H19" s="8">
+        <v>95.19</v>
+      </c>
+      <c r="I19" s="8">
+        <v>106.47</v>
+      </c>
+      <c r="J19" s="8">
+        <v>117.75</v>
+      </c>
+      <c r="K19" s="8">
+        <v>128.41999999999999</v>
+      </c>
+      <c r="M19" s="9">
+        <v>15</v>
+      </c>
+      <c r="N19" s="8">
+        <v>139.08000000000001</v>
+      </c>
+      <c r="O19" s="8">
+        <v>185.81</v>
+      </c>
+      <c r="P19" s="8">
+        <v>232.54</v>
+      </c>
+      <c r="Q19" s="8">
+        <v>279.27</v>
+      </c>
+      <c r="R19" s="8">
+        <v>325.99</v>
+      </c>
+      <c r="S19" s="8">
+        <v>562</v>
+      </c>
+      <c r="T19" s="8">
+        <v>798</v>
+      </c>
+      <c r="U19" s="8">
+        <v>1034</v>
+      </c>
+      <c r="V19" s="8">
+        <v>1270</v>
+      </c>
+      <c r="W19" s="8">
+        <v>1506</v>
+      </c>
+    </row>
+    <row r="20" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A20" s="5">
+        <v>16</v>
+      </c>
+      <c r="B20" s="8">
+        <v>43.97</v>
+      </c>
+      <c r="C20" s="8">
+        <v>60.61</v>
+      </c>
+      <c r="D20" s="8">
+        <v>77.260000000000005</v>
+      </c>
+      <c r="E20" s="8">
+        <v>79.5</v>
+      </c>
+      <c r="F20" s="8">
+        <v>81.739999999999995</v>
+      </c>
+      <c r="G20" s="8">
+        <v>83.98</v>
+      </c>
+      <c r="H20" s="8">
+        <v>95.49</v>
+      </c>
+      <c r="I20" s="8">
+        <v>107</v>
+      </c>
+      <c r="J20" s="8">
+        <v>118.52</v>
+      </c>
+      <c r="K20" s="8">
+        <v>128.80000000000001</v>
+      </c>
+      <c r="M20" s="9">
+        <v>16</v>
+      </c>
+      <c r="N20" s="8">
+        <v>139.08000000000001</v>
+      </c>
+      <c r="O20" s="8">
+        <v>185.81</v>
+      </c>
+      <c r="P20" s="8">
+        <v>232.54</v>
+      </c>
+      <c r="Q20" s="8">
+        <v>279.27</v>
+      </c>
+      <c r="R20" s="8">
+        <v>325.99</v>
+      </c>
+      <c r="S20" s="8">
+        <v>562</v>
+      </c>
+      <c r="T20" s="8">
+        <v>798</v>
+      </c>
+      <c r="U20" s="8">
+        <v>1034</v>
+      </c>
+      <c r="V20" s="8">
+        <v>1270</v>
+      </c>
+      <c r="W20" s="8">
+        <v>1506</v>
+      </c>
+    </row>
+    <row r="21" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A21" s="5">
+        <v>17</v>
+      </c>
+      <c r="B21" s="8">
+        <v>45.61</v>
+      </c>
+      <c r="C21" s="8">
+        <v>62.1</v>
+      </c>
+      <c r="D21" s="8">
+        <v>78.599999999999994</v>
+      </c>
+      <c r="E21" s="8">
+        <v>80.41</v>
+      </c>
+      <c r="F21" s="8">
+        <v>82.23</v>
+      </c>
+      <c r="G21" s="8">
+        <v>84.04</v>
+      </c>
+      <c r="H21" s="8">
+        <v>95.79</v>
+      </c>
+      <c r="I21" s="8">
+        <v>107.53</v>
+      </c>
+      <c r="J21" s="8">
+        <v>119.28</v>
+      </c>
+      <c r="K21" s="8">
+        <v>129.18</v>
+      </c>
+      <c r="M21" s="9">
+        <v>17</v>
+      </c>
+      <c r="N21" s="8">
+        <v>139.08000000000001</v>
+      </c>
+      <c r="O21" s="8">
+        <v>185.81</v>
+      </c>
+      <c r="P21" s="8">
+        <v>232.54</v>
+      </c>
+      <c r="Q21" s="8">
+        <v>279.27</v>
+      </c>
+      <c r="R21" s="8">
+        <v>325.99</v>
+      </c>
+      <c r="S21" s="8">
+        <v>562</v>
+      </c>
+      <c r="T21" s="8">
+        <v>798</v>
+      </c>
+      <c r="U21" s="8">
+        <v>1034</v>
+      </c>
+      <c r="V21" s="8">
+        <v>1270</v>
+      </c>
+      <c r="W21" s="8">
+        <v>1506</v>
+      </c>
+    </row>
+    <row r="22" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A22" s="5">
+        <v>18</v>
+      </c>
+      <c r="B22" s="8">
+        <v>47.25</v>
+      </c>
+      <c r="C22" s="8">
+        <v>63.59</v>
+      </c>
+      <c r="D22" s="8">
+        <v>79.930000000000007</v>
+      </c>
+      <c r="E22" s="8">
+        <v>81.319999999999993</v>
+      </c>
+      <c r="F22" s="8">
+        <v>82.72</v>
+      </c>
+      <c r="G22" s="8">
+        <v>84.11</v>
+      </c>
+      <c r="H22" s="8">
+        <v>96.09</v>
+      </c>
+      <c r="I22" s="8">
+        <v>108.06</v>
+      </c>
+      <c r="J22" s="8">
+        <v>120.04</v>
+      </c>
+      <c r="K22" s="8">
+        <v>129.56</v>
+      </c>
+      <c r="M22" s="9">
+        <v>18</v>
+      </c>
+      <c r="N22" s="8">
+        <v>139.08000000000001</v>
+      </c>
+      <c r="O22" s="8">
+        <v>185.81</v>
+      </c>
+      <c r="P22" s="8">
+        <v>232.54</v>
+      </c>
+      <c r="Q22" s="8">
+        <v>279.27</v>
+      </c>
+      <c r="R22" s="8">
+        <v>325.99</v>
+      </c>
+      <c r="S22" s="8">
+        <v>562</v>
+      </c>
+      <c r="T22" s="8">
+        <v>798</v>
+      </c>
+      <c r="U22" s="8">
+        <v>1034</v>
+      </c>
+      <c r="V22" s="8">
+        <v>1270</v>
+      </c>
+      <c r="W22" s="8">
+        <v>1506</v>
+      </c>
+    </row>
+    <row r="23" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A23" s="5">
+        <v>19</v>
+      </c>
+      <c r="B23" s="8">
+        <v>48.88</v>
+      </c>
+      <c r="C23" s="8">
+        <v>65.08</v>
+      </c>
+      <c r="D23" s="8">
+        <v>81.27</v>
+      </c>
+      <c r="E23" s="8">
+        <v>82.24</v>
+      </c>
+      <c r="F23" s="8">
+        <v>83.2</v>
+      </c>
+      <c r="G23" s="8">
+        <v>84.17</v>
+      </c>
+      <c r="H23" s="8">
+        <v>96.38</v>
+      </c>
+      <c r="I23" s="8">
+        <v>108.6</v>
+      </c>
+      <c r="J23" s="8">
+        <v>120.81</v>
+      </c>
+      <c r="K23" s="8">
+        <v>129.94</v>
+      </c>
+      <c r="M23" s="9">
+        <v>19</v>
+      </c>
+      <c r="N23" s="8">
+        <v>139.08000000000001</v>
+      </c>
+      <c r="O23" s="8">
+        <v>185.81</v>
+      </c>
+      <c r="P23" s="8">
+        <v>232.54</v>
+      </c>
+      <c r="Q23" s="8">
+        <v>279.27</v>
+      </c>
+      <c r="R23" s="8">
+        <v>325.99</v>
+      </c>
+      <c r="S23" s="8">
+        <v>562</v>
+      </c>
+      <c r="T23" s="8">
+        <v>798</v>
+      </c>
+      <c r="U23" s="8">
+        <v>1034</v>
+      </c>
+      <c r="V23" s="8">
+        <v>1270</v>
+      </c>
+      <c r="W23" s="8">
+        <v>1506</v>
+      </c>
+    </row>
+    <row r="24" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A24" s="5">
+        <v>20</v>
+      </c>
+      <c r="B24" s="8">
+        <v>50.52</v>
+      </c>
+      <c r="C24" s="8">
+        <v>66.569999999999993</v>
+      </c>
+      <c r="D24" s="8">
+        <v>82.61</v>
+      </c>
+      <c r="E24" s="8">
+        <v>83.15</v>
+      </c>
+      <c r="F24" s="8">
+        <v>83.69</v>
+      </c>
+      <c r="G24" s="8">
+        <v>84.23</v>
+      </c>
+      <c r="H24" s="8">
+        <v>96.68</v>
+      </c>
+      <c r="I24" s="8">
+        <v>109.13</v>
+      </c>
+      <c r="J24" s="8">
+        <v>121.57</v>
+      </c>
+      <c r="K24" s="8">
+        <v>130.33000000000001</v>
+      </c>
+      <c r="M24" s="9">
+        <v>20</v>
+      </c>
+      <c r="N24" s="8">
+        <v>139.08000000000001</v>
+      </c>
+      <c r="O24" s="8">
+        <v>185.81</v>
+      </c>
+      <c r="P24" s="8">
+        <v>232.54</v>
+      </c>
+      <c r="Q24" s="8">
+        <v>279.27</v>
+      </c>
+      <c r="R24" s="8">
+        <v>325.99</v>
+      </c>
+      <c r="S24" s="8">
+        <v>562</v>
+      </c>
+      <c r="T24" s="8">
+        <v>798</v>
+      </c>
+      <c r="U24" s="8">
+        <v>1034</v>
+      </c>
+      <c r="V24" s="8">
+        <v>1270</v>
+      </c>
+      <c r="W24" s="8">
+        <v>1506</v>
+      </c>
+    </row>
+    <row r="25" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A25" s="5">
+        <v>21</v>
+      </c>
+      <c r="B25" s="8">
+        <v>52.16</v>
+      </c>
+      <c r="C25" s="8">
+        <v>68.06</v>
+      </c>
+      <c r="D25" s="8">
+        <v>83.95</v>
+      </c>
+      <c r="E25" s="8">
+        <v>84.07</v>
+      </c>
+      <c r="F25" s="8">
+        <v>84.18</v>
+      </c>
+      <c r="G25" s="8">
+        <v>84.29</v>
+      </c>
+      <c r="H25" s="8">
+        <v>96.98</v>
+      </c>
+      <c r="I25" s="8">
+        <v>109.66</v>
+      </c>
+      <c r="J25" s="8">
+        <v>122.34</v>
+      </c>
+      <c r="K25" s="8">
+        <v>130.71</v>
+      </c>
+      <c r="M25" s="9">
+        <v>21</v>
+      </c>
+      <c r="N25" s="8">
+        <v>139.08000000000001</v>
+      </c>
+      <c r="O25" s="8">
+        <v>185.81</v>
+      </c>
+      <c r="P25" s="8">
+        <v>232.54</v>
+      </c>
+      <c r="Q25" s="8">
+        <v>279.27</v>
+      </c>
+      <c r="R25" s="8">
+        <v>325.99</v>
+      </c>
+      <c r="S25" s="8">
+        <v>562</v>
+      </c>
+      <c r="T25" s="8">
+        <v>798</v>
+      </c>
+      <c r="U25" s="8">
+        <v>1034</v>
+      </c>
+      <c r="V25" s="8">
+        <v>1270</v>
+      </c>
+      <c r="W25" s="8">
+        <v>1506</v>
+      </c>
+    </row>
+    <row r="26" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A26" s="5">
+        <v>22</v>
+      </c>
+      <c r="B26" s="8">
+        <v>53.8</v>
+      </c>
+      <c r="C26" s="8">
+        <v>69.55</v>
+      </c>
+      <c r="D26" s="8">
+        <v>85.29</v>
+      </c>
+      <c r="E26" s="8">
+        <v>84.98</v>
+      </c>
+      <c r="F26" s="8">
+        <v>84.67</v>
+      </c>
+      <c r="G26" s="8">
+        <v>84.36</v>
+      </c>
+      <c r="H26" s="8">
+        <v>97.27</v>
+      </c>
+      <c r="I26" s="8">
+        <v>110.19</v>
+      </c>
+      <c r="J26" s="8">
+        <v>123.1</v>
+      </c>
+      <c r="K26" s="8">
+        <v>131.09</v>
+      </c>
+      <c r="M26" s="9">
+        <v>22</v>
+      </c>
+      <c r="N26" s="8">
+        <v>139.08000000000001</v>
+      </c>
+      <c r="O26" s="8">
+        <v>185.81</v>
+      </c>
+      <c r="P26" s="8">
+        <v>232.54</v>
+      </c>
+      <c r="Q26" s="8">
+        <v>279.27</v>
+      </c>
+      <c r="R26" s="8">
+        <v>325.99</v>
+      </c>
+      <c r="S26" s="8">
+        <v>562</v>
+      </c>
+      <c r="T26" s="8">
+        <v>798</v>
+      </c>
+      <c r="U26" s="8">
+        <v>1034</v>
+      </c>
+      <c r="V26" s="8">
+        <v>1270</v>
+      </c>
+      <c r="W26" s="8">
+        <v>1506</v>
+      </c>
+    </row>
+    <row r="27" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A27" s="5">
+        <v>23</v>
+      </c>
+      <c r="B27" s="8">
+        <v>55.44</v>
+      </c>
+      <c r="C27" s="8">
+        <v>71.03</v>
+      </c>
+      <c r="D27" s="8">
+        <v>86.63</v>
+      </c>
+      <c r="E27" s="8">
+        <v>85.9</v>
+      </c>
+      <c r="F27" s="8">
+        <v>85.16</v>
+      </c>
+      <c r="G27" s="8">
+        <v>84.42</v>
+      </c>
+      <c r="H27" s="8">
+        <v>97.57</v>
+      </c>
+      <c r="I27" s="8">
+        <v>110.72</v>
+      </c>
+      <c r="J27" s="8">
+        <v>123.86</v>
+      </c>
+      <c r="K27" s="8">
+        <v>131.47</v>
+      </c>
+      <c r="M27" s="9">
+        <v>23</v>
+      </c>
+      <c r="N27" s="8">
+        <v>139.08000000000001</v>
+      </c>
+      <c r="O27" s="8">
+        <v>185.81</v>
+      </c>
+      <c r="P27" s="8">
+        <v>232.54</v>
+      </c>
+      <c r="Q27" s="8">
+        <v>279.27</v>
+      </c>
+      <c r="R27" s="8">
+        <v>325.99</v>
+      </c>
+      <c r="S27" s="8">
+        <v>562</v>
+      </c>
+      <c r="T27" s="8">
+        <v>798</v>
+      </c>
+      <c r="U27" s="8">
+        <v>1034</v>
+      </c>
+      <c r="V27" s="8">
+        <v>1270</v>
+      </c>
+      <c r="W27" s="8">
+        <v>1506</v>
+      </c>
+    </row>
+    <row r="28" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A28" s="5">
+        <v>24</v>
+      </c>
+      <c r="B28" s="8">
+        <v>57.08</v>
+      </c>
+      <c r="C28" s="8">
+        <v>72.52</v>
+      </c>
+      <c r="D28" s="8">
+        <v>87.97</v>
+      </c>
+      <c r="E28" s="8">
+        <v>86.81</v>
+      </c>
+      <c r="F28" s="8">
+        <v>85.65</v>
+      </c>
+      <c r="G28" s="8">
+        <v>84.48</v>
+      </c>
+      <c r="H28" s="8">
+        <v>97.87</v>
+      </c>
+      <c r="I28" s="8">
+        <v>111.25</v>
+      </c>
+      <c r="J28" s="8">
+        <v>124.63</v>
+      </c>
+      <c r="K28" s="8">
+        <v>131.85</v>
+      </c>
+      <c r="M28" s="9">
+        <v>24</v>
+      </c>
+      <c r="N28" s="8">
+        <v>139.08000000000001</v>
+      </c>
+      <c r="O28" s="8">
+        <v>185.81</v>
+      </c>
+      <c r="P28" s="8">
+        <v>232.54</v>
+      </c>
+      <c r="Q28" s="8">
+        <v>279.27</v>
+      </c>
+      <c r="R28" s="8">
+        <v>325.99</v>
+      </c>
+      <c r="S28" s="8">
+        <v>562</v>
+      </c>
+      <c r="T28" s="8">
+        <v>798</v>
+      </c>
+      <c r="U28" s="8">
+        <v>1034</v>
+      </c>
+      <c r="V28" s="8">
+        <v>1270</v>
+      </c>
+      <c r="W28" s="8">
+        <v>1506</v>
+      </c>
+    </row>
+    <row r="29" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A29" s="5">
+        <v>25</v>
+      </c>
+      <c r="B29" s="8">
+        <v>58.71</v>
+      </c>
+      <c r="C29" s="8">
+        <v>74.010000000000005</v>
+      </c>
+      <c r="D29" s="8">
+        <v>89.31</v>
+      </c>
+      <c r="E29" s="8">
+        <v>87.72</v>
+      </c>
+      <c r="F29" s="8">
+        <v>86.14</v>
+      </c>
+      <c r="G29" s="8">
+        <v>84.55</v>
+      </c>
+      <c r="H29" s="8">
+        <v>98.16</v>
+      </c>
+      <c r="I29" s="8">
+        <v>111.78</v>
+      </c>
+      <c r="J29" s="8">
+        <v>125.39</v>
+      </c>
+      <c r="K29" s="8">
+        <v>132.24</v>
+      </c>
+      <c r="M29" s="9">
+        <v>25</v>
+      </c>
+      <c r="N29" s="8">
+        <v>139.08000000000001</v>
+      </c>
+      <c r="O29" s="8">
+        <v>185.81</v>
+      </c>
+      <c r="P29" s="8">
+        <v>232.54</v>
+      </c>
+      <c r="Q29" s="8">
+        <v>279.27</v>
+      </c>
+      <c r="R29" s="8">
+        <v>325.99</v>
+      </c>
+      <c r="S29" s="8">
+        <v>562</v>
+      </c>
+      <c r="T29" s="8">
+        <v>798</v>
+      </c>
+      <c r="U29" s="8">
+        <v>1034</v>
+      </c>
+      <c r="V29" s="8">
+        <v>1270</v>
+      </c>
+      <c r="W29" s="8">
+        <v>1506</v>
+      </c>
+    </row>
+    <row r="30" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A30" s="5">
+        <v>26</v>
+      </c>
+      <c r="B30" s="8">
+        <v>60.35</v>
+      </c>
+      <c r="C30" s="8">
+        <v>75.5</v>
+      </c>
+      <c r="D30" s="8">
+        <v>90.65</v>
+      </c>
+      <c r="E30" s="8">
+        <v>88.64</v>
+      </c>
+      <c r="F30" s="8">
+        <v>86.62</v>
+      </c>
+      <c r="G30" s="8">
+        <v>84.61</v>
+      </c>
+      <c r="H30" s="8">
+        <v>98.46</v>
+      </c>
+      <c r="I30" s="8">
+        <v>112.31</v>
+      </c>
+      <c r="J30" s="8">
+        <v>126.16</v>
+      </c>
+      <c r="K30" s="8">
+        <v>132.62</v>
+      </c>
+      <c r="M30" s="9">
+        <v>26</v>
+      </c>
+      <c r="N30" s="8">
+        <v>139.08000000000001</v>
+      </c>
+      <c r="O30" s="8">
+        <v>185.81</v>
+      </c>
+      <c r="P30" s="8">
+        <v>232.54</v>
+      </c>
+      <c r="Q30" s="8">
+        <v>279.27</v>
+      </c>
+      <c r="R30" s="8">
+        <v>325.99</v>
+      </c>
+      <c r="S30" s="8">
+        <v>562</v>
+      </c>
+      <c r="T30" s="8">
+        <v>798</v>
+      </c>
+      <c r="U30" s="8">
+        <v>1034</v>
+      </c>
+      <c r="V30" s="8">
+        <v>1270</v>
+      </c>
+      <c r="W30" s="8">
+        <v>1506</v>
+      </c>
+    </row>
+    <row r="31" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A31" s="5">
+        <v>27</v>
+      </c>
+      <c r="B31" s="8">
+        <v>61.99</v>
+      </c>
+      <c r="C31" s="8">
+        <v>76.989999999999995</v>
+      </c>
+      <c r="D31" s="8">
+        <v>91.99</v>
+      </c>
+      <c r="E31" s="8">
+        <v>89.55</v>
+      </c>
+      <c r="F31" s="8">
+        <v>87.11</v>
+      </c>
+      <c r="G31" s="8">
+        <v>84.67</v>
+      </c>
+      <c r="H31" s="8">
+        <v>98.76</v>
+      </c>
+      <c r="I31" s="8">
+        <v>112.84</v>
+      </c>
+      <c r="J31" s="8">
+        <v>126.92</v>
+      </c>
+      <c r="K31" s="8">
+        <v>133</v>
+      </c>
+      <c r="M31" s="9">
+        <v>27</v>
+      </c>
+      <c r="N31" s="8">
+        <v>139.08000000000001</v>
+      </c>
+      <c r="O31" s="8">
+        <v>185.81</v>
+      </c>
+      <c r="P31" s="8">
+        <v>232.54</v>
+      </c>
+      <c r="Q31" s="8">
+        <v>279.27</v>
+      </c>
+      <c r="R31" s="8">
+        <v>325.99</v>
+      </c>
+      <c r="S31" s="8">
+        <v>562</v>
+      </c>
+      <c r="T31" s="8">
+        <v>798</v>
+      </c>
+      <c r="U31" s="8">
+        <v>1034</v>
+      </c>
+      <c r="V31" s="8">
+        <v>1270</v>
+      </c>
+      <c r="W31" s="8">
+        <v>1506</v>
+      </c>
+    </row>
+    <row r="32" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A32" s="5">
+        <v>28</v>
+      </c>
+      <c r="B32" s="8">
+        <v>63.63</v>
+      </c>
+      <c r="C32" s="8">
+        <v>78.48</v>
+      </c>
+      <c r="D32" s="8">
+        <v>93.33</v>
+      </c>
+      <c r="E32" s="8">
+        <v>90.47</v>
+      </c>
+      <c r="F32" s="8">
+        <v>87.6</v>
+      </c>
+      <c r="G32" s="8">
+        <v>84.74</v>
+      </c>
+      <c r="H32" s="8">
+        <v>99.05</v>
+      </c>
+      <c r="I32" s="8">
+        <v>113.37</v>
+      </c>
+      <c r="J32" s="8">
+        <v>127.69</v>
+      </c>
+      <c r="K32" s="8">
+        <v>133.38</v>
+      </c>
+      <c r="M32" s="9">
+        <v>28</v>
+      </c>
+      <c r="N32" s="8">
+        <v>139.08000000000001</v>
+      </c>
+      <c r="O32" s="8">
+        <v>185.81</v>
+      </c>
+      <c r="P32" s="8">
+        <v>232.54</v>
+      </c>
+      <c r="Q32" s="8">
+        <v>279.27</v>
+      </c>
+      <c r="R32" s="8">
+        <v>325.99</v>
+      </c>
+      <c r="S32" s="8">
+        <v>562</v>
+      </c>
+      <c r="T32" s="8">
+        <v>798</v>
+      </c>
+      <c r="U32" s="8">
+        <v>1034</v>
+      </c>
+      <c r="V32" s="8">
+        <v>1270</v>
+      </c>
+      <c r="W32" s="8">
+        <v>1506</v>
+      </c>
+    </row>
+    <row r="33" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A33" s="5">
+        <v>29</v>
+      </c>
+      <c r="B33" s="8">
+        <v>65.27</v>
+      </c>
+      <c r="C33" s="8">
+        <v>79.97</v>
+      </c>
+      <c r="D33" s="8">
+        <v>94.67</v>
+      </c>
+      <c r="E33" s="8">
+        <v>91.38</v>
+      </c>
+      <c r="F33" s="8">
+        <v>88.09</v>
+      </c>
+      <c r="G33" s="8">
+        <v>84.8</v>
+      </c>
+      <c r="H33" s="8">
+        <v>99.35</v>
+      </c>
+      <c r="I33" s="8">
+        <v>113.9</v>
+      </c>
+      <c r="J33" s="8">
+        <v>128.44999999999999</v>
+      </c>
+      <c r="K33" s="8">
+        <v>133.76</v>
+      </c>
+      <c r="M33" s="9">
+        <v>29</v>
+      </c>
+      <c r="N33" s="8">
+        <v>139.08000000000001</v>
+      </c>
+      <c r="O33" s="8">
+        <v>185.81</v>
+      </c>
+      <c r="P33" s="8">
+        <v>232.54</v>
+      </c>
+      <c r="Q33" s="8">
+        <v>279.27</v>
+      </c>
+      <c r="R33" s="8">
+        <v>325.99</v>
+      </c>
+      <c r="S33" s="8">
+        <v>562</v>
+      </c>
+      <c r="T33" s="8">
+        <v>798</v>
+      </c>
+      <c r="U33" s="8">
+        <v>1034</v>
+      </c>
+      <c r="V33" s="8">
+        <v>1270</v>
+      </c>
+      <c r="W33" s="8">
+        <v>1506</v>
+      </c>
+    </row>
+    <row r="34" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A34" s="5">
+        <v>30</v>
+      </c>
+      <c r="B34" s="8">
+        <v>66.91</v>
+      </c>
+      <c r="C34" s="8">
+        <v>81.459999999999994</v>
+      </c>
+      <c r="D34" s="8">
+        <v>96.01</v>
+      </c>
+      <c r="E34" s="8">
+        <v>92.29</v>
+      </c>
+      <c r="F34" s="8">
+        <v>88.58</v>
+      </c>
+      <c r="G34" s="8">
+        <v>84.86</v>
+      </c>
+      <c r="H34" s="8">
+        <v>99.65</v>
+      </c>
+      <c r="I34" s="8">
+        <v>114.43</v>
+      </c>
+      <c r="J34" s="8">
+        <v>129.21</v>
+      </c>
+      <c r="K34" s="8">
+        <v>134.15</v>
+      </c>
+      <c r="M34" s="9">
+        <v>30</v>
+      </c>
+      <c r="N34" s="8">
+        <v>139.08000000000001</v>
+      </c>
+      <c r="O34" s="8">
+        <v>185.81</v>
+      </c>
+      <c r="P34" s="8">
+        <v>232.54</v>
+      </c>
+      <c r="Q34" s="8">
+        <v>279.27</v>
+      </c>
+      <c r="R34" s="8">
+        <v>325.99</v>
+      </c>
+      <c r="S34" s="8">
+        <v>562</v>
+      </c>
+      <c r="T34" s="8">
+        <v>798</v>
+      </c>
+      <c r="U34" s="8">
+        <v>1034</v>
+      </c>
+      <c r="V34" s="8">
+        <v>1270</v>
+      </c>
+      <c r="W34" s="8">
+        <v>1506</v>
+      </c>
+    </row>
+    <row r="35" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A35" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B35" s="8">
+        <v>40.803333333333335</v>
+      </c>
+      <c r="C35" s="8">
+        <v>56.356666666666669</v>
+      </c>
+      <c r="D35" s="8">
+        <v>71.911000000000016</v>
+      </c>
+      <c r="E35" s="8">
+        <v>73.928000000000011</v>
+      </c>
+      <c r="F35" s="8">
+        <v>75.945666666666682</v>
+      </c>
+      <c r="G35" s="8">
+        <v>77.962999999999994</v>
+      </c>
+      <c r="H35" s="8">
+        <v>89.435999999999993</v>
+      </c>
+      <c r="I35" s="8">
+        <v>100.90933333333332</v>
+      </c>
+      <c r="J35" s="8">
+        <v>112.383</v>
+      </c>
+      <c r="K35" s="8">
+        <v>125.73133333333334</v>
+      </c>
+      <c r="M35" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="N35" s="10">
+        <v>139.07999999999996</v>
+      </c>
+      <c r="O35" s="10">
+        <v>185.81000000000006</v>
+      </c>
+      <c r="P35" s="10">
+        <v>232.54</v>
+      </c>
+      <c r="Q35" s="10">
+        <v>279.27000000000021</v>
+      </c>
+      <c r="R35" s="10">
+        <v>325.98999999999984</v>
+      </c>
+      <c r="S35" s="10">
+        <v>562</v>
+      </c>
+      <c r="T35" s="10">
+        <v>798</v>
+      </c>
+      <c r="U35" s="10">
+        <v>1034</v>
+      </c>
+      <c r="V35" s="10">
+        <v>1270</v>
+      </c>
+      <c r="W35" s="10">
+        <v>1506</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B2:K2"/>
+    <mergeCell ref="M1:W1"/>
+    <mergeCell ref="N2:W2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{918B0DAF-F95D-4AE3-B8B6-445C4F5FB350}">
   <dimension ref="A1:W35"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.140625" customWidth="1"/>
-    <col min="13" max="23" width="11.140625" customWidth="1"/>
+    <col min="1" max="1" width="11.1796875" customWidth="1"/>
+    <col min="13" max="23" width="11.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>36</v>
       </c>
@@ -783,7 +3113,7 @@
       <c r="V1" s="14"/>
       <c r="W1" s="15"/>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -815,7 +3145,7 @@
       <c r="V2" s="12"/>
       <c r="W2" s="12"/>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
         <v>2</v>
       </c>
@@ -883,7 +3213,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
         <v>3</v>
       </c>
@@ -951,7 +3281,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A5" s="5">
         <v>1</v>
       </c>
@@ -1019,7 +3349,7 @@
         <v>1401.94</v>
       </c>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A6" s="5">
         <v>2</v>
       </c>
@@ -1087,7 +3417,7 @@
         <v>1401.94</v>
       </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A7" s="5">
         <v>3</v>
       </c>
@@ -1155,7 +3485,7 @@
         <v>1401.94</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A8" s="5">
         <v>4</v>
       </c>
@@ -1223,7 +3553,7 @@
         <v>1401.94</v>
       </c>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A9" s="5">
         <v>5</v>
       </c>
@@ -1291,7 +3621,7 @@
         <v>1401.94</v>
       </c>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A10" s="5">
         <v>6</v>
       </c>
@@ -1359,7 +3689,7 @@
         <v>1401.94</v>
       </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A11" s="5">
         <v>7</v>
       </c>
@@ -1427,7 +3757,7 @@
         <v>1401.94</v>
       </c>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A12" s="5">
         <v>8</v>
       </c>
@@ -1495,7 +3825,7 @@
         <v>1401.94</v>
       </c>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A13" s="5">
         <v>9</v>
       </c>
@@ -1563,7 +3893,7 @@
         <v>1401.94</v>
       </c>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A14" s="5">
         <v>10</v>
       </c>
@@ -1631,7 +3961,7 @@
         <v>1401.94</v>
       </c>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A15" s="5">
         <v>11</v>
       </c>
@@ -1699,7 +4029,7 @@
         <v>1401.94</v>
       </c>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A16" s="5">
         <v>12</v>
       </c>
@@ -1767,7 +4097,7 @@
         <v>1401.94</v>
       </c>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A17" s="5">
         <v>13</v>
       </c>
@@ -1835,7 +4165,7 @@
         <v>1401.94</v>
       </c>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A18" s="5">
         <v>14</v>
       </c>
@@ -1903,7 +4233,7 @@
         <v>1401.94</v>
       </c>
     </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A19" s="5">
         <v>15</v>
       </c>
@@ -1971,7 +4301,7 @@
         <v>1401.94</v>
       </c>
     </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A20" s="5">
         <v>16</v>
       </c>
@@ -2039,7 +4369,7 @@
         <v>1401.94</v>
       </c>
     </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A21" s="5">
         <v>17</v>
       </c>
@@ -2107,7 +4437,7 @@
         <v>1401.94</v>
       </c>
     </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A22" s="5">
         <v>18</v>
       </c>
@@ -2175,7 +4505,7 @@
         <v>1401.94</v>
       </c>
     </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A23" s="5">
         <v>19</v>
       </c>
@@ -2243,7 +4573,7 @@
         <v>1401.94</v>
       </c>
     </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A24" s="5">
         <v>20</v>
       </c>
@@ -2311,7 +4641,7 @@
         <v>1401.94</v>
       </c>
     </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A25" s="5">
         <v>21</v>
       </c>
@@ -2379,7 +4709,7 @@
         <v>1401.94</v>
       </c>
     </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A26" s="5">
         <v>22</v>
       </c>
@@ -2447,7 +4777,7 @@
         <v>1401.94</v>
       </c>
     </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A27" s="5">
         <v>23</v>
       </c>
@@ -2515,7 +4845,7 @@
         <v>1401.94</v>
       </c>
     </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A28" s="5">
         <v>24</v>
       </c>
@@ -2583,7 +4913,7 @@
         <v>1401.94</v>
       </c>
     </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A29" s="5">
         <v>25</v>
       </c>
@@ -2651,7 +4981,7 @@
         <v>1401.94</v>
       </c>
     </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A30" s="5">
         <v>26</v>
       </c>
@@ -2719,7 +5049,7 @@
         <v>1401.94</v>
       </c>
     </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A31" s="5">
         <v>27</v>
       </c>
@@ -2787,7 +5117,7 @@
         <v>1401.94</v>
       </c>
     </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A32" s="5">
         <v>28</v>
       </c>
@@ -2855,7 +5185,7 @@
         <v>1401.94</v>
       </c>
     </row>
-    <row r="33" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A33" s="5">
         <v>29</v>
       </c>
@@ -2923,7 +5253,7 @@
         <v>1401.94</v>
       </c>
     </row>
-    <row r="34" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A34" s="5">
         <v>30</v>
       </c>
@@ -2991,7 +5321,7 @@
         <v>1401.94</v>
       </c>
     </row>
-    <row r="35" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A35" s="5" t="s">
         <v>14</v>
       </c>
@@ -3069,16 +5399,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89E0380B-3232-4FC8-8E48-B6A283DD6300}">
   <dimension ref="A1:W35"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.140625" customWidth="1"/>
-    <col min="13" max="23" width="11.140625" customWidth="1"/>
+    <col min="1" max="1" width="11.1796875" customWidth="1"/>
+    <col min="13" max="23" width="11.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>34</v>
       </c>
@@ -3106,7 +5436,7 @@
       <c r="V1" s="14"/>
       <c r="W1" s="15"/>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -3138,7 +5468,7 @@
       <c r="V2" s="12"/>
       <c r="W2" s="12"/>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
         <v>2</v>
       </c>
@@ -3206,7 +5536,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
         <v>3</v>
       </c>
@@ -3274,7 +5604,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A5" s="5">
         <v>1</v>
       </c>
@@ -3342,7 +5672,7 @@
         <v>1348.06</v>
       </c>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A6" s="5">
         <v>2</v>
       </c>
@@ -3410,7 +5740,7 @@
         <v>1348.06</v>
       </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A7" s="5">
         <v>3</v>
       </c>
@@ -3478,7 +5808,7 @@
         <v>1348.06</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A8" s="5">
         <v>4</v>
       </c>
@@ -3546,7 +5876,7 @@
         <v>1348.06</v>
       </c>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A9" s="5">
         <v>5</v>
       </c>
@@ -3614,7 +5944,7 @@
         <v>1348.06</v>
       </c>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A10" s="5">
         <v>6</v>
       </c>
@@ -3682,7 +6012,7 @@
         <v>1348.06</v>
       </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A11" s="5">
         <v>7</v>
       </c>
@@ -3750,7 +6080,7 @@
         <v>1348.06</v>
       </c>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A12" s="5">
         <v>8</v>
       </c>
@@ -3818,7 +6148,7 @@
         <v>1348.06</v>
       </c>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A13" s="5">
         <v>9</v>
       </c>
@@ -3886,7 +6216,7 @@
         <v>1348.06</v>
       </c>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A14" s="5">
         <v>10</v>
       </c>
@@ -3954,7 +6284,7 @@
         <v>1348.06</v>
       </c>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A15" s="5">
         <v>11</v>
       </c>
@@ -4022,7 +6352,7 @@
         <v>1348.06</v>
       </c>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A16" s="5">
         <v>12</v>
       </c>
@@ -4090,7 +6420,7 @@
         <v>1348.06</v>
       </c>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A17" s="5">
         <v>13</v>
       </c>
@@ -4158,7 +6488,7 @@
         <v>1348.06</v>
       </c>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A18" s="5">
         <v>14</v>
       </c>
@@ -4226,7 +6556,7 @@
         <v>1348.06</v>
       </c>
     </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A19" s="5">
         <v>15</v>
       </c>
@@ -4294,7 +6624,7 @@
         <v>1348.06</v>
       </c>
     </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A20" s="5">
         <v>16</v>
       </c>
@@ -4362,7 +6692,7 @@
         <v>1348.06</v>
       </c>
     </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A21" s="5">
         <v>17</v>
       </c>
@@ -4430,7 +6760,7 @@
         <v>1348.06</v>
       </c>
     </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A22" s="5">
         <v>18</v>
       </c>
@@ -4498,7 +6828,7 @@
         <v>1348.06</v>
       </c>
     </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A23" s="5">
         <v>19</v>
       </c>
@@ -4566,7 +6896,7 @@
         <v>1348.06</v>
       </c>
     </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A24" s="5">
         <v>20</v>
       </c>
@@ -4634,7 +6964,7 @@
         <v>1348.06</v>
       </c>
     </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A25" s="5">
         <v>21</v>
       </c>
@@ -4702,7 +7032,7 @@
         <v>1348.06</v>
       </c>
     </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A26" s="5">
         <v>22</v>
       </c>
@@ -4770,7 +7100,7 @@
         <v>1348.06</v>
       </c>
     </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A27" s="5">
         <v>23</v>
       </c>
@@ -4838,7 +7168,7 @@
         <v>1348.06</v>
       </c>
     </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A28" s="5">
         <v>24</v>
       </c>
@@ -4906,7 +7236,7 @@
         <v>1348.06</v>
       </c>
     </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A29" s="5">
         <v>25</v>
       </c>
@@ -4974,7 +7304,7 @@
         <v>1348.06</v>
       </c>
     </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A30" s="5">
         <v>26</v>
       </c>
@@ -5042,7 +7372,7 @@
         <v>1348.06</v>
       </c>
     </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A31" s="5">
         <v>27</v>
       </c>
@@ -5110,7 +7440,7 @@
         <v>1348.06</v>
       </c>
     </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A32" s="5">
         <v>28</v>
       </c>
@@ -5178,7 +7508,7 @@
         <v>1348.06</v>
       </c>
     </row>
-    <row r="33" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A33" s="5">
         <v>29</v>
       </c>
@@ -5246,7 +7576,7 @@
         <v>1348.06</v>
       </c>
     </row>
-    <row r="34" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A34" s="5">
         <v>30</v>
       </c>
@@ -5314,7 +7644,7 @@
         <v>1348.06</v>
       </c>
     </row>
-    <row r="35" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A35" s="5" t="s">
         <v>14</v>
       </c>
@@ -5392,16 +7722,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3EEC94F4-4E93-438D-92F8-5C9CBA48C22A}">
   <dimension ref="A1:W35"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.140625" customWidth="1"/>
-    <col min="13" max="23" width="11.140625" customWidth="1"/>
+    <col min="1" max="1" width="11.1796875" customWidth="1"/>
+    <col min="13" max="23" width="11.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>32</v>
       </c>
@@ -5429,7 +7759,7 @@
       <c r="V1" s="14"/>
       <c r="W1" s="15"/>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -5461,7 +7791,7 @@
       <c r="V2" s="12"/>
       <c r="W2" s="12"/>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
         <v>2</v>
       </c>
@@ -5529,7 +7859,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
         <v>3</v>
       </c>
@@ -5597,7 +7927,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A5" s="5">
         <v>1</v>
       </c>
@@ -5665,7 +7995,7 @@
         <v>1290.8800000000001</v>
       </c>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A6" s="5">
         <v>2</v>
       </c>
@@ -5733,7 +8063,7 @@
         <v>1290.8800000000001</v>
       </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A7" s="5">
         <v>3</v>
       </c>
@@ -5801,7 +8131,7 @@
         <v>1290.8800000000001</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A8" s="5">
         <v>4</v>
       </c>
@@ -5869,7 +8199,7 @@
         <v>1290.8800000000001</v>
       </c>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A9" s="5">
         <v>5</v>
       </c>
@@ -5937,7 +8267,7 @@
         <v>1290.8800000000001</v>
       </c>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A10" s="5">
         <v>6</v>
       </c>
@@ -6005,7 +8335,7 @@
         <v>1290.8800000000001</v>
       </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A11" s="5">
         <v>7</v>
       </c>
@@ -6073,7 +8403,7 @@
         <v>1290.8800000000001</v>
       </c>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A12" s="5">
         <v>8</v>
       </c>
@@ -6141,7 +8471,7 @@
         <v>1290.8800000000001</v>
       </c>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A13" s="5">
         <v>9</v>
       </c>
@@ -6209,7 +8539,7 @@
         <v>1290.8800000000001</v>
       </c>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A14" s="5">
         <v>10</v>
       </c>
@@ -6277,7 +8607,7 @@
         <v>1290.8800000000001</v>
       </c>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A15" s="5">
         <v>11</v>
       </c>
@@ -6345,7 +8675,7 @@
         <v>1290.8800000000001</v>
       </c>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A16" s="5">
         <v>12</v>
       </c>
@@ -6413,7 +8743,7 @@
         <v>1290.8800000000001</v>
       </c>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A17" s="5">
         <v>13</v>
       </c>
@@ -6481,7 +8811,7 @@
         <v>1290.8800000000001</v>
       </c>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A18" s="5">
         <v>14</v>
       </c>
@@ -6549,7 +8879,7 @@
         <v>1290.8800000000001</v>
       </c>
     </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A19" s="5">
         <v>15</v>
       </c>
@@ -6617,7 +8947,7 @@
         <v>1290.8800000000001</v>
       </c>
     </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A20" s="5">
         <v>16</v>
       </c>
@@ -6685,7 +9015,7 @@
         <v>1290.8800000000001</v>
       </c>
     </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A21" s="5">
         <v>17</v>
       </c>
@@ -6753,7 +9083,7 @@
         <v>1290.8800000000001</v>
       </c>
     </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A22" s="5">
         <v>18</v>
       </c>
@@ -6821,7 +9151,7 @@
         <v>1290.8800000000001</v>
       </c>
     </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A23" s="5">
         <v>19</v>
       </c>
@@ -6889,7 +9219,7 @@
         <v>1290.8800000000001</v>
       </c>
     </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A24" s="5">
         <v>20</v>
       </c>
@@ -6957,7 +9287,7 @@
         <v>1290.8800000000001</v>
       </c>
     </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A25" s="5">
         <v>21</v>
       </c>
@@ -7025,7 +9355,7 @@
         <v>1290.8800000000001</v>
       </c>
     </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A26" s="5">
         <v>22</v>
       </c>
@@ -7093,7 +9423,7 @@
         <v>1290.8800000000001</v>
       </c>
     </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A27" s="5">
         <v>23</v>
       </c>
@@ -7161,7 +9491,7 @@
         <v>1290.8800000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A28" s="5">
         <v>24</v>
       </c>
@@ -7229,7 +9559,7 @@
         <v>1290.8800000000001</v>
       </c>
     </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A29" s="5">
         <v>25</v>
       </c>
@@ -7297,7 +9627,7 @@
         <v>1290.8800000000001</v>
       </c>
     </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A30" s="5">
         <v>26</v>
       </c>
@@ -7365,7 +9695,7 @@
         <v>1290.8800000000001</v>
       </c>
     </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A31" s="5">
         <v>27</v>
       </c>
@@ -7433,7 +9763,7 @@
         <v>1290.8800000000001</v>
       </c>
     </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A32" s="5">
         <v>28</v>
       </c>
@@ -7501,7 +9831,7 @@
         <v>1290.8800000000001</v>
       </c>
     </row>
-    <row r="33" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A33" s="5">
         <v>29</v>
       </c>
@@ -7569,7 +9899,7 @@
         <v>1290.8800000000001</v>
       </c>
     </row>
-    <row r="34" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A34" s="5">
         <v>30</v>
       </c>
@@ -7637,7 +9967,7 @@
         <v>1290.8800000000001</v>
       </c>
     </row>
-    <row r="35" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A35" s="5" t="s">
         <v>14</v>
       </c>
@@ -7715,16 +10045,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{612EBB24-0E24-4D37-B6A7-8B4DA2BD1A51}">
   <dimension ref="A1:W35"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.140625" customWidth="1"/>
-    <col min="13" max="23" width="11.140625" customWidth="1"/>
+    <col min="1" max="1" width="11.1796875" customWidth="1"/>
+    <col min="13" max="23" width="11.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>30</v>
       </c>
@@ -7752,7 +10082,7 @@
       <c r="V1" s="14"/>
       <c r="W1" s="15"/>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -7784,7 +10114,7 @@
       <c r="V2" s="12"/>
       <c r="W2" s="12"/>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
         <v>2</v>
       </c>
@@ -7852,7 +10182,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
         <v>3</v>
       </c>
@@ -7920,7 +10250,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A5" s="5">
         <v>1</v>
       </c>
@@ -7988,7 +10318,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A6" s="5">
         <v>2</v>
       </c>
@@ -8056,7 +10386,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A7" s="5">
         <v>3</v>
       </c>
@@ -8124,7 +10454,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A8" s="5">
         <v>4</v>
       </c>
@@ -8192,7 +10522,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A9" s="5">
         <v>5</v>
       </c>
@@ -8260,7 +10590,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A10" s="5">
         <v>6</v>
       </c>
@@ -8328,7 +10658,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A11" s="5">
         <v>7</v>
       </c>
@@ -8396,7 +10726,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A12" s="5">
         <v>8</v>
       </c>
@@ -8464,7 +10794,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A13" s="5">
         <v>9</v>
       </c>
@@ -8532,7 +10862,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A14" s="5">
         <v>10</v>
       </c>
@@ -8600,7 +10930,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A15" s="5">
         <v>11</v>
       </c>
@@ -8668,7 +10998,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A16" s="5">
         <v>12</v>
       </c>
@@ -8736,7 +11066,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A17" s="5">
         <v>13</v>
       </c>
@@ -8804,7 +11134,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A18" s="5">
         <v>14</v>
       </c>
@@ -8872,7 +11202,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A19" s="5">
         <v>15</v>
       </c>
@@ -8940,7 +11270,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A20" s="5">
         <v>16</v>
       </c>
@@ -9008,7 +11338,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A21" s="5">
         <v>17</v>
       </c>
@@ -9076,7 +11406,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A22" s="5">
         <v>18</v>
       </c>
@@ -9144,7 +11474,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A23" s="5">
         <v>19</v>
       </c>
@@ -9212,7 +11542,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A24" s="5">
         <v>20</v>
       </c>
@@ -9280,7 +11610,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A25" s="5">
         <v>21</v>
       </c>
@@ -9348,7 +11678,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A26" s="5">
         <v>22</v>
       </c>
@@ -9416,7 +11746,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A27" s="5">
         <v>23</v>
       </c>
@@ -9484,7 +11814,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A28" s="5">
         <v>24</v>
       </c>
@@ -9552,7 +11882,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A29" s="5">
         <v>25</v>
       </c>
@@ -9620,7 +11950,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A30" s="5">
         <v>26</v>
       </c>
@@ -9688,7 +12018,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A31" s="5">
         <v>27</v>
       </c>
@@ -9756,7 +12086,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A32" s="5">
         <v>28</v>
       </c>
@@ -9824,7 +12154,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="33" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A33" s="5">
         <v>29</v>
       </c>
@@ -9892,7 +12222,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="34" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A34" s="5">
         <v>30</v>
       </c>
@@ -9960,7 +12290,7 @@
         <v>1400.65</v>
       </c>
     </row>
-    <row r="35" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A35" s="5" t="s">
         <v>14</v>
       </c>
@@ -10038,16 +12368,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A2E7E46-B70B-4DB0-97AE-2138287FA00A}">
   <dimension ref="A1:W35"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.140625" customWidth="1"/>
-    <col min="13" max="23" width="11.140625" customWidth="1"/>
+    <col min="1" max="1" width="11.1796875" customWidth="1"/>
+    <col min="13" max="23" width="11.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>28</v>
       </c>
@@ -10075,7 +12405,7 @@
       <c r="V1" s="14"/>
       <c r="W1" s="15"/>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -10107,7 +12437,7 @@
       <c r="V2" s="12"/>
       <c r="W2" s="12"/>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
         <v>2</v>
       </c>
@@ -10175,7 +12505,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
         <v>3</v>
       </c>
@@ -10243,7 +12573,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A5" s="5">
         <v>1</v>
       </c>
@@ -10311,7 +12641,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A6" s="5">
         <v>2</v>
       </c>
@@ -10379,7 +12709,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A7" s="5">
         <v>3</v>
       </c>
@@ -10447,7 +12777,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A8" s="5">
         <v>4</v>
       </c>
@@ -10515,7 +12845,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A9" s="5">
         <v>5</v>
       </c>
@@ -10583,7 +12913,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A10" s="5">
         <v>6</v>
       </c>
@@ -10651,7 +12981,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A11" s="5">
         <v>7</v>
       </c>
@@ -10719,7 +13049,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A12" s="5">
         <v>8</v>
       </c>
@@ -10787,7 +13117,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A13" s="5">
         <v>9</v>
       </c>
@@ -10855,7 +13185,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A14" s="5">
         <v>10</v>
       </c>
@@ -10923,7 +13253,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A15" s="5">
         <v>11</v>
       </c>
@@ -10991,7 +13321,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A16" s="5">
         <v>12</v>
       </c>
@@ -11059,7 +13389,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A17" s="5">
         <v>13</v>
       </c>
@@ -11127,7 +13457,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A18" s="5">
         <v>14</v>
       </c>
@@ -11195,7 +13525,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A19" s="5">
         <v>15</v>
       </c>
@@ -11263,7 +13593,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A20" s="5">
         <v>16</v>
       </c>
@@ -11331,7 +13661,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A21" s="5">
         <v>17</v>
       </c>
@@ -11399,7 +13729,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A22" s="5">
         <v>18</v>
       </c>
@@ -11467,7 +13797,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A23" s="5">
         <v>19</v>
       </c>
@@ -11535,7 +13865,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A24" s="5">
         <v>20</v>
       </c>
@@ -11603,7 +13933,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A25" s="5">
         <v>21</v>
       </c>
@@ -11671,7 +14001,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A26" s="5">
         <v>22</v>
       </c>
@@ -11739,7 +14069,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A27" s="5">
         <v>23</v>
       </c>
@@ -11807,7 +14137,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A28" s="5">
         <v>24</v>
       </c>
@@ -11875,7 +14205,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A29" s="5">
         <v>25</v>
       </c>
@@ -11943,7 +14273,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A30" s="5">
         <v>26</v>
       </c>
@@ -12011,7 +14341,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A31" s="5">
         <v>27</v>
       </c>
@@ -12079,7 +14409,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A32" s="5">
         <v>28</v>
       </c>
@@ -12147,7 +14477,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="33" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A33" s="5">
         <v>29</v>
       </c>
@@ -12215,7 +14545,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="34" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A34" s="5">
         <v>30</v>
       </c>
@@ -12283,7 +14613,7 @@
         <v>1337.64</v>
       </c>
     </row>
-    <row r="35" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A35" s="5" t="s">
         <v>14</v>
       </c>
@@ -12361,16 +14691,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D32525DC-1FAE-40FA-B3A1-6E6C0B62B72E}">
   <dimension ref="A1:W35"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.140625" customWidth="1"/>
-    <col min="13" max="23" width="11.140625" customWidth="1"/>
+    <col min="1" max="1" width="11.1796875" customWidth="1"/>
+    <col min="13" max="23" width="11.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>26</v>
       </c>
@@ -12398,7 +14728,7 @@
       <c r="V1" s="14"/>
       <c r="W1" s="15"/>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -12430,7 +14760,7 @@
       <c r="V2" s="12"/>
       <c r="W2" s="12"/>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
         <v>2</v>
       </c>
@@ -12498,7 +14828,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
         <v>3</v>
       </c>
@@ -12566,7 +14896,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A5" s="5">
         <v>1</v>
       </c>
@@ -12634,7 +14964,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A6" s="5">
         <v>2</v>
       </c>
@@ -12702,7 +15032,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A7" s="5">
         <v>3</v>
       </c>
@@ -12770,7 +15100,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A8" s="5">
         <v>4</v>
       </c>
@@ -12838,7 +15168,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A9" s="5">
         <v>5</v>
       </c>
@@ -12906,7 +15236,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A10" s="5">
         <v>6</v>
       </c>
@@ -12974,7 +15304,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A11" s="5">
         <v>7</v>
       </c>
@@ -13042,7 +15372,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A12" s="5">
         <v>8</v>
       </c>
@@ -13110,7 +15440,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A13" s="5">
         <v>9</v>
       </c>
@@ -13178,7 +15508,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A14" s="5">
         <v>10</v>
       </c>
@@ -13246,7 +15576,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A15" s="5">
         <v>11</v>
       </c>
@@ -13314,7 +15644,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A16" s="5">
         <v>12</v>
       </c>
@@ -13382,7 +15712,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A17" s="5">
         <v>13</v>
       </c>
@@ -13450,7 +15780,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A18" s="5">
         <v>14</v>
       </c>
@@ -13518,7 +15848,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A19" s="5">
         <v>15</v>
       </c>
@@ -13586,7 +15916,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A20" s="5">
         <v>16</v>
       </c>
@@ -13654,7 +15984,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A21" s="5">
         <v>17</v>
       </c>
@@ -13722,7 +16052,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A22" s="5">
         <v>18</v>
       </c>
@@ -13790,7 +16120,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A23" s="5">
         <v>19</v>
       </c>
@@ -13858,7 +16188,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A24" s="5">
         <v>20</v>
       </c>
@@ -13926,7 +16256,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A25" s="5">
         <v>21</v>
       </c>
@@ -13994,7 +16324,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A26" s="5">
         <v>22</v>
       </c>
@@ -14062,7 +16392,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A27" s="5">
         <v>23</v>
       </c>
@@ -14130,7 +16460,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A28" s="5">
         <v>24</v>
       </c>
@@ -14198,7 +16528,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A29" s="5">
         <v>25</v>
       </c>
@@ -14266,7 +16596,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A30" s="5">
         <v>26</v>
       </c>
@@ -14334,7 +16664,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A31" s="5">
         <v>27</v>
       </c>
@@ -14402,7 +16732,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A32" s="5">
         <v>28</v>
       </c>
@@ -14470,7 +16800,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="33" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A33" s="5">
         <v>29</v>
       </c>
@@ -14538,7 +16868,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="34" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A34" s="5">
         <v>30</v>
       </c>
@@ -14606,7 +16936,7 @@
         <v>1207.19</v>
       </c>
     </row>
-    <row r="35" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A35" s="5" t="s">
         <v>14</v>
       </c>
@@ -14684,15 +17014,15 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <sheetPr codeName="Sheet9">
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
   <dimension ref="H31"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="31" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="8:8" x14ac:dyDescent="0.35">
       <c r="H31" s="1"/>
     </row>
   </sheetData>

</xml_diff>